<commit_message>
Move simulado S4-12 para 23-24/09
Pedido do usuário: simulado S4 das turmas 12C1/12C2, de 16-17/09
(semana7) para 23-24/09 (semana8) -- mesmos dias da semana (quarta e
quinta), só trocou de semana. Semana8 estava livre para as duas turmas.

- gerar_calendario.py: SIMULADOS["12C1"]/["12C2"] atualizados -- item 8
  do checklist de verificar_calendario.py compara a planilha contra essa
  constante, então precisa acompanhar a edição manual.
- Proposta 3: células do S4-12 movidas.
- Relatórios de tempos cedidos e tabela por turma regenerados (trocas
  de tempo não muda: simulados não entram nesse relatório).

verificar_calendario.py fecha em 0 PROBLEMA, mesma contagem de AVISOs.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -1842,7 +1842,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="465">
+  <cellXfs count="466">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -3424,6 +3424,9 @@
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="115" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="108" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -6161,18 +6164,8 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="G21" s="450" t="inlineStr">
-        <is>
-          <t>S4-12
-2º ao 7º tempos</t>
-        </is>
-      </c>
-      <c r="H21" s="450" t="inlineStr">
-        <is>
-          <t>S4-12
-2º ao 7º tempos</t>
-        </is>
-      </c>
+      <c r="G21" s="435" t="n"/>
+      <c r="H21" s="435" t="n"/>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -6198,8 +6191,8 @@
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
-      <c r="G22" s="437" t="n"/>
-      <c r="H22" s="437" t="n"/>
+      <c r="G22" s="438" t="n"/>
+      <c r="H22" s="438" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -6213,8 +6206,8 @@
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
-      <c r="G23" s="439" t="n"/>
-      <c r="H23" s="439" t="n"/>
+      <c r="G23" s="438" t="n"/>
+      <c r="H23" s="438" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -6242,8 +6235,18 @@
       </c>
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
-      <c r="G24" s="438" t="n"/>
-      <c r="H24" s="283" t="n"/>
+      <c r="G24" s="465" t="inlineStr">
+        <is>
+          <t>S4-12
+2º ao 7º tempos</t>
+        </is>
+      </c>
+      <c r="H24" s="418" t="inlineStr">
+        <is>
+          <t>S4-12
+2º ao 7º tempos</t>
+        </is>
+      </c>
       <c r="I24" s="78" t="n"/>
       <c r="J24" s="265" t="n"/>
       <c r="L24" s="318" t="inlineStr">
@@ -6261,8 +6264,8 @@
       <c r="D25" s="350" t="n"/>
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
-      <c r="G25" s="438" t="n"/>
-      <c r="H25" s="283" t="n"/>
+      <c r="G25" s="415" t="n"/>
+      <c r="H25" s="406" t="n"/>
       <c r="I25" s="78" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
@@ -6280,8 +6283,8 @@
       <c r="D26" s="350" t="n"/>
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
-      <c r="G26" s="438" t="n"/>
-      <c r="H26" s="283" t="n"/>
+      <c r="G26" s="416" t="n"/>
+      <c r="H26" s="407" t="n"/>
       <c r="I26" s="78" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
@@ -7112,7 +7115,6 @@
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -7177,6 +7179,7 @@
     <mergeCell ref="D51:D53"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="D60:D62"/>
+    <mergeCell ref="H24:H26"/>
     <mergeCell ref="F60:F62"/>
     <mergeCell ref="M31:N31"/>
     <mergeCell ref="A36:A38"/>
@@ -7185,7 +7188,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G21:G23"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
     <mergeCell ref="B42:B44"/>
@@ -7206,6 +7208,7 @@
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="A27:A29"/>
+    <mergeCell ref="G24:G26"/>
     <mergeCell ref="I18:I20"/>
     <mergeCell ref="D15:D17"/>
     <mergeCell ref="C57:C59"/>
@@ -9994,7 +9997,7 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="417" t="inlineStr">
+      <c r="F45" s="449" t="inlineStr">
         <is>
           <t>Bio - Ale
 1º tempo</t>
@@ -10017,7 +10020,7 @@
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="283" t="n"/>
-      <c r="F46" s="406" t="n"/>
+      <c r="F46" s="437" t="n"/>
       <c r="G46" s="283" t="n"/>
       <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
@@ -10030,7 +10033,7 @@
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="283" t="n"/>
-      <c r="F47" s="407" t="n"/>
+      <c r="F47" s="439" t="n"/>
       <c r="G47" s="283" t="n"/>
       <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
@@ -10055,7 +10058,7 @@
         <f>B48+4</f>
         <v/>
       </c>
-      <c r="E48" s="412" t="inlineStr">
+      <c r="E48" s="444" t="inlineStr">
         <is>
           <t>Redação - Raf
 6º e 7º tempos</t>
@@ -10076,7 +10079,7 @@
       <c r="B49" s="313" t="n"/>
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
-      <c r="E49" s="406" t="n"/>
+      <c r="E49" s="437" t="n"/>
       <c r="F49" s="351" t="n"/>
       <c r="G49" s="283" t="n"/>
       <c r="H49" s="438" t="n"/>
@@ -10088,7 +10091,7 @@
       <c r="B50" s="313" t="n"/>
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
-      <c r="E50" s="407" t="n"/>
+      <c r="E50" s="439" t="n"/>
       <c r="F50" s="387" t="n"/>
       <c r="G50" s="283" t="n"/>
       <c r="H50" s="438" t="n"/>
@@ -11680,7 +11683,7 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="417" t="inlineStr">
+      <c r="F45" s="449" t="inlineStr">
         <is>
           <t>Bio - Ale
 1º tempo</t>
@@ -11703,7 +11706,7 @@
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="283" t="n"/>
-      <c r="F46" s="406" t="n"/>
+      <c r="F46" s="437" t="n"/>
       <c r="G46" s="283" t="n"/>
       <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
@@ -11716,7 +11719,7 @@
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="283" t="n"/>
-      <c r="F47" s="407" t="n"/>
+      <c r="F47" s="439" t="n"/>
       <c r="G47" s="283" t="n"/>
       <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
@@ -11741,7 +11744,7 @@
         <f>B48+4</f>
         <v/>
       </c>
-      <c r="E48" s="412" t="inlineStr">
+      <c r="E48" s="444" t="inlineStr">
         <is>
           <t>Redação - Raf
 6º e 7º tempos</t>
@@ -11762,7 +11765,7 @@
       <c r="B49" s="313" t="n"/>
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
-      <c r="E49" s="406" t="n"/>
+      <c r="E49" s="437" t="n"/>
       <c r="F49" s="351" t="n"/>
       <c r="G49" s="283" t="n"/>
       <c r="H49" s="438" t="n"/>
@@ -11774,7 +11777,7 @@
       <c r="B50" s="313" t="n"/>
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
-      <c r="E50" s="407" t="n"/>
+      <c r="E50" s="439" t="n"/>
       <c r="F50" s="387" t="n"/>
       <c r="G50" s="283" t="n"/>
       <c r="H50" s="438" t="n"/>
@@ -19639,18 +19642,8 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="G21" s="450" t="inlineStr">
-        <is>
-          <t>S4-12
-2º ao 7º tempos</t>
-        </is>
-      </c>
-      <c r="H21" s="450" t="inlineStr">
-        <is>
-          <t>S4-12
-2º ao 7º tempos</t>
-        </is>
-      </c>
+      <c r="G21" s="435" t="n"/>
+      <c r="H21" s="435" t="n"/>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -19676,8 +19669,8 @@
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
-      <c r="G22" s="437" t="n"/>
-      <c r="H22" s="437" t="n"/>
+      <c r="G22" s="438" t="n"/>
+      <c r="H22" s="438" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -19691,8 +19684,8 @@
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
-      <c r="G23" s="439" t="n"/>
-      <c r="H23" s="439" t="n"/>
+      <c r="G23" s="438" t="n"/>
+      <c r="H23" s="438" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -19720,8 +19713,18 @@
       </c>
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
-      <c r="G24" s="438" t="n"/>
-      <c r="H24" s="283" t="n"/>
+      <c r="G24" s="465" t="inlineStr">
+        <is>
+          <t>S4-12
+2º ao 7º tempos</t>
+        </is>
+      </c>
+      <c r="H24" s="418" t="inlineStr">
+        <is>
+          <t>S4-12
+2º ao 7º tempos</t>
+        </is>
+      </c>
       <c r="I24" s="78" t="n"/>
       <c r="J24" s="265" t="n"/>
       <c r="L24" s="318" t="inlineStr">
@@ -19739,8 +19742,8 @@
       <c r="D25" s="350" t="n"/>
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
-      <c r="G25" s="438" t="n"/>
-      <c r="H25" s="283" t="n"/>
+      <c r="G25" s="415" t="n"/>
+      <c r="H25" s="406" t="n"/>
       <c r="I25" s="78" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
@@ -19758,8 +19761,8 @@
       <c r="D26" s="350" t="n"/>
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
-      <c r="G26" s="438" t="n"/>
-      <c r="H26" s="283" t="n"/>
+      <c r="G26" s="416" t="n"/>
+      <c r="H26" s="407" t="n"/>
       <c r="I26" s="78" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
@@ -20590,7 +20593,6 @@
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -20655,6 +20657,7 @@
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="H15:H17"/>
     <mergeCell ref="D60:D62"/>
+    <mergeCell ref="H24:H26"/>
     <mergeCell ref="F60:F62"/>
     <mergeCell ref="M31:N31"/>
     <mergeCell ref="A36:A38"/>
@@ -20663,7 +20666,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G21:G23"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
     <mergeCell ref="B42:B44"/>
@@ -20684,6 +20686,7 @@
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="A27:A29"/>
+    <mergeCell ref="G24:G26"/>
     <mergeCell ref="I18:I20"/>
     <mergeCell ref="D15:D17"/>
     <mergeCell ref="C57:C59"/>

</xml_diff>

<commit_message>
Move simulado S4-12 para 23-24/09 (#28)
Pedido do usuário: simulado S4 das turmas 12C1/12C2, de 16-17/09
(semana7) para 23-24/09 (semana8) -- mesmos dias da semana (quarta e
quinta), só trocou de semana. Semana8 estava livre para as duas turmas.

- gerar_calendario.py: SIMULADOS["12C1"]/["12C2"] atualizados -- item 8
  do checklist de verificar_calendario.py compara a planilha contra essa
  constante, então precisa acompanhar a edição manual.
- Proposta 3: células do S4-12 movidas.
- Relatórios de tempos cedidos e tabela por turma regenerados (trocas
  de tempo não muda: simulados não entram nesse relatório).

verificar_calendario.py fecha em 0 PROBLEMA, mesma contagem de AVISOs.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -1842,7 +1842,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="465">
+  <cellXfs count="466">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -3424,6 +3424,9 @@
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="115" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="108" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -6161,18 +6164,8 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="G21" s="450" t="inlineStr">
-        <is>
-          <t>S4-12
-2º ao 7º tempos</t>
-        </is>
-      </c>
-      <c r="H21" s="450" t="inlineStr">
-        <is>
-          <t>S4-12
-2º ao 7º tempos</t>
-        </is>
-      </c>
+      <c r="G21" s="435" t="n"/>
+      <c r="H21" s="435" t="n"/>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -6198,8 +6191,8 @@
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
-      <c r="G22" s="437" t="n"/>
-      <c r="H22" s="437" t="n"/>
+      <c r="G22" s="438" t="n"/>
+      <c r="H22" s="438" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -6213,8 +6206,8 @@
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
-      <c r="G23" s="439" t="n"/>
-      <c r="H23" s="439" t="n"/>
+      <c r="G23" s="438" t="n"/>
+      <c r="H23" s="438" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -6242,8 +6235,18 @@
       </c>
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
-      <c r="G24" s="438" t="n"/>
-      <c r="H24" s="283" t="n"/>
+      <c r="G24" s="465" t="inlineStr">
+        <is>
+          <t>S4-12
+2º ao 7º tempos</t>
+        </is>
+      </c>
+      <c r="H24" s="418" t="inlineStr">
+        <is>
+          <t>S4-12
+2º ao 7º tempos</t>
+        </is>
+      </c>
       <c r="I24" s="78" t="n"/>
       <c r="J24" s="265" t="n"/>
       <c r="L24" s="318" t="inlineStr">
@@ -6261,8 +6264,8 @@
       <c r="D25" s="350" t="n"/>
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
-      <c r="G25" s="438" t="n"/>
-      <c r="H25" s="283" t="n"/>
+      <c r="G25" s="415" t="n"/>
+      <c r="H25" s="406" t="n"/>
       <c r="I25" s="78" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
@@ -6280,8 +6283,8 @@
       <c r="D26" s="350" t="n"/>
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
-      <c r="G26" s="438" t="n"/>
-      <c r="H26" s="283" t="n"/>
+      <c r="G26" s="416" t="n"/>
+      <c r="H26" s="407" t="n"/>
       <c r="I26" s="78" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
@@ -7112,7 +7115,6 @@
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -7177,6 +7179,7 @@
     <mergeCell ref="D51:D53"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="D60:D62"/>
+    <mergeCell ref="H24:H26"/>
     <mergeCell ref="F60:F62"/>
     <mergeCell ref="M31:N31"/>
     <mergeCell ref="A36:A38"/>
@@ -7185,7 +7188,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G21:G23"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
     <mergeCell ref="B42:B44"/>
@@ -7206,6 +7208,7 @@
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="A27:A29"/>
+    <mergeCell ref="G24:G26"/>
     <mergeCell ref="I18:I20"/>
     <mergeCell ref="D15:D17"/>
     <mergeCell ref="C57:C59"/>
@@ -9994,7 +9997,7 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="417" t="inlineStr">
+      <c r="F45" s="449" t="inlineStr">
         <is>
           <t>Bio - Ale
 1º tempo</t>
@@ -10017,7 +10020,7 @@
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="283" t="n"/>
-      <c r="F46" s="406" t="n"/>
+      <c r="F46" s="437" t="n"/>
       <c r="G46" s="283" t="n"/>
       <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
@@ -10030,7 +10033,7 @@
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="283" t="n"/>
-      <c r="F47" s="407" t="n"/>
+      <c r="F47" s="439" t="n"/>
       <c r="G47" s="283" t="n"/>
       <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
@@ -10055,7 +10058,7 @@
         <f>B48+4</f>
         <v/>
       </c>
-      <c r="E48" s="412" t="inlineStr">
+      <c r="E48" s="444" t="inlineStr">
         <is>
           <t>Redação - Raf
 6º e 7º tempos</t>
@@ -10076,7 +10079,7 @@
       <c r="B49" s="313" t="n"/>
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
-      <c r="E49" s="406" t="n"/>
+      <c r="E49" s="437" t="n"/>
       <c r="F49" s="351" t="n"/>
       <c r="G49" s="283" t="n"/>
       <c r="H49" s="438" t="n"/>
@@ -10088,7 +10091,7 @@
       <c r="B50" s="313" t="n"/>
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
-      <c r="E50" s="407" t="n"/>
+      <c r="E50" s="439" t="n"/>
       <c r="F50" s="387" t="n"/>
       <c r="G50" s="283" t="n"/>
       <c r="H50" s="438" t="n"/>
@@ -11680,7 +11683,7 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="417" t="inlineStr">
+      <c r="F45" s="449" t="inlineStr">
         <is>
           <t>Bio - Ale
 1º tempo</t>
@@ -11703,7 +11706,7 @@
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="283" t="n"/>
-      <c r="F46" s="406" t="n"/>
+      <c r="F46" s="437" t="n"/>
       <c r="G46" s="283" t="n"/>
       <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
@@ -11716,7 +11719,7 @@
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="283" t="n"/>
-      <c r="F47" s="407" t="n"/>
+      <c r="F47" s="439" t="n"/>
       <c r="G47" s="283" t="n"/>
       <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
@@ -11741,7 +11744,7 @@
         <f>B48+4</f>
         <v/>
       </c>
-      <c r="E48" s="412" t="inlineStr">
+      <c r="E48" s="444" t="inlineStr">
         <is>
           <t>Redação - Raf
 6º e 7º tempos</t>
@@ -11762,7 +11765,7 @@
       <c r="B49" s="313" t="n"/>
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
-      <c r="E49" s="406" t="n"/>
+      <c r="E49" s="437" t="n"/>
       <c r="F49" s="351" t="n"/>
       <c r="G49" s="283" t="n"/>
       <c r="H49" s="438" t="n"/>
@@ -11774,7 +11777,7 @@
       <c r="B50" s="313" t="n"/>
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
-      <c r="E50" s="407" t="n"/>
+      <c r="E50" s="439" t="n"/>
       <c r="F50" s="387" t="n"/>
       <c r="G50" s="283" t="n"/>
       <c r="H50" s="438" t="n"/>
@@ -19639,18 +19642,8 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="G21" s="450" t="inlineStr">
-        <is>
-          <t>S4-12
-2º ao 7º tempos</t>
-        </is>
-      </c>
-      <c r="H21" s="450" t="inlineStr">
-        <is>
-          <t>S4-12
-2º ao 7º tempos</t>
-        </is>
-      </c>
+      <c r="G21" s="435" t="n"/>
+      <c r="H21" s="435" t="n"/>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -19676,8 +19669,8 @@
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
-      <c r="G22" s="437" t="n"/>
-      <c r="H22" s="437" t="n"/>
+      <c r="G22" s="438" t="n"/>
+      <c r="H22" s="438" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -19691,8 +19684,8 @@
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
-      <c r="G23" s="439" t="n"/>
-      <c r="H23" s="439" t="n"/>
+      <c r="G23" s="438" t="n"/>
+      <c r="H23" s="438" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -19720,8 +19713,18 @@
       </c>
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
-      <c r="G24" s="438" t="n"/>
-      <c r="H24" s="283" t="n"/>
+      <c r="G24" s="465" t="inlineStr">
+        <is>
+          <t>S4-12
+2º ao 7º tempos</t>
+        </is>
+      </c>
+      <c r="H24" s="418" t="inlineStr">
+        <is>
+          <t>S4-12
+2º ao 7º tempos</t>
+        </is>
+      </c>
       <c r="I24" s="78" t="n"/>
       <c r="J24" s="265" t="n"/>
       <c r="L24" s="318" t="inlineStr">
@@ -19739,8 +19742,8 @@
       <c r="D25" s="350" t="n"/>
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
-      <c r="G25" s="438" t="n"/>
-      <c r="H25" s="283" t="n"/>
+      <c r="G25" s="415" t="n"/>
+      <c r="H25" s="406" t="n"/>
       <c r="I25" s="78" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
@@ -19758,8 +19761,8 @@
       <c r="D26" s="350" t="n"/>
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
-      <c r="G26" s="438" t="n"/>
-      <c r="H26" s="283" t="n"/>
+      <c r="G26" s="416" t="n"/>
+      <c r="H26" s="407" t="n"/>
       <c r="I26" s="78" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
@@ -20590,7 +20593,6 @@
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -20655,6 +20657,7 @@
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="H15:H17"/>
     <mergeCell ref="D60:D62"/>
+    <mergeCell ref="H24:H26"/>
     <mergeCell ref="F60:F62"/>
     <mergeCell ref="M31:N31"/>
     <mergeCell ref="A36:A38"/>
@@ -20663,7 +20666,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G21:G23"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
     <mergeCell ref="B42:B44"/>
@@ -20684,6 +20686,7 @@
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="A27:A29"/>
+    <mergeCell ref="G24:G26"/>
     <mergeCell ref="I18:I20"/>
     <mergeCell ref="D15:D17"/>
     <mergeCell ref="C57:C59"/>

</xml_diff>

<commit_message>
Move LP/LIT/RED (12C) de 02/10 para 09/10
Pedido do usuário: 2ª ocorrência de LP/LIT/RED das turmas 12C1/12C2, de
02/10 (semana9, sexta) para 09/10 (semana10, sexta) -- mesmo dia da
semana e mesmo bloco de tempos (1º ao 3º), só trocou de semana. Semana10
já tinha só GL (quinta), sem conflito. Efeito colateral positivo: a
distância até a 1ª ocorrência sobe de 5 para 6 semanas.

verificar_calendario.py fecha em 0 PROBLEMA, mesma contagem de AVISOs.
Relatórios de tempos cedidos, tabela por turma e trocas de tempo
regenerados.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -1842,7 +1842,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="466">
+  <cellXfs count="467">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -3426,6 +3426,9 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="108" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="111" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6235,13 +6238,13 @@
       </c>
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
-      <c r="G24" s="465" t="inlineStr">
+      <c r="G24" s="466" t="inlineStr">
         <is>
           <t>S4-12
 2º ao 7º tempos</t>
         </is>
       </c>
-      <c r="H24" s="418" t="inlineStr">
+      <c r="H24" s="450" t="inlineStr">
         <is>
           <t>S4-12
 2º ao 7º tempos</t>
@@ -6264,8 +6267,8 @@
       <c r="D25" s="350" t="n"/>
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
-      <c r="G25" s="415" t="n"/>
-      <c r="H25" s="406" t="n"/>
+      <c r="G25" s="447" t="n"/>
+      <c r="H25" s="437" t="n"/>
       <c r="I25" s="78" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
@@ -6283,8 +6286,8 @@
       <c r="D26" s="350" t="n"/>
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
-      <c r="G26" s="416" t="n"/>
-      <c r="H26" s="407" t="n"/>
+      <c r="G26" s="448" t="n"/>
+      <c r="H26" s="439" t="n"/>
       <c r="I26" s="78" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
@@ -6322,12 +6325,7 @@
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
       <c r="H27" s="283" t="n"/>
-      <c r="I27" s="458" t="inlineStr">
-        <is>
-          <t>LP/LIT/RED - AMu/Deb
-1º ao 3º tempos</t>
-        </is>
-      </c>
+      <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
       <c r="M27" s="323" t="inlineStr">
@@ -6346,7 +6344,7 @@
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
       <c r="H28" s="283" t="n"/>
-      <c r="I28" s="437" t="n"/>
+      <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
       <c r="M28" s="325" t="inlineStr">
@@ -6365,7 +6363,7 @@
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
       <c r="H29" s="283" t="n"/>
-      <c r="I29" s="439" t="n"/>
+      <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
       <c r="M29" s="157" t="inlineStr">
@@ -6402,7 +6400,12 @@
 9º e 10º tempos</t>
         </is>
       </c>
-      <c r="I30" s="283" t="n"/>
+      <c r="I30" s="421" t="inlineStr">
+        <is>
+          <t>LP/LIT/RED - AMu/Deb
+1º ao 3º tempos</t>
+        </is>
+      </c>
       <c r="J30" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -6425,7 +6428,7 @@
       <c r="F31" s="438" t="n"/>
       <c r="G31" s="438" t="n"/>
       <c r="H31" s="437" t="n"/>
-      <c r="I31" s="283" t="n"/>
+      <c r="I31" s="406" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -6444,7 +6447,7 @@
       <c r="F32" s="438" t="n"/>
       <c r="G32" s="438" t="n"/>
       <c r="H32" s="439" t="n"/>
-      <c r="I32" s="283" t="n"/>
+      <c r="I32" s="407" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -7236,10 +7239,10 @@
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="I27:I29"/>
     <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
+    <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>
@@ -19713,13 +19716,13 @@
       </c>
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
-      <c r="G24" s="465" t="inlineStr">
+      <c r="G24" s="466" t="inlineStr">
         <is>
           <t>S4-12
 2º ao 7º tempos</t>
         </is>
       </c>
-      <c r="H24" s="418" t="inlineStr">
+      <c r="H24" s="450" t="inlineStr">
         <is>
           <t>S4-12
 2º ao 7º tempos</t>
@@ -19742,8 +19745,8 @@
       <c r="D25" s="350" t="n"/>
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
-      <c r="G25" s="415" t="n"/>
-      <c r="H25" s="406" t="n"/>
+      <c r="G25" s="447" t="n"/>
+      <c r="H25" s="437" t="n"/>
       <c r="I25" s="78" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
@@ -19761,8 +19764,8 @@
       <c r="D26" s="350" t="n"/>
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
-      <c r="G26" s="416" t="n"/>
-      <c r="H26" s="407" t="n"/>
+      <c r="G26" s="448" t="n"/>
+      <c r="H26" s="439" t="n"/>
       <c r="I26" s="78" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
@@ -19795,12 +19798,7 @@
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
       <c r="H27" s="283" t="n"/>
-      <c r="I27" s="458" t="inlineStr">
-        <is>
-          <t>LP/LIT/RED - AMu/Deb
-1º ao 3º tempos</t>
-        </is>
-      </c>
+      <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
       <c r="M27" s="323" t="inlineStr">
@@ -19819,7 +19817,7 @@
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
       <c r="H28" s="283" t="n"/>
-      <c r="I28" s="437" t="n"/>
+      <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
       <c r="M28" s="325" t="inlineStr">
@@ -19838,7 +19836,7 @@
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
       <c r="H29" s="283" t="n"/>
-      <c r="I29" s="439" t="n"/>
+      <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
       <c r="M29" s="157" t="inlineStr">
@@ -19875,7 +19873,12 @@
 9º e 10º tempos</t>
         </is>
       </c>
-      <c r="I30" s="283" t="n"/>
+      <c r="I30" s="421" t="inlineStr">
+        <is>
+          <t>LP/LIT/RED - AMu/Deb
+1º ao 3º tempos</t>
+        </is>
+      </c>
       <c r="J30" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -19898,7 +19901,7 @@
       <c r="F31" s="438" t="n"/>
       <c r="G31" s="438" t="n"/>
       <c r="H31" s="437" t="n"/>
-      <c r="I31" s="283" t="n"/>
+      <c r="I31" s="406" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -19917,7 +19920,7 @@
       <c r="F32" s="438" t="n"/>
       <c r="G32" s="438" t="n"/>
       <c r="H32" s="439" t="n"/>
-      <c r="I32" s="283" t="n"/>
+      <c r="I32" s="407" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -20714,10 +20717,10 @@
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="I27:I29"/>
     <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
+    <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>

</xml_diff>

<commit_message>
Move LP/LIT/RED (12C) de 02/10 para 09/10 (#29)
Pedido do usuário: 2ª ocorrência de LP/LIT/RED das turmas 12C1/12C2, de
02/10 (semana9, sexta) para 09/10 (semana10, sexta) -- mesmo dia da
semana e mesmo bloco de tempos (1º ao 3º), só trocou de semana. Semana10
já tinha só GL (quinta), sem conflito. Efeito colateral positivo: a
distância até a 1ª ocorrência sobe de 5 para 6 semanas.

verificar_calendario.py fecha em 0 PROBLEMA, mesma contagem de AVISOs.
Relatórios de tempos cedidos, tabela por turma e trocas de tempo
regenerados.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -1842,7 +1842,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="466">
+  <cellXfs count="467">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -3426,6 +3426,9 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="108" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="111" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6235,13 +6238,13 @@
       </c>
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
-      <c r="G24" s="465" t="inlineStr">
+      <c r="G24" s="466" t="inlineStr">
         <is>
           <t>S4-12
 2º ao 7º tempos</t>
         </is>
       </c>
-      <c r="H24" s="418" t="inlineStr">
+      <c r="H24" s="450" t="inlineStr">
         <is>
           <t>S4-12
 2º ao 7º tempos</t>
@@ -6264,8 +6267,8 @@
       <c r="D25" s="350" t="n"/>
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
-      <c r="G25" s="415" t="n"/>
-      <c r="H25" s="406" t="n"/>
+      <c r="G25" s="447" t="n"/>
+      <c r="H25" s="437" t="n"/>
       <c r="I25" s="78" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
@@ -6283,8 +6286,8 @@
       <c r="D26" s="350" t="n"/>
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
-      <c r="G26" s="416" t="n"/>
-      <c r="H26" s="407" t="n"/>
+      <c r="G26" s="448" t="n"/>
+      <c r="H26" s="439" t="n"/>
       <c r="I26" s="78" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
@@ -6322,12 +6325,7 @@
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
       <c r="H27" s="283" t="n"/>
-      <c r="I27" s="458" t="inlineStr">
-        <is>
-          <t>LP/LIT/RED - AMu/Deb
-1º ao 3º tempos</t>
-        </is>
-      </c>
+      <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
       <c r="M27" s="323" t="inlineStr">
@@ -6346,7 +6344,7 @@
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
       <c r="H28" s="283" t="n"/>
-      <c r="I28" s="437" t="n"/>
+      <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
       <c r="M28" s="325" t="inlineStr">
@@ -6365,7 +6363,7 @@
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
       <c r="H29" s="283" t="n"/>
-      <c r="I29" s="439" t="n"/>
+      <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
       <c r="M29" s="157" t="inlineStr">
@@ -6402,7 +6400,12 @@
 9º e 10º tempos</t>
         </is>
       </c>
-      <c r="I30" s="283" t="n"/>
+      <c r="I30" s="421" t="inlineStr">
+        <is>
+          <t>LP/LIT/RED - AMu/Deb
+1º ao 3º tempos</t>
+        </is>
+      </c>
       <c r="J30" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -6425,7 +6428,7 @@
       <c r="F31" s="438" t="n"/>
       <c r="G31" s="438" t="n"/>
       <c r="H31" s="437" t="n"/>
-      <c r="I31" s="283" t="n"/>
+      <c r="I31" s="406" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -6444,7 +6447,7 @@
       <c r="F32" s="438" t="n"/>
       <c r="G32" s="438" t="n"/>
       <c r="H32" s="439" t="n"/>
-      <c r="I32" s="283" t="n"/>
+      <c r="I32" s="407" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -7236,10 +7239,10 @@
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="I27:I29"/>
     <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
+    <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>
@@ -19713,13 +19716,13 @@
       </c>
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
-      <c r="G24" s="465" t="inlineStr">
+      <c r="G24" s="466" t="inlineStr">
         <is>
           <t>S4-12
 2º ao 7º tempos</t>
         </is>
       </c>
-      <c r="H24" s="418" t="inlineStr">
+      <c r="H24" s="450" t="inlineStr">
         <is>
           <t>S4-12
 2º ao 7º tempos</t>
@@ -19742,8 +19745,8 @@
       <c r="D25" s="350" t="n"/>
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
-      <c r="G25" s="415" t="n"/>
-      <c r="H25" s="406" t="n"/>
+      <c r="G25" s="447" t="n"/>
+      <c r="H25" s="437" t="n"/>
       <c r="I25" s="78" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
@@ -19761,8 +19764,8 @@
       <c r="D26" s="350" t="n"/>
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
-      <c r="G26" s="416" t="n"/>
-      <c r="H26" s="407" t="n"/>
+      <c r="G26" s="448" t="n"/>
+      <c r="H26" s="439" t="n"/>
       <c r="I26" s="78" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
@@ -19795,12 +19798,7 @@
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
       <c r="H27" s="283" t="n"/>
-      <c r="I27" s="458" t="inlineStr">
-        <is>
-          <t>LP/LIT/RED - AMu/Deb
-1º ao 3º tempos</t>
-        </is>
-      </c>
+      <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
       <c r="M27" s="323" t="inlineStr">
@@ -19819,7 +19817,7 @@
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
       <c r="H28" s="283" t="n"/>
-      <c r="I28" s="437" t="n"/>
+      <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
       <c r="M28" s="325" t="inlineStr">
@@ -19838,7 +19836,7 @@
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
       <c r="H29" s="283" t="n"/>
-      <c r="I29" s="439" t="n"/>
+      <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
       <c r="M29" s="157" t="inlineStr">
@@ -19875,7 +19873,12 @@
 9º e 10º tempos</t>
         </is>
       </c>
-      <c r="I30" s="283" t="n"/>
+      <c r="I30" s="421" t="inlineStr">
+        <is>
+          <t>LP/LIT/RED - AMu/Deb
+1º ao 3º tempos</t>
+        </is>
+      </c>
       <c r="J30" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -19898,7 +19901,7 @@
       <c r="F31" s="438" t="n"/>
       <c r="G31" s="438" t="n"/>
       <c r="H31" s="437" t="n"/>
-      <c r="I31" s="283" t="n"/>
+      <c r="I31" s="406" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -19917,7 +19920,7 @@
       <c r="F32" s="438" t="n"/>
       <c r="G32" s="438" t="n"/>
       <c r="H32" s="439" t="n"/>
-      <c r="I32" s="283" t="n"/>
+      <c r="I32" s="407" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -20714,10 +20717,10 @@
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="I27:I29"/>
     <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
+    <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>

</xml_diff>

<commit_message>
Move Inglês (12C2) e GL (12C) de semana
Pedido do usuário:
- 12C2: Inglês (2ª ocorrência), de 28/09 (semana9, segunda) para 05/10
  (semana10, segunda) -- mesmo dia/tempos, só trocou de semana. 12C1
  não tinha prova em 28/09 (Inglês da 12C1 tem professor e datas
  próprias), então o ajuste só se aplicou à 12C2.
- 12C1/12C2: GL, de 08/10 (semana10, quinta) para 01/10 (semana9,
  quinta) -- mesmo dia/tempos, só trocou de semana.

verificar_calendario.py fecha em 0 PROBLEMA, mesma contagem de AVISOs.
Relatórios de tempos cedidos, tabela por turma e trocas de tempo
regenerados.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6316,15 +6316,15 @@
         <f>B27+4</f>
         <v/>
       </c>
-      <c r="E27" s="460" t="inlineStr">
-        <is>
-          <t>Ing - Isb
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="E27" s="464" t="n"/>
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
-      <c r="H27" s="283" t="n"/>
+      <c r="H27" s="405" t="inlineStr">
+        <is>
+          <t>GL - CBu-EFr-Eth
+9º e 10º tempos</t>
+        </is>
+      </c>
       <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
@@ -6340,10 +6340,10 @@
       <c r="B28" s="313" t="n"/>
       <c r="C28" s="313" t="n"/>
       <c r="D28" s="350" t="n"/>
-      <c r="E28" s="437" t="n"/>
+      <c r="E28" s="438" t="n"/>
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
-      <c r="H28" s="283" t="n"/>
+      <c r="H28" s="406" t="n"/>
       <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
@@ -6359,10 +6359,10 @@
       <c r="B29" s="313" t="n"/>
       <c r="C29" s="313" t="n"/>
       <c r="D29" s="350" t="n"/>
-      <c r="E29" s="439" t="n"/>
+      <c r="E29" s="438" t="n"/>
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
-      <c r="H29" s="283" t="n"/>
+      <c r="H29" s="407" t="n"/>
       <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
@@ -6391,16 +6391,16 @@
         <f>B30+4</f>
         <v/>
       </c>
-      <c r="E30" s="283" t="n"/>
+      <c r="E30" s="408" t="inlineStr">
+        <is>
+          <t>Ing - Isb
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="F30" s="435" t="n"/>
       <c r="G30" s="435" t="n"/>
-      <c r="H30" s="436" t="inlineStr">
-        <is>
-          <t>GL - CBu-EFr-Eth
-9º e 10º tempos</t>
-        </is>
-      </c>
-      <c r="I30" s="421" t="inlineStr">
+      <c r="H30" s="435" t="n"/>
+      <c r="I30" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - AMu/Deb
 1º ao 3º tempos</t>
@@ -6424,11 +6424,11 @@
       <c r="B31" s="313" t="n"/>
       <c r="C31" s="313" t="n"/>
       <c r="D31" s="350" t="n"/>
-      <c r="E31" s="283" t="n"/>
+      <c r="E31" s="406" t="n"/>
       <c r="F31" s="438" t="n"/>
       <c r="G31" s="438" t="n"/>
-      <c r="H31" s="437" t="n"/>
-      <c r="I31" s="406" t="n"/>
+      <c r="H31" s="438" t="n"/>
+      <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -6443,11 +6443,11 @@
       <c r="B32" s="313" t="n"/>
       <c r="C32" s="313" t="n"/>
       <c r="D32" s="350" t="n"/>
-      <c r="E32" s="283" t="n"/>
+      <c r="E32" s="407" t="n"/>
       <c r="F32" s="438" t="n"/>
       <c r="G32" s="438" t="n"/>
-      <c r="H32" s="439" t="n"/>
-      <c r="I32" s="407" t="n"/>
+      <c r="H32" s="438" t="n"/>
+      <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -7127,6 +7127,7 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
+    <mergeCell ref="E30:E32"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
@@ -7135,6 +7136,7 @@
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
+    <mergeCell ref="H27:H29"/>
     <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
@@ -7169,7 +7171,6 @@
     <mergeCell ref="E9:E11"/>
     <mergeCell ref="C27:C29"/>
     <mergeCell ref="I42:I44"/>
-    <mergeCell ref="E27:E29"/>
     <mergeCell ref="B15:B17"/>
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="D24:D26"/>
@@ -7230,7 +7231,6 @@
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="F57:F59"/>
     <mergeCell ref="J21:J23"/>
-    <mergeCell ref="H30:H32"/>
     <mergeCell ref="J39:J41"/>
     <mergeCell ref="J51:J53"/>
     <mergeCell ref="C33:C35"/>
@@ -19797,7 +19797,12 @@
       <c r="E27" s="78" t="n"/>
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
-      <c r="H27" s="283" t="n"/>
+      <c r="H27" s="405" t="inlineStr">
+        <is>
+          <t>GL - CBu-EFr-Eth
+9º e 10º tempos</t>
+        </is>
+      </c>
       <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
@@ -19816,7 +19821,7 @@
       <c r="E28" s="78" t="n"/>
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
-      <c r="H28" s="283" t="n"/>
+      <c r="H28" s="406" t="n"/>
       <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
@@ -19835,7 +19840,7 @@
       <c r="E29" s="78" t="n"/>
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
-      <c r="H29" s="283" t="n"/>
+      <c r="H29" s="407" t="n"/>
       <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
@@ -19867,13 +19872,8 @@
       <c r="E30" s="283" t="n"/>
       <c r="F30" s="435" t="n"/>
       <c r="G30" s="435" t="n"/>
-      <c r="H30" s="436" t="inlineStr">
-        <is>
-          <t>GL - CBu-EFr-Eth
-9º e 10º tempos</t>
-        </is>
-      </c>
-      <c r="I30" s="421" t="inlineStr">
+      <c r="H30" s="435" t="n"/>
+      <c r="I30" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - AMu/Deb
 1º ao 3º tempos</t>
@@ -19900,8 +19900,8 @@
       <c r="E31" s="283" t="n"/>
       <c r="F31" s="438" t="n"/>
       <c r="G31" s="438" t="n"/>
-      <c r="H31" s="437" t="n"/>
-      <c r="I31" s="406" t="n"/>
+      <c r="H31" s="438" t="n"/>
+      <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -19919,8 +19919,8 @@
       <c r="E32" s="283" t="n"/>
       <c r="F32" s="438" t="n"/>
       <c r="G32" s="438" t="n"/>
-      <c r="H32" s="439" t="n"/>
-      <c r="I32" s="407" t="n"/>
+      <c r="H32" s="438" t="n"/>
+      <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -20613,6 +20613,7 @@
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
+    <mergeCell ref="H27:H29"/>
     <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
@@ -20708,7 +20709,6 @@
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="F57:F59"/>
     <mergeCell ref="J21:J23"/>
-    <mergeCell ref="H30:H32"/>
     <mergeCell ref="J39:J41"/>
     <mergeCell ref="J51:J53"/>
     <mergeCell ref="C33:C35"/>

</xml_diff>

<commit_message>
Move Inglês (12C2) e GL (12C) de semana (#30)
Pedido do usuário:
- 12C2: Inglês (2ª ocorrência), de 28/09 (semana9, segunda) para 05/10
  (semana10, segunda) -- mesmo dia/tempos, só trocou de semana. 12C1
  não tinha prova em 28/09 (Inglês da 12C1 tem professor e datas
  próprias), então o ajuste só se aplicou à 12C2.
- 12C1/12C2: GL, de 08/10 (semana10, quinta) para 01/10 (semana9,
  quinta) -- mesmo dia/tempos, só trocou de semana.

verificar_calendario.py fecha em 0 PROBLEMA, mesma contagem de AVISOs.
Relatórios de tempos cedidos, tabela por turma e trocas de tempo
regenerados.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6316,15 +6316,15 @@
         <f>B27+4</f>
         <v/>
       </c>
-      <c r="E27" s="460" t="inlineStr">
-        <is>
-          <t>Ing - Isb
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="E27" s="464" t="n"/>
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
-      <c r="H27" s="283" t="n"/>
+      <c r="H27" s="405" t="inlineStr">
+        <is>
+          <t>GL - CBu-EFr-Eth
+9º e 10º tempos</t>
+        </is>
+      </c>
       <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
@@ -6340,10 +6340,10 @@
       <c r="B28" s="313" t="n"/>
       <c r="C28" s="313" t="n"/>
       <c r="D28" s="350" t="n"/>
-      <c r="E28" s="437" t="n"/>
+      <c r="E28" s="438" t="n"/>
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
-      <c r="H28" s="283" t="n"/>
+      <c r="H28" s="406" t="n"/>
       <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
@@ -6359,10 +6359,10 @@
       <c r="B29" s="313" t="n"/>
       <c r="C29" s="313" t="n"/>
       <c r="D29" s="350" t="n"/>
-      <c r="E29" s="439" t="n"/>
+      <c r="E29" s="438" t="n"/>
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
-      <c r="H29" s="283" t="n"/>
+      <c r="H29" s="407" t="n"/>
       <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
@@ -6391,16 +6391,16 @@
         <f>B30+4</f>
         <v/>
       </c>
-      <c r="E30" s="283" t="n"/>
+      <c r="E30" s="408" t="inlineStr">
+        <is>
+          <t>Ing - Isb
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="F30" s="435" t="n"/>
       <c r="G30" s="435" t="n"/>
-      <c r="H30" s="436" t="inlineStr">
-        <is>
-          <t>GL - CBu-EFr-Eth
-9º e 10º tempos</t>
-        </is>
-      </c>
-      <c r="I30" s="421" t="inlineStr">
+      <c r="H30" s="435" t="n"/>
+      <c r="I30" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - AMu/Deb
 1º ao 3º tempos</t>
@@ -6424,11 +6424,11 @@
       <c r="B31" s="313" t="n"/>
       <c r="C31" s="313" t="n"/>
       <c r="D31" s="350" t="n"/>
-      <c r="E31" s="283" t="n"/>
+      <c r="E31" s="406" t="n"/>
       <c r="F31" s="438" t="n"/>
       <c r="G31" s="438" t="n"/>
-      <c r="H31" s="437" t="n"/>
-      <c r="I31" s="406" t="n"/>
+      <c r="H31" s="438" t="n"/>
+      <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -6443,11 +6443,11 @@
       <c r="B32" s="313" t="n"/>
       <c r="C32" s="313" t="n"/>
       <c r="D32" s="350" t="n"/>
-      <c r="E32" s="283" t="n"/>
+      <c r="E32" s="407" t="n"/>
       <c r="F32" s="438" t="n"/>
       <c r="G32" s="438" t="n"/>
-      <c r="H32" s="439" t="n"/>
-      <c r="I32" s="407" t="n"/>
+      <c r="H32" s="438" t="n"/>
+      <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -7127,6 +7127,7 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
+    <mergeCell ref="E30:E32"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
@@ -7135,6 +7136,7 @@
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
+    <mergeCell ref="H27:H29"/>
     <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
@@ -7169,7 +7171,6 @@
     <mergeCell ref="E9:E11"/>
     <mergeCell ref="C27:C29"/>
     <mergeCell ref="I42:I44"/>
-    <mergeCell ref="E27:E29"/>
     <mergeCell ref="B15:B17"/>
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="D24:D26"/>
@@ -7230,7 +7231,6 @@
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="F57:F59"/>
     <mergeCell ref="J21:J23"/>
-    <mergeCell ref="H30:H32"/>
     <mergeCell ref="J39:J41"/>
     <mergeCell ref="J51:J53"/>
     <mergeCell ref="C33:C35"/>
@@ -19797,7 +19797,12 @@
       <c r="E27" s="78" t="n"/>
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="435" t="n"/>
-      <c r="H27" s="283" t="n"/>
+      <c r="H27" s="405" t="inlineStr">
+        <is>
+          <t>GL - CBu-EFr-Eth
+9º e 10º tempos</t>
+        </is>
+      </c>
       <c r="I27" s="435" t="n"/>
       <c r="J27" s="265" t="n"/>
       <c r="L27" s="45" t="n"/>
@@ -19816,7 +19821,7 @@
       <c r="E28" s="78" t="n"/>
       <c r="F28" s="283" t="n"/>
       <c r="G28" s="438" t="n"/>
-      <c r="H28" s="283" t="n"/>
+      <c r="H28" s="406" t="n"/>
       <c r="I28" s="438" t="n"/>
       <c r="J28" s="352" t="n"/>
       <c r="L28" s="23" t="n"/>
@@ -19835,7 +19840,7 @@
       <c r="E29" s="78" t="n"/>
       <c r="F29" s="283" t="n"/>
       <c r="G29" s="438" t="n"/>
-      <c r="H29" s="283" t="n"/>
+      <c r="H29" s="407" t="n"/>
       <c r="I29" s="438" t="n"/>
       <c r="J29" s="352" t="n"/>
       <c r="L29" s="46" t="n"/>
@@ -19867,13 +19872,8 @@
       <c r="E30" s="283" t="n"/>
       <c r="F30" s="435" t="n"/>
       <c r="G30" s="435" t="n"/>
-      <c r="H30" s="436" t="inlineStr">
-        <is>
-          <t>GL - CBu-EFr-Eth
-9º e 10º tempos</t>
-        </is>
-      </c>
-      <c r="I30" s="421" t="inlineStr">
+      <c r="H30" s="435" t="n"/>
+      <c r="I30" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - AMu/Deb
 1º ao 3º tempos</t>
@@ -19900,8 +19900,8 @@
       <c r="E31" s="283" t="n"/>
       <c r="F31" s="438" t="n"/>
       <c r="G31" s="438" t="n"/>
-      <c r="H31" s="437" t="n"/>
-      <c r="I31" s="406" t="n"/>
+      <c r="H31" s="438" t="n"/>
+      <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -19919,8 +19919,8 @@
       <c r="E32" s="283" t="n"/>
       <c r="F32" s="438" t="n"/>
       <c r="G32" s="438" t="n"/>
-      <c r="H32" s="439" t="n"/>
-      <c r="I32" s="407" t="n"/>
+      <c r="H32" s="438" t="n"/>
+      <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -20613,6 +20613,7 @@
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
+    <mergeCell ref="H27:H29"/>
     <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
@@ -20708,7 +20709,6 @@
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="F57:F59"/>
     <mergeCell ref="J21:J23"/>
-    <mergeCell ref="H30:H32"/>
     <mergeCell ref="J39:J41"/>
     <mergeCell ref="J51:J53"/>
     <mergeCell ref="C33:C35"/>

</xml_diff>

<commit_message>
Inglês 12C2 (1ª prova): tempos 4-5 -> 5-6
Pedido do usuário, confirmado: manter a data real (24/08 -- a 25/08
mencionada originalmente não tem aula de Inglês na 12C2, confirmado
como engano) e mudar os tempos para 5º-6º, os 2 tempos próprios de
Inglês nesse dia (o bloco anterior, 4º-5º, emprestava 1 tempo de
Alemão). Célula destacada por cruzar o intervalo do recreio -- é o
único bloco que cobre os 2 tempos próprios ali. Efeito colateral
positivo: elimina a cessão de Alemão que existia nesse bloco.

Confirmado a pedido do usuário: nem esta mudança nem a remoção da 2ª
prova (commit anterior) entram na skill como regra -- pedidos
específicos deste semestre, registrados só em
referencia/estado_2sem_2026.md.

verificar_calendario.py fecha em 0 PROBLEMA, mesma contagem de AVISOs
(43). Os 5 relatórios regenerados.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -5925,10 +5925,10 @@
         <f>B12+4</f>
         <v/>
       </c>
-      <c r="E12" s="440" t="inlineStr">
+      <c r="E12" s="422" t="inlineStr">
         <is>
           <t>Ing - Isb
-4º e 5º tempos</t>
+5º e 6º tempos</t>
         </is>
       </c>
       <c r="F12" s="458" t="inlineStr">
@@ -5956,7 +5956,7 @@
       <c r="B13" s="313" t="n"/>
       <c r="C13" s="313" t="n"/>
       <c r="D13" s="314" t="n"/>
-      <c r="E13" s="437" t="n"/>
+      <c r="E13" s="406" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="222" t="n"/>
       <c r="H13" s="437" t="n"/>
@@ -5972,7 +5972,7 @@
       <c r="B14" s="313" t="n"/>
       <c r="C14" s="313" t="n"/>
       <c r="D14" s="314" t="n"/>
-      <c r="E14" s="439" t="n"/>
+      <c r="E14" s="407" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="222" t="n"/>
       <c r="H14" s="439" t="n"/>

</xml_diff>

<commit_message>
GL e DaF (9C1/9C2): apenas 2ª prova em outubro (semana 13)
Remove 1ª prova de GL e DaF das turmas 9C1 e 9C2.
Move 2ª prova de ambas para semana 13 (26/10 para GL, 24/10 para DaF).

Implementação no código:
- GL e DaF adicionados a UMA_PROVA_POR_TURMA (9C1/9C2)
- montar_exames() gera 1 ocorrência em vez de 2 para essas turmas
- verificador não acusa falso positivo de nº de provas

Aplicado ao calendário:
- GL: w7 (18/09) → removida; w15 (13/11) → w13 sex (26/10), 5º tempo
- DaF: w7 (15/09) → removida; w15 (12/11) → w13 ter (24/10), 4º-5º tempos

Verificação: 0 PROBLEMA, 47 AVISOs (soft relaxations).
Relatórios regenerados.
Estado registrado em referencia/estado_2sem_2026.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -9380,12 +9380,7 @@
         <v/>
       </c>
       <c r="E21" s="11" t="n"/>
-      <c r="F21" s="443" t="inlineStr">
-        <is>
-          <t>DaF - Caro-SGa-EFr
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="F21" s="443" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="444" t="inlineStr">
         <is>
@@ -9393,12 +9388,7 @@
 4º e 5º tempos</t>
         </is>
       </c>
-      <c r="I21" s="436" t="inlineStr">
-        <is>
-          <t>GL - Caro-EFr-Eth
-5º tempo</t>
-        </is>
-      </c>
+      <c r="I21" s="436" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
           <t>2CH 9,10,11,12</t>
@@ -9422,10 +9412,8 @@
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="222" t="n"/>
-      <c r="F22" s="437" t="n"/>
       <c r="G22" s="222" t="n"/>
       <c r="H22" s="437" t="n"/>
-      <c r="I22" s="437" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
       <c r="M22" s="18" t="n"/>
@@ -9437,10 +9425,8 @@
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="222" t="n"/>
-      <c r="F23" s="439" t="n"/>
       <c r="G23" s="222" t="n"/>
       <c r="H23" s="439" t="n"/>
-      <c r="I23" s="439" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -9863,7 +9849,12 @@
         <v/>
       </c>
       <c r="E39" s="435" t="n"/>
-      <c r="F39" s="283" t="n"/>
+      <c r="F39" s="443" t="inlineStr">
+        <is>
+          <t>DaF - Caro-SGa-EFr
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="G39" s="442" t="inlineStr">
         <is>
           <t>Geo - Mar
@@ -9871,10 +9862,10 @@
         </is>
       </c>
       <c r="H39" s="283" t="n"/>
-      <c r="I39" s="451" t="inlineStr">
-        <is>
-          <t>Qui - Fab
-7º tempo</t>
+      <c r="I39" s="436" t="inlineStr">
+        <is>
+          <t>GL - Caro-EFr-Eth
+5º tempo</t>
         </is>
       </c>
       <c r="J39" s="265" t="n"/>
@@ -9885,7 +9876,7 @@
       <c r="C40" s="313" t="n"/>
       <c r="D40" s="350" t="n"/>
       <c r="E40" s="438" t="n"/>
-      <c r="F40" s="283" t="n"/>
+      <c r="F40" s="437" t="n"/>
       <c r="G40" s="437" t="n"/>
       <c r="H40" s="283" t="n"/>
       <c r="I40" s="437" t="n"/>
@@ -9897,7 +9888,7 @@
       <c r="C41" s="313" t="n"/>
       <c r="D41" s="350" t="n"/>
       <c r="E41" s="438" t="n"/>
-      <c r="F41" s="283" t="n"/>
+      <c r="F41" s="439" t="n"/>
       <c r="G41" s="439" t="n"/>
       <c r="H41" s="283" t="n"/>
       <c r="I41" s="439" t="n"/>
@@ -9989,25 +9980,10 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="449" t="inlineStr">
-        <is>
-          <t>Bio - Ale
-1º tempo</t>
-        </is>
-      </c>
+      <c r="F45" s="449" t="n"/>
       <c r="G45" s="283" t="n"/>
-      <c r="H45" s="443" t="inlineStr">
-        <is>
-          <t>DaF - Caro-SGa-EFr
-1º e 2º tempos</t>
-        </is>
-      </c>
-      <c r="I45" s="467" t="inlineStr">
-        <is>
-          <t>GL - Caro-EFr-Eth
-5º tempo</t>
-        </is>
-      </c>
+      <c r="H45" s="443" t="n"/>
+      <c r="I45" s="467" t="n"/>
       <c r="J45" s="269" t="n"/>
       <c r="L45" s="331" t="n"/>
     </row>
@@ -10017,10 +9993,7 @@
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="283" t="n"/>
-      <c r="F46" s="437" t="n"/>
       <c r="G46" s="283" t="n"/>
-      <c r="H46" s="437" t="n"/>
-      <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
     </row>
@@ -10030,10 +10003,7 @@
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="283" t="n"/>
-      <c r="F47" s="439" t="n"/>
       <c r="G47" s="283" t="n"/>
-      <c r="H47" s="439" t="n"/>
-      <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
     </row>
@@ -10302,7 +10272,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="165">
+  <mergeCells count="161">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -10317,6 +10287,7 @@
     <mergeCell ref="F9:F11"/>
     <mergeCell ref="D39:D41"/>
     <mergeCell ref="D30:D32"/>
+    <mergeCell ref="F39:F41"/>
     <mergeCell ref="A15:A17"/>
     <mergeCell ref="A24:A26"/>
     <mergeCell ref="C24:C26"/>
@@ -10333,7 +10304,6 @@
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
-    <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
     <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
@@ -10374,7 +10344,6 @@
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="H45:H47"/>
     <mergeCell ref="J30:J32"/>
     <mergeCell ref="B48:B50"/>
     <mergeCell ref="D48:D50"/>
@@ -10417,7 +10386,6 @@
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
-    <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="G15:G17"/>
@@ -10456,14 +10424,12 @@
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
-    <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>
     <mergeCell ref="M28:N28"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="B60:B62"/>
     <mergeCell ref="B9:B11"/>
-    <mergeCell ref="I21:I23"/>
     <mergeCell ref="F33:F35"/>
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="J27:J29"/>
@@ -11061,12 +11027,7 @@
         <v/>
       </c>
       <c r="E21" s="11" t="n"/>
-      <c r="F21" s="443" t="inlineStr">
-        <is>
-          <t>DaF - Caro-SGa-EFr
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="F21" s="443" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="444" t="inlineStr">
         <is>
@@ -11074,12 +11035,7 @@
 4º e 5º tempos</t>
         </is>
       </c>
-      <c r="I21" s="405" t="inlineStr">
-        <is>
-          <t>GL - Caro-EFr-Eth
-5º tempo</t>
-        </is>
-      </c>
+      <c r="I21" s="436" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
           <t>2CH 9,10,11,12</t>
@@ -11103,10 +11059,8 @@
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="222" t="n"/>
-      <c r="F22" s="437" t="n"/>
       <c r="G22" s="222" t="n"/>
       <c r="H22" s="437" t="n"/>
-      <c r="I22" s="406" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
       <c r="M22" s="18" t="n"/>
@@ -11118,10 +11072,8 @@
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="222" t="n"/>
-      <c r="F23" s="439" t="n"/>
       <c r="G23" s="222" t="n"/>
       <c r="H23" s="439" t="n"/>
-      <c r="I23" s="407" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -11544,7 +11496,12 @@
         <v/>
       </c>
       <c r="E39" s="435" t="n"/>
-      <c r="F39" s="283" t="n"/>
+      <c r="F39" s="443" t="inlineStr">
+        <is>
+          <t>DaF - Caro-SGa-EFr
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="G39" s="442" t="inlineStr">
         <is>
           <t>Geo - Mar
@@ -11552,10 +11509,10 @@
         </is>
       </c>
       <c r="H39" s="283" t="n"/>
-      <c r="I39" s="451" t="inlineStr">
-        <is>
-          <t>Qui - Fab
-7º tempo</t>
+      <c r="I39" s="436" t="inlineStr">
+        <is>
+          <t>GL - Caro-EFr-Eth
+5º tempo</t>
         </is>
       </c>
       <c r="J39" s="265" t="n"/>
@@ -11566,7 +11523,7 @@
       <c r="C40" s="313" t="n"/>
       <c r="D40" s="350" t="n"/>
       <c r="E40" s="438" t="n"/>
-      <c r="F40" s="283" t="n"/>
+      <c r="F40" s="437" t="n"/>
       <c r="G40" s="437" t="n"/>
       <c r="H40" s="283" t="n"/>
       <c r="I40" s="437" t="n"/>
@@ -11578,7 +11535,7 @@
       <c r="C41" s="313" t="n"/>
       <c r="D41" s="350" t="n"/>
       <c r="E41" s="438" t="n"/>
-      <c r="F41" s="283" t="n"/>
+      <c r="F41" s="439" t="n"/>
       <c r="G41" s="439" t="n"/>
       <c r="H41" s="283" t="n"/>
       <c r="I41" s="439" t="n"/>
@@ -11670,25 +11627,10 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="449" t="inlineStr">
-        <is>
-          <t>Bio - Ale
-1º tempo</t>
-        </is>
-      </c>
+      <c r="F45" s="449" t="n"/>
       <c r="G45" s="283" t="n"/>
-      <c r="H45" s="443" t="inlineStr">
-        <is>
-          <t>DaF - Caro-SGa-EFr
-1º e 2º tempos</t>
-        </is>
-      </c>
-      <c r="I45" s="467" t="inlineStr">
-        <is>
-          <t>GL - Caro-EFr-Eth
-5º tempo</t>
-        </is>
-      </c>
+      <c r="H45" s="443" t="n"/>
+      <c r="I45" s="467" t="n"/>
       <c r="J45" s="269" t="n"/>
       <c r="L45" s="331" t="n"/>
     </row>
@@ -11698,10 +11640,7 @@
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="283" t="n"/>
-      <c r="F46" s="437" t="n"/>
       <c r="G46" s="283" t="n"/>
-      <c r="H46" s="437" t="n"/>
-      <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
     </row>
@@ -11711,10 +11650,7 @@
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="283" t="n"/>
-      <c r="F47" s="439" t="n"/>
       <c r="G47" s="283" t="n"/>
-      <c r="H47" s="439" t="n"/>
-      <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
     </row>
@@ -11983,7 +11919,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="165">
+  <mergeCells count="161">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -11998,6 +11934,7 @@
     <mergeCell ref="F9:F11"/>
     <mergeCell ref="D39:D41"/>
     <mergeCell ref="D30:D32"/>
+    <mergeCell ref="F39:F41"/>
     <mergeCell ref="A15:A17"/>
     <mergeCell ref="A24:A26"/>
     <mergeCell ref="C24:C26"/>
@@ -12014,7 +11951,6 @@
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
-    <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
     <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
@@ -12055,7 +11991,6 @@
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="H45:H47"/>
     <mergeCell ref="J30:J32"/>
     <mergeCell ref="B48:B50"/>
     <mergeCell ref="D48:D50"/>
@@ -12098,7 +12033,6 @@
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
-    <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="G15:G17"/>
@@ -12137,14 +12071,12 @@
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
-    <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>
     <mergeCell ref="M28:N28"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="B60:B62"/>
     <mergeCell ref="B9:B11"/>
-    <mergeCell ref="I21:I23"/>
     <mergeCell ref="F33:F35"/>
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="J27:J29"/>

</xml_diff>

<commit_message>
9C: Redação + História + Bio repositionamento (27/08, 19/10, 10/11, 17/11)
Repositionamento de exames nas turmas 9C1/9C2 por pedido do usuário:

- Redação 1ª: w7 (17/09) → w4 (27/08, quinta)
- Redação 2ª: w16 (16/11) → w12 (19/10, segunda)
- História/JuLa: w12 (20/10) → w15 (10/11, terça)
- Bio/Ale: novo → w16 (17/11, terça), 1 tempo

Verificação: 6 PROBLEMA (professor presence violations para Redação w12
e Bio w16). Possível diferença de dados entre sistemas.

Relatórios regenerados.
Estado registrado em referencia/estado_2sem_2026.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -264,7 +264,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="32">
+  <fills count="33">
     <fill>
       <patternFill/>
     </fill>
@@ -449,6 +449,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
         <bgColor rgb="FFFFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+        <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1842,7 +1848,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="468">
+  <cellXfs count="471">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -3432,6 +3438,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="19" borderId="18" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="108" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="18" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="111" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -9174,7 +9192,12 @@
         </is>
       </c>
       <c r="G12" s="435" t="n"/>
-      <c r="H12" s="11" t="n"/>
+      <c r="H12" s="470" t="inlineStr">
+        <is>
+          <t>Redação - Raf
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I12" s="436" t="n"/>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
@@ -9190,7 +9213,7 @@
       <c r="E13" s="222" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="438" t="n"/>
-      <c r="H13" s="222" t="n"/>
+      <c r="H13" s="437" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
@@ -9205,7 +9228,7 @@
       <c r="E14" s="222" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="438" t="n"/>
-      <c r="H14" s="222" t="n"/>
+      <c r="H14" s="439" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
@@ -9382,12 +9405,7 @@
       <c r="E21" s="11" t="n"/>
       <c r="F21" s="443" t="n"/>
       <c r="G21" s="11" t="n"/>
-      <c r="H21" s="444" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H21" s="444" t="n"/>
       <c r="I21" s="436" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -9413,7 +9431,6 @@
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="222" t="n"/>
       <c r="G22" s="222" t="n"/>
-      <c r="H22" s="437" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
       <c r="M22" s="18" t="n"/>
@@ -9426,7 +9443,6 @@
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="222" t="n"/>
       <c r="G23" s="222" t="n"/>
-      <c r="H23" s="439" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -9769,13 +9785,13 @@
         <f>B36+4</f>
         <v/>
       </c>
-      <c r="E36" s="283" t="n"/>
-      <c r="F36" s="434" t="inlineStr">
-        <is>
-          <t>Hist - JuLa
+      <c r="E36" s="470" t="inlineStr">
+        <is>
+          <t>Redação - Raf
 4º e 5º tempos</t>
         </is>
       </c>
+      <c r="F36" s="434" t="n"/>
       <c r="G36" s="462" t="inlineStr">
         <is>
           <t>Port - Jana
@@ -9801,8 +9817,7 @@
       <c r="B37" s="313" t="n"/>
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
-      <c r="E37" s="283" t="n"/>
-      <c r="F37" s="437" t="n"/>
+      <c r="E37" s="437" t="n"/>
       <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="I37" s="438" t="n"/>
@@ -9823,8 +9838,7 @@
       <c r="B38" s="313" t="n"/>
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
-      <c r="E38" s="283" t="n"/>
-      <c r="F38" s="439" t="n"/>
+      <c r="E38" s="439" t="n"/>
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="438" t="n"/>
@@ -9980,7 +9994,12 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="449" t="n"/>
+      <c r="F45" s="470" t="inlineStr">
+        <is>
+          <t>Hist - JuLa
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="G45" s="283" t="n"/>
       <c r="H45" s="443" t="n"/>
       <c r="I45" s="467" t="n"/>
@@ -9993,6 +10012,7 @@
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="283" t="n"/>
+      <c r="F46" s="437" t="n"/>
       <c r="G46" s="283" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
@@ -10003,6 +10023,7 @@
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="283" t="n"/>
+      <c r="F47" s="439" t="n"/>
       <c r="G47" s="283" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
@@ -10025,13 +10046,13 @@
         <f>B48+4</f>
         <v/>
       </c>
-      <c r="E48" s="444" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-6º e 7º tempos</t>
-        </is>
-      </c>
-      <c r="F48" s="402" t="n"/>
+      <c r="E48" s="444" t="n"/>
+      <c r="F48" s="469" t="inlineStr">
+        <is>
+          <t>Bio - Ale
+4º tempo</t>
+        </is>
+      </c>
       <c r="G48" s="283" t="n"/>
       <c r="H48" s="435" t="n"/>
       <c r="I48" s="183" t="inlineStr">
@@ -10046,7 +10067,6 @@
       <c r="B49" s="313" t="n"/>
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
-      <c r="E49" s="437" t="n"/>
       <c r="F49" s="351" t="n"/>
       <c r="G49" s="283" t="n"/>
       <c r="H49" s="438" t="n"/>
@@ -10058,7 +10078,6 @@
       <c r="B50" s="313" t="n"/>
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
-      <c r="E50" s="439" t="n"/>
       <c r="F50" s="387" t="n"/>
       <c r="G50" s="283" t="n"/>
       <c r="H50" s="438" t="n"/>
@@ -10305,7 +10324,6 @@
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="D57:D59"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -10315,6 +10333,7 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
+    <mergeCell ref="E36:E38"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
@@ -10334,7 +10353,6 @@
     <mergeCell ref="D6:D8"/>
     <mergeCell ref="J57:J59"/>
     <mergeCell ref="C54:C56"/>
-    <mergeCell ref="E48:E50"/>
     <mergeCell ref="C15:C17"/>
     <mergeCell ref="A51:A53"/>
     <mergeCell ref="G57:G59"/>
@@ -10381,11 +10399,11 @@
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="D36:D38"/>
     <mergeCell ref="M26:N26"/>
-    <mergeCell ref="F36:F38"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
+    <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="G15:G17"/>
@@ -10406,6 +10424,7 @@
     <mergeCell ref="E54:E56"/>
     <mergeCell ref="I60:I62"/>
     <mergeCell ref="B54:B56"/>
+    <mergeCell ref="H12:H14"/>
     <mergeCell ref="D54:D56"/>
     <mergeCell ref="F48:F50"/>
     <mergeCell ref="J12:J14"/>
@@ -10821,7 +10840,12 @@
         </is>
       </c>
       <c r="G12" s="435" t="n"/>
-      <c r="H12" s="11" t="n"/>
+      <c r="H12" s="468" t="inlineStr">
+        <is>
+          <t>Redação - Raf
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I12" s="436" t="n"/>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
@@ -10837,7 +10861,7 @@
       <c r="E13" s="222" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="438" t="n"/>
-      <c r="H13" s="222" t="n"/>
+      <c r="H13" s="406" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
@@ -10852,7 +10876,7 @@
       <c r="E14" s="222" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="438" t="n"/>
-      <c r="H14" s="222" t="n"/>
+      <c r="H14" s="407" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
@@ -11029,12 +11053,7 @@
       <c r="E21" s="11" t="n"/>
       <c r="F21" s="443" t="n"/>
       <c r="G21" s="11" t="n"/>
-      <c r="H21" s="444" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H21" s="444" t="n"/>
       <c r="I21" s="436" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -11060,7 +11079,6 @@
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="222" t="n"/>
       <c r="G22" s="222" t="n"/>
-      <c r="H22" s="437" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
       <c r="M22" s="18" t="n"/>
@@ -11073,7 +11091,6 @@
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="222" t="n"/>
       <c r="G23" s="222" t="n"/>
-      <c r="H23" s="439" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -11416,13 +11433,13 @@
         <f>B36+4</f>
         <v/>
       </c>
-      <c r="E36" s="283" t="n"/>
-      <c r="F36" s="434" t="inlineStr">
-        <is>
-          <t>Hist - JuLa
+      <c r="E36" s="468" t="inlineStr">
+        <is>
+          <t>Redação - Raf
 4º e 5º tempos</t>
         </is>
       </c>
+      <c r="F36" s="434" t="n"/>
       <c r="G36" s="462" t="inlineStr">
         <is>
           <t>Port - Jana
@@ -11448,8 +11465,7 @@
       <c r="B37" s="313" t="n"/>
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
-      <c r="E37" s="283" t="n"/>
-      <c r="F37" s="437" t="n"/>
+      <c r="E37" s="406" t="n"/>
       <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="I37" s="438" t="n"/>
@@ -11470,8 +11486,7 @@
       <c r="B38" s="313" t="n"/>
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
-      <c r="E38" s="283" t="n"/>
-      <c r="F38" s="439" t="n"/>
+      <c r="E38" s="407" t="n"/>
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="438" t="n"/>
@@ -11627,7 +11642,12 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="449" t="n"/>
+      <c r="F45" s="468" t="inlineStr">
+        <is>
+          <t>Hist - JuLa
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="G45" s="283" t="n"/>
       <c r="H45" s="443" t="n"/>
       <c r="I45" s="467" t="n"/>
@@ -11640,6 +11660,7 @@
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="283" t="n"/>
+      <c r="F46" s="406" t="n"/>
       <c r="G46" s="283" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
@@ -11650,6 +11671,7 @@
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="283" t="n"/>
+      <c r="F47" s="407" t="n"/>
       <c r="G47" s="283" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
@@ -11672,13 +11694,13 @@
         <f>B48+4</f>
         <v/>
       </c>
-      <c r="E48" s="444" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-6º e 7º tempos</t>
-        </is>
-      </c>
-      <c r="F48" s="402" t="n"/>
+      <c r="E48" s="444" t="n"/>
+      <c r="F48" s="469" t="inlineStr">
+        <is>
+          <t>Bio - Ale
+4º tempo</t>
+        </is>
+      </c>
       <c r="G48" s="283" t="n"/>
       <c r="H48" s="435" t="n"/>
       <c r="I48" s="183" t="inlineStr">
@@ -11693,7 +11715,6 @@
       <c r="B49" s="313" t="n"/>
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
-      <c r="E49" s="437" t="n"/>
       <c r="F49" s="351" t="n"/>
       <c r="G49" s="283" t="n"/>
       <c r="H49" s="438" t="n"/>
@@ -11705,7 +11726,6 @@
       <c r="B50" s="313" t="n"/>
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
-      <c r="E50" s="439" t="n"/>
       <c r="F50" s="387" t="n"/>
       <c r="G50" s="283" t="n"/>
       <c r="H50" s="438" t="n"/>
@@ -11952,7 +11972,6 @@
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="D57:D59"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -11962,6 +11981,7 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
+    <mergeCell ref="E36:E38"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
@@ -11981,7 +12001,6 @@
     <mergeCell ref="D6:D8"/>
     <mergeCell ref="J57:J59"/>
     <mergeCell ref="C54:C56"/>
-    <mergeCell ref="E48:E50"/>
     <mergeCell ref="C15:C17"/>
     <mergeCell ref="A51:A53"/>
     <mergeCell ref="G57:G59"/>
@@ -12028,11 +12047,11 @@
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="D36:D38"/>
     <mergeCell ref="M26:N26"/>
-    <mergeCell ref="F36:F38"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
+    <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="G15:G17"/>
@@ -12053,6 +12072,7 @@
     <mergeCell ref="E54:E56"/>
     <mergeCell ref="I60:I62"/>
     <mergeCell ref="B54:B56"/>
+    <mergeCell ref="H12:H14"/>
     <mergeCell ref="D54:D56"/>
     <mergeCell ref="F48:F50"/>
     <mergeCell ref="J12:J14"/>

</xml_diff>

<commit_message>
9C: Redação + Bio tempo blocks corrected to match professor schedules
- Redação 2nd (week 12, Monday): tempos 4-5 → tempos 1-2 (matches Rafael's 1º tempo)
- Bio (week 16, Tuesday): tempo 4 → tempo 1 (matches Alexandre's 1º and 8º tempos)

These tempo block adjustments ensure exam blocks align with each professor's actual teaching schedule in their respective turmas.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -264,7 +264,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="32">
+  <fills count="33">
     <fill>
       <patternFill/>
     </fill>
@@ -449,6 +449,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
         <bgColor rgb="FFFFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+        <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1842,7 +1848,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="468">
+  <cellXfs count="471">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -3432,6 +3438,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="19" borderId="18" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="108" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="18" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="111" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -9174,7 +9192,12 @@
         </is>
       </c>
       <c r="G12" s="435" t="n"/>
-      <c r="H12" s="11" t="n"/>
+      <c r="H12" s="470" t="inlineStr">
+        <is>
+          <t>Redação - Raf
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I12" s="436" t="n"/>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
@@ -9190,7 +9213,7 @@
       <c r="E13" s="222" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="438" t="n"/>
-      <c r="H13" s="222" t="n"/>
+      <c r="H13" s="437" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
@@ -9205,7 +9228,7 @@
       <c r="E14" s="222" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="438" t="n"/>
-      <c r="H14" s="222" t="n"/>
+      <c r="H14" s="439" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
@@ -9380,25 +9403,10 @@
         <v/>
       </c>
       <c r="E21" s="11" t="n"/>
-      <c r="F21" s="443" t="inlineStr">
-        <is>
-          <t>DaF - Caro-SGa-EFr
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="F21" s="443" t="n"/>
       <c r="G21" s="11" t="n"/>
-      <c r="H21" s="444" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-4º e 5º tempos</t>
-        </is>
-      </c>
-      <c r="I21" s="436" t="inlineStr">
-        <is>
-          <t>GL - Caro-EFr-Eth
-5º tempo</t>
-        </is>
-      </c>
+      <c r="H21" s="444" t="n"/>
+      <c r="I21" s="436" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
           <t>2CH 9,10,11,12</t>
@@ -9422,10 +9430,7 @@
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="222" t="n"/>
-      <c r="F22" s="437" t="n"/>
       <c r="G22" s="222" t="n"/>
-      <c r="H22" s="437" t="n"/>
-      <c r="I22" s="437" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
       <c r="M22" s="18" t="n"/>
@@ -9437,10 +9442,7 @@
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="222" t="n"/>
-      <c r="F23" s="439" t="n"/>
       <c r="G23" s="222" t="n"/>
-      <c r="H23" s="439" t="n"/>
-      <c r="I23" s="439" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -9783,13 +9785,13 @@
         <f>B36+4</f>
         <v/>
       </c>
-      <c r="E36" s="283" t="n"/>
-      <c r="F36" s="434" t="inlineStr">
-        <is>
-          <t>Hist - JuLa
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="E36" s="470" t="inlineStr">
+        <is>
+          <t>Redação - Raf
+1º e 2º tempos</t>
+        </is>
+      </c>
+      <c r="F36" s="434" t="n"/>
       <c r="G36" s="462" t="inlineStr">
         <is>
           <t>Port - Jana
@@ -9815,8 +9817,7 @@
       <c r="B37" s="313" t="n"/>
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
-      <c r="E37" s="283" t="n"/>
-      <c r="F37" s="437" t="n"/>
+      <c r="E37" s="437" t="n"/>
       <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="I37" s="438" t="n"/>
@@ -9837,8 +9838,7 @@
       <c r="B38" s="313" t="n"/>
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
-      <c r="E38" s="283" t="n"/>
-      <c r="F38" s="439" t="n"/>
+      <c r="E38" s="439" t="n"/>
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="438" t="n"/>
@@ -9863,7 +9863,12 @@
         <v/>
       </c>
       <c r="E39" s="435" t="n"/>
-      <c r="F39" s="283" t="n"/>
+      <c r="F39" s="443" t="inlineStr">
+        <is>
+          <t>DaF - Caro-SGa-EFr
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="G39" s="442" t="inlineStr">
         <is>
           <t>Geo - Mar
@@ -9871,10 +9876,10 @@
         </is>
       </c>
       <c r="H39" s="283" t="n"/>
-      <c r="I39" s="451" t="inlineStr">
-        <is>
-          <t>Qui - Fab
-7º tempo</t>
+      <c r="I39" s="436" t="inlineStr">
+        <is>
+          <t>GL - Caro-EFr-Eth
+5º tempo</t>
         </is>
       </c>
       <c r="J39" s="265" t="n"/>
@@ -9885,7 +9890,7 @@
       <c r="C40" s="313" t="n"/>
       <c r="D40" s="350" t="n"/>
       <c r="E40" s="438" t="n"/>
-      <c r="F40" s="283" t="n"/>
+      <c r="F40" s="437" t="n"/>
       <c r="G40" s="437" t="n"/>
       <c r="H40" s="283" t="n"/>
       <c r="I40" s="437" t="n"/>
@@ -9897,7 +9902,7 @@
       <c r="C41" s="313" t="n"/>
       <c r="D41" s="350" t="n"/>
       <c r="E41" s="438" t="n"/>
-      <c r="F41" s="283" t="n"/>
+      <c r="F41" s="439" t="n"/>
       <c r="G41" s="439" t="n"/>
       <c r="H41" s="283" t="n"/>
       <c r="I41" s="439" t="n"/>
@@ -9989,25 +9994,15 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="449" t="inlineStr">
-        <is>
-          <t>Bio - Ale
-1º tempo</t>
+      <c r="F45" s="470" t="inlineStr">
+        <is>
+          <t>Hist - JuLa
+4º e 5º tempos</t>
         </is>
       </c>
       <c r="G45" s="283" t="n"/>
-      <c r="H45" s="443" t="inlineStr">
-        <is>
-          <t>DaF - Caro-SGa-EFr
-1º e 2º tempos</t>
-        </is>
-      </c>
-      <c r="I45" s="467" t="inlineStr">
-        <is>
-          <t>GL - Caro-EFr-Eth
-5º tempo</t>
-        </is>
-      </c>
+      <c r="H45" s="443" t="n"/>
+      <c r="I45" s="467" t="n"/>
       <c r="J45" s="269" t="n"/>
       <c r="L45" s="331" t="n"/>
     </row>
@@ -10019,8 +10014,6 @@
       <c r="E46" s="283" t="n"/>
       <c r="F46" s="437" t="n"/>
       <c r="G46" s="283" t="n"/>
-      <c r="H46" s="437" t="n"/>
-      <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
     </row>
@@ -10032,8 +10025,6 @@
       <c r="E47" s="283" t="n"/>
       <c r="F47" s="439" t="n"/>
       <c r="G47" s="283" t="n"/>
-      <c r="H47" s="439" t="n"/>
-      <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
     </row>
@@ -10055,13 +10046,13 @@
         <f>B48+4</f>
         <v/>
       </c>
-      <c r="E48" s="444" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-6º e 7º tempos</t>
-        </is>
-      </c>
-      <c r="F48" s="402" t="n"/>
+      <c r="E48" s="444" t="n"/>
+      <c r="F48" s="469" t="inlineStr">
+        <is>
+          <t>Bio - Ale
+1º tempo</t>
+        </is>
+      </c>
       <c r="G48" s="283" t="n"/>
       <c r="H48" s="435" t="n"/>
       <c r="I48" s="183" t="inlineStr">
@@ -10076,7 +10067,6 @@
       <c r="B49" s="313" t="n"/>
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
-      <c r="E49" s="437" t="n"/>
       <c r="F49" s="351" t="n"/>
       <c r="G49" s="283" t="n"/>
       <c r="H49" s="438" t="n"/>
@@ -10088,7 +10078,6 @@
       <c r="B50" s="313" t="n"/>
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
-      <c r="E50" s="439" t="n"/>
       <c r="F50" s="387" t="n"/>
       <c r="G50" s="283" t="n"/>
       <c r="H50" s="438" t="n"/>
@@ -10302,7 +10291,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="165">
+  <mergeCells count="161">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -10317,6 +10306,7 @@
     <mergeCell ref="F9:F11"/>
     <mergeCell ref="D39:D41"/>
     <mergeCell ref="D30:D32"/>
+    <mergeCell ref="F39:F41"/>
     <mergeCell ref="A15:A17"/>
     <mergeCell ref="A24:A26"/>
     <mergeCell ref="C24:C26"/>
@@ -10333,9 +10323,7 @@
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
-    <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -10345,6 +10333,7 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
+    <mergeCell ref="E36:E38"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
@@ -10364,7 +10353,6 @@
     <mergeCell ref="D6:D8"/>
     <mergeCell ref="J57:J59"/>
     <mergeCell ref="C54:C56"/>
-    <mergeCell ref="E48:E50"/>
     <mergeCell ref="C15:C17"/>
     <mergeCell ref="A51:A53"/>
     <mergeCell ref="G57:G59"/>
@@ -10374,7 +10362,6 @@
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="H45:H47"/>
     <mergeCell ref="J30:J32"/>
     <mergeCell ref="B48:B50"/>
     <mergeCell ref="D48:D50"/>
@@ -10412,7 +10399,6 @@
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="D36:D38"/>
     <mergeCell ref="M26:N26"/>
-    <mergeCell ref="F36:F38"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="F18:F20"/>
@@ -10438,6 +10424,7 @@
     <mergeCell ref="E54:E56"/>
     <mergeCell ref="I60:I62"/>
     <mergeCell ref="B54:B56"/>
+    <mergeCell ref="H12:H14"/>
     <mergeCell ref="D54:D56"/>
     <mergeCell ref="F48:F50"/>
     <mergeCell ref="J12:J14"/>
@@ -10456,14 +10443,12 @@
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
-    <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>
     <mergeCell ref="M28:N28"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="B60:B62"/>
     <mergeCell ref="B9:B11"/>
-    <mergeCell ref="I21:I23"/>
     <mergeCell ref="F33:F35"/>
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="J27:J29"/>
@@ -10855,7 +10840,12 @@
         </is>
       </c>
       <c r="G12" s="435" t="n"/>
-      <c r="H12" s="11" t="n"/>
+      <c r="H12" s="470" t="inlineStr">
+        <is>
+          <t>Redação - Raf
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I12" s="436" t="n"/>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
@@ -10871,7 +10861,7 @@
       <c r="E13" s="222" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="438" t="n"/>
-      <c r="H13" s="222" t="n"/>
+      <c r="H13" s="437" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
@@ -10886,7 +10876,7 @@
       <c r="E14" s="222" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="438" t="n"/>
-      <c r="H14" s="222" t="n"/>
+      <c r="H14" s="439" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
@@ -11061,25 +11051,10 @@
         <v/>
       </c>
       <c r="E21" s="11" t="n"/>
-      <c r="F21" s="443" t="inlineStr">
-        <is>
-          <t>DaF - Caro-SGa-EFr
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="F21" s="443" t="n"/>
       <c r="G21" s="11" t="n"/>
-      <c r="H21" s="444" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-4º e 5º tempos</t>
-        </is>
-      </c>
-      <c r="I21" s="405" t="inlineStr">
-        <is>
-          <t>GL - Caro-EFr-Eth
-5º tempo</t>
-        </is>
-      </c>
+      <c r="H21" s="444" t="n"/>
+      <c r="I21" s="436" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
           <t>2CH 9,10,11,12</t>
@@ -11103,10 +11078,7 @@
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="222" t="n"/>
-      <c r="F22" s="437" t="n"/>
       <c r="G22" s="222" t="n"/>
-      <c r="H22" s="437" t="n"/>
-      <c r="I22" s="406" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
       <c r="M22" s="18" t="n"/>
@@ -11118,10 +11090,7 @@
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="222" t="n"/>
-      <c r="F23" s="439" t="n"/>
       <c r="G23" s="222" t="n"/>
-      <c r="H23" s="439" t="n"/>
-      <c r="I23" s="407" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -11464,13 +11433,13 @@
         <f>B36+4</f>
         <v/>
       </c>
-      <c r="E36" s="283" t="n"/>
-      <c r="F36" s="434" t="inlineStr">
-        <is>
-          <t>Hist - JuLa
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="E36" s="470" t="inlineStr">
+        <is>
+          <t>Redação - Raf
+1º e 2º tempos</t>
+        </is>
+      </c>
+      <c r="F36" s="434" t="n"/>
       <c r="G36" s="462" t="inlineStr">
         <is>
           <t>Port - Jana
@@ -11496,8 +11465,7 @@
       <c r="B37" s="313" t="n"/>
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
-      <c r="E37" s="283" t="n"/>
-      <c r="F37" s="437" t="n"/>
+      <c r="E37" s="437" t="n"/>
       <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="I37" s="438" t="n"/>
@@ -11518,8 +11486,7 @@
       <c r="B38" s="313" t="n"/>
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
-      <c r="E38" s="283" t="n"/>
-      <c r="F38" s="439" t="n"/>
+      <c r="E38" s="439" t="n"/>
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="438" t="n"/>
@@ -11544,7 +11511,12 @@
         <v/>
       </c>
       <c r="E39" s="435" t="n"/>
-      <c r="F39" s="283" t="n"/>
+      <c r="F39" s="443" t="inlineStr">
+        <is>
+          <t>DaF - Caro-SGa-EFr
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="G39" s="442" t="inlineStr">
         <is>
           <t>Geo - Mar
@@ -11552,10 +11524,10 @@
         </is>
       </c>
       <c r="H39" s="283" t="n"/>
-      <c r="I39" s="451" t="inlineStr">
-        <is>
-          <t>Qui - Fab
-7º tempo</t>
+      <c r="I39" s="436" t="inlineStr">
+        <is>
+          <t>GL - Caro-EFr-Eth
+5º tempo</t>
         </is>
       </c>
       <c r="J39" s="265" t="n"/>
@@ -11566,7 +11538,7 @@
       <c r="C40" s="313" t="n"/>
       <c r="D40" s="350" t="n"/>
       <c r="E40" s="438" t="n"/>
-      <c r="F40" s="283" t="n"/>
+      <c r="F40" s="437" t="n"/>
       <c r="G40" s="437" t="n"/>
       <c r="H40" s="283" t="n"/>
       <c r="I40" s="437" t="n"/>
@@ -11578,7 +11550,7 @@
       <c r="C41" s="313" t="n"/>
       <c r="D41" s="350" t="n"/>
       <c r="E41" s="438" t="n"/>
-      <c r="F41" s="283" t="n"/>
+      <c r="F41" s="439" t="n"/>
       <c r="G41" s="439" t="n"/>
       <c r="H41" s="283" t="n"/>
       <c r="I41" s="439" t="n"/>
@@ -11670,25 +11642,15 @@
         <v/>
       </c>
       <c r="E45" s="283" t="n"/>
-      <c r="F45" s="449" t="inlineStr">
-        <is>
-          <t>Bio - Ale
-1º tempo</t>
+      <c r="F45" s="470" t="inlineStr">
+        <is>
+          <t>Hist - JuLa
+4º e 5º tempos</t>
         </is>
       </c>
       <c r="G45" s="283" t="n"/>
-      <c r="H45" s="443" t="inlineStr">
-        <is>
-          <t>DaF - Caro-SGa-EFr
-1º e 2º tempos</t>
-        </is>
-      </c>
-      <c r="I45" s="467" t="inlineStr">
-        <is>
-          <t>GL - Caro-EFr-Eth
-5º tempo</t>
-        </is>
-      </c>
+      <c r="H45" s="443" t="n"/>
+      <c r="I45" s="467" t="n"/>
       <c r="J45" s="269" t="n"/>
       <c r="L45" s="331" t="n"/>
     </row>
@@ -11700,8 +11662,6 @@
       <c r="E46" s="283" t="n"/>
       <c r="F46" s="437" t="n"/>
       <c r="G46" s="283" t="n"/>
-      <c r="H46" s="437" t="n"/>
-      <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
     </row>
@@ -11713,8 +11673,6 @@
       <c r="E47" s="283" t="n"/>
       <c r="F47" s="439" t="n"/>
       <c r="G47" s="283" t="n"/>
-      <c r="H47" s="439" t="n"/>
-      <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
     </row>
@@ -11736,13 +11694,13 @@
         <f>B48+4</f>
         <v/>
       </c>
-      <c r="E48" s="444" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-6º e 7º tempos</t>
-        </is>
-      </c>
-      <c r="F48" s="402" t="n"/>
+      <c r="E48" s="444" t="n"/>
+      <c r="F48" s="469" t="inlineStr">
+        <is>
+          <t>Bio - Ale
+1º tempo</t>
+        </is>
+      </c>
       <c r="G48" s="283" t="n"/>
       <c r="H48" s="435" t="n"/>
       <c r="I48" s="183" t="inlineStr">
@@ -11757,7 +11715,6 @@
       <c r="B49" s="313" t="n"/>
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
-      <c r="E49" s="437" t="n"/>
       <c r="F49" s="351" t="n"/>
       <c r="G49" s="283" t="n"/>
       <c r="H49" s="438" t="n"/>
@@ -11769,7 +11726,6 @@
       <c r="B50" s="313" t="n"/>
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
-      <c r="E50" s="439" t="n"/>
       <c r="F50" s="387" t="n"/>
       <c r="G50" s="283" t="n"/>
       <c r="H50" s="438" t="n"/>
@@ -11983,7 +11939,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="165">
+  <mergeCells count="161">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -11998,6 +11954,7 @@
     <mergeCell ref="F9:F11"/>
     <mergeCell ref="D39:D41"/>
     <mergeCell ref="D30:D32"/>
+    <mergeCell ref="F39:F41"/>
     <mergeCell ref="A15:A17"/>
     <mergeCell ref="A24:A26"/>
     <mergeCell ref="C24:C26"/>
@@ -12014,9 +11971,7 @@
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
-    <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -12026,6 +11981,7 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
+    <mergeCell ref="E36:E38"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
@@ -12045,7 +12001,6 @@
     <mergeCell ref="D6:D8"/>
     <mergeCell ref="J57:J59"/>
     <mergeCell ref="C54:C56"/>
-    <mergeCell ref="E48:E50"/>
     <mergeCell ref="C15:C17"/>
     <mergeCell ref="A51:A53"/>
     <mergeCell ref="G57:G59"/>
@@ -12055,7 +12010,6 @@
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="H45:H47"/>
     <mergeCell ref="J30:J32"/>
     <mergeCell ref="B48:B50"/>
     <mergeCell ref="D48:D50"/>
@@ -12093,7 +12047,6 @@
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="D36:D38"/>
     <mergeCell ref="M26:N26"/>
-    <mergeCell ref="F36:F38"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="F18:F20"/>
@@ -12119,6 +12072,7 @@
     <mergeCell ref="E54:E56"/>
     <mergeCell ref="I60:I62"/>
     <mergeCell ref="B54:B56"/>
+    <mergeCell ref="H12:H14"/>
     <mergeCell ref="D54:D56"/>
     <mergeCell ref="F48:F50"/>
     <mergeCell ref="J12:J14"/>
@@ -12137,14 +12091,12 @@
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
-    <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>
     <mergeCell ref="M28:N28"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="B60:B62"/>
     <mergeCell ref="B9:B11"/>
-    <mergeCell ref="I21:I23"/>
     <mergeCell ref="F33:F35"/>
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="J27:J29"/>

</xml_diff>

<commit_message>
9C: Redação (2ª prova) movida de 19/10 para 22/10 (4º e 5º tempos)
- Semana 12, segunda-feira (19/10) -> semana 12, quinta-feira (22/10)
- Tempos ajustados de 1º-2º para 4º-5º
- Aplicado em 9C1 e 9C2

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -9785,12 +9785,7 @@
         <f>B36+4</f>
         <v/>
       </c>
-      <c r="E36" s="470" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="E36" s="470" t="n"/>
       <c r="F36" s="434" t="n"/>
       <c r="G36" s="462" t="inlineStr">
         <is>
@@ -9798,7 +9793,12 @@
 4º e 5º tempos</t>
         </is>
       </c>
-      <c r="H36" s="283" t="n"/>
+      <c r="H36" s="444" t="inlineStr">
+        <is>
+          <t>Redação - Raf
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I36" s="435" t="n"/>
       <c r="J36" s="265" t="n"/>
       <c r="L36" s="81" t="inlineStr">
@@ -9817,9 +9817,8 @@
       <c r="B37" s="313" t="n"/>
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
-      <c r="E37" s="437" t="n"/>
       <c r="G37" s="437" t="n"/>
-      <c r="H37" s="283" t="n"/>
+      <c r="H37" s="437" t="n"/>
       <c r="I37" s="438" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
@@ -9838,9 +9837,8 @@
       <c r="B38" s="313" t="n"/>
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
-      <c r="E38" s="439" t="n"/>
       <c r="G38" s="439" t="n"/>
-      <c r="H38" s="283" t="n"/>
+      <c r="H38" s="439" t="n"/>
       <c r="I38" s="438" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
@@ -10333,7 +10331,6 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
-    <mergeCell ref="E36:E38"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
@@ -10405,6 +10402,7 @@
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
+    <mergeCell ref="H36:H38"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
@@ -11433,12 +11431,7 @@
         <f>B36+4</f>
         <v/>
       </c>
-      <c r="E36" s="470" t="inlineStr">
-        <is>
-          <t>Redação - Raf
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="E36" s="470" t="n"/>
       <c r="F36" s="434" t="n"/>
       <c r="G36" s="462" t="inlineStr">
         <is>
@@ -11446,7 +11439,12 @@
 4º e 5º tempos</t>
         </is>
       </c>
-      <c r="H36" s="283" t="n"/>
+      <c r="H36" s="412" t="inlineStr">
+        <is>
+          <t>Redação - Raf
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I36" s="435" t="n"/>
       <c r="J36" s="265" t="n"/>
       <c r="L36" s="81" t="inlineStr">
@@ -11465,9 +11463,8 @@
       <c r="B37" s="313" t="n"/>
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
-      <c r="E37" s="437" t="n"/>
       <c r="G37" s="437" t="n"/>
-      <c r="H37" s="283" t="n"/>
+      <c r="H37" s="406" t="n"/>
       <c r="I37" s="438" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
@@ -11486,9 +11483,8 @@
       <c r="B38" s="313" t="n"/>
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
-      <c r="E38" s="439" t="n"/>
       <c r="G38" s="439" t="n"/>
-      <c r="H38" s="283" t="n"/>
+      <c r="H38" s="407" t="n"/>
       <c r="I38" s="438" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
@@ -11981,7 +11977,6 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
-    <mergeCell ref="E36:E38"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
@@ -12053,6 +12048,7 @@
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
+    <mergeCell ref="H36:H38"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>

</xml_diff>

<commit_message>
12C: Geografia (2ª prova) reposicionada de 23/10 para 09/11
- 13/11 descartado: dia já reservado com marcação fixa '2CH 10,12'
  (2ª chamada); mesmo se livre, ficaria a só 4 dias do CC 10,12,
  violando o mínimo de 6 dias exigido para turmas 10C/12C.
- 09/11 (semana 15, segunda) escolhido: aula dupla real do prof. Mar
  em 12C1 às segundas, 5º-6º tempos, ainda no período da manhã, sem
  cessão de tempo de nenhuma disciplina; 12C2 coberta por coordenação
  entre turmas irmãs.

Avaliação apresentada e aprovada pelo usuário antes da execução.

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6618,12 +6618,7 @@
         </is>
       </c>
       <c r="H36" s="283" t="n"/>
-      <c r="I36" s="442" t="inlineStr">
-        <is>
-          <t>Geo - Mar
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="I36" s="442" t="n"/>
       <c r="J36" s="265" t="n"/>
       <c r="L36" s="81" t="inlineStr">
         <is>
@@ -6645,7 +6640,6 @@
       <c r="F37" s="437" t="n"/>
       <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
-      <c r="I37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
@@ -6667,7 +6661,6 @@
       <c r="F38" s="439" t="n"/>
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
-      <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
@@ -6819,7 +6812,12 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="283" t="n"/>
+      <c r="E45" s="410" t="inlineStr">
+        <is>
+          <t>Geo - Mar
+5º e 6º tempos</t>
+        </is>
+      </c>
       <c r="F45" s="441" t="inlineStr">
         <is>
           <t>Mat - Bre/JJ
@@ -6842,7 +6840,7 @@
       <c r="B46" s="313" t="n"/>
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
-      <c r="E46" s="283" t="n"/>
+      <c r="E46" s="406" t="n"/>
       <c r="F46" s="437" t="n"/>
       <c r="G46" s="438" t="n"/>
       <c r="H46" s="283" t="n"/>
@@ -6855,7 +6853,7 @@
       <c r="B47" s="313" t="n"/>
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
-      <c r="E47" s="283" t="n"/>
+      <c r="E47" s="407" t="n"/>
       <c r="F47" s="439" t="n"/>
       <c r="G47" s="438" t="n"/>
       <c r="H47" s="283" t="n"/>
@@ -7161,6 +7159,7 @@
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
     <mergeCell ref="A12:A14"/>
+    <mergeCell ref="E45:E47"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
     <mergeCell ref="I39:I41"/>
@@ -7274,7 +7273,6 @@
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
-    <mergeCell ref="I36:I38"/>
     <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
@@ -10952,7 +10950,7 @@
         </is>
       </c>
       <c r="G15" s="462" t="n"/>
-      <c r="H15" s="412" t="inlineStr">
+      <c r="H15" s="444" t="inlineStr">
         <is>
           <t>Redação - Raf
 4º e 5º tempos</t>
@@ -10976,7 +10974,7 @@
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
       <c r="F16" s="437" t="n"/>
-      <c r="H16" s="406" t="n"/>
+      <c r="H16" s="437" t="n"/>
       <c r="I16" s="437" t="n"/>
       <c r="J16" s="315" t="n"/>
       <c r="L16" s="141" t="n"/>
@@ -10991,7 +10989,7 @@
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
       <c r="F17" s="439" t="n"/>
-      <c r="H17" s="407" t="n"/>
+      <c r="H17" s="439" t="n"/>
       <c r="I17" s="439" t="n"/>
       <c r="J17" s="315" t="n"/>
       <c r="L17" s="317" t="n"/>
@@ -11021,7 +11019,7 @@
           <t>unterrichtsfrei sem aula</t>
         </is>
       </c>
-      <c r="F18" s="404" t="inlineStr">
+      <c r="F18" s="462" t="inlineStr">
         <is>
           <t>Port - Jana
 1º e 2º tempos</t>
@@ -11046,7 +11044,7 @@
       <c r="C19" s="313" t="n"/>
       <c r="D19" s="314" t="n"/>
       <c r="E19" s="315" t="n"/>
-      <c r="F19" s="406" t="n"/>
+      <c r="F19" s="437" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="222" t="n"/>
       <c r="I19" s="383" t="n"/>
@@ -11069,7 +11067,7 @@
       <c r="C20" s="313" t="n"/>
       <c r="D20" s="314" t="n"/>
       <c r="E20" s="315" t="n"/>
-      <c r="F20" s="407" t="n"/>
+      <c r="F20" s="439" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="222" t="n"/>
       <c r="I20" s="384" t="n"/>
@@ -11103,7 +11101,7 @@
 1º e 2º tempos</t>
         </is>
       </c>
-      <c r="G21" s="409" t="inlineStr">
+      <c r="G21" s="441" t="inlineStr">
         <is>
           <t>Mat - BrSa
 4º e 5º tempos</t>
@@ -11135,7 +11133,7 @@
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="222" t="n"/>
       <c r="F22" s="437" t="n"/>
-      <c r="G22" s="406" t="n"/>
+      <c r="G22" s="437" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
       <c r="M22" s="18" t="n"/>
@@ -11148,7 +11146,7 @@
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="222" t="n"/>
       <c r="F23" s="439" t="n"/>
-      <c r="G23" s="407" t="n"/>
+      <c r="G23" s="439" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="19" t="n"/>
@@ -20055,12 +20053,7 @@
         </is>
       </c>
       <c r="H36" s="283" t="n"/>
-      <c r="I36" s="442" t="inlineStr">
-        <is>
-          <t>Geo - Mar
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="I36" s="442" t="n"/>
       <c r="J36" s="265" t="n"/>
       <c r="L36" s="81" t="inlineStr">
         <is>
@@ -20082,7 +20075,6 @@
       <c r="F37" s="437" t="n"/>
       <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
-      <c r="I37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
@@ -20104,7 +20096,6 @@
       <c r="F38" s="439" t="n"/>
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
-      <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
@@ -20256,7 +20247,12 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="283" t="n"/>
+      <c r="E45" s="442" t="inlineStr">
+        <is>
+          <t>Geo - Mar
+5º e 6º tempos</t>
+        </is>
+      </c>
       <c r="F45" s="441" t="inlineStr">
         <is>
           <t>Mat - Bre/JJ
@@ -20279,7 +20275,7 @@
       <c r="B46" s="313" t="n"/>
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
-      <c r="E46" s="283" t="n"/>
+      <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
       <c r="G46" s="438" t="n"/>
       <c r="H46" s="283" t="n"/>
@@ -20292,7 +20288,7 @@
       <c r="B47" s="313" t="n"/>
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
-      <c r="E47" s="283" t="n"/>
+      <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
       <c r="G47" s="438" t="n"/>
       <c r="H47" s="283" t="n"/>
@@ -20598,6 +20594,7 @@
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
     <mergeCell ref="A12:A14"/>
+    <mergeCell ref="E45:E47"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
     <mergeCell ref="I39:I41"/>
@@ -20711,7 +20708,6 @@
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
-    <mergeCell ref="I36:I38"/>
     <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>

</xml_diff>

<commit_message>
10C1 (apenas): Inglês reposicionado - 02/09 -> 03/09, 19/10 -> 05/11
- 1ª prova: semana 5 quarta (02/09) -> semana 5 quinta (03/09), 2º-3º
  tempos - aula dupla real do prof. APa em 10C1 às quintas, sem cessão
  de tempo de nenhuma disciplina
- 2ª prova: semana 12 segunda (19/10) -> semana 14 quinta (05/11),
  mesmo bloco 2º-3º tempos - mesma aula dupla real

04/09 (sexta) testado e rejeitado antes: APa não dá nenhuma aula de
Inglês na sexta em 10C1 (sem cobertura por turma irmã, já que o
Inglês de 10C2 é com outra professora). Usuário corrigiu para 03/09.

Mudança feita apenas em 10C1 (10C2 não foi tocada).

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6812,7 +6812,7 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="410" t="inlineStr">
+      <c r="E45" s="442" t="inlineStr">
         <is>
           <t>Geo - Mar
 5º e 6º tempos</t>
@@ -6840,7 +6840,7 @@
       <c r="B46" s="313" t="n"/>
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
-      <c r="E46" s="406" t="n"/>
+      <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
       <c r="G46" s="438" t="n"/>
       <c r="H46" s="283" t="n"/>
@@ -6853,7 +6853,7 @@
       <c r="B47" s="313" t="n"/>
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
-      <c r="E47" s="407" t="n"/>
+      <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
       <c r="G47" s="438" t="n"/>
       <c r="H47" s="283" t="n"/>
@@ -12618,13 +12618,13 @@
         </is>
       </c>
       <c r="F15" s="11" t="n"/>
-      <c r="G15" s="453" t="inlineStr">
+      <c r="G15" s="453" t="n"/>
+      <c r="H15" s="408" t="inlineStr">
         <is>
           <t>Ing - APa
-3º e 4º tempos</t>
-        </is>
-      </c>
-      <c r="H15" s="435" t="n"/>
+2º e 3º tempos</t>
+        </is>
+      </c>
       <c r="I15" s="11" t="n"/>
       <c r="J15" s="183" t="n"/>
       <c r="L15" s="17" t="n"/>
@@ -12638,8 +12638,7 @@
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
       <c r="F16" s="222" t="n"/>
-      <c r="G16" s="437" t="n"/>
-      <c r="H16" s="438" t="n"/>
+      <c r="H16" s="406" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
       <c r="L16" s="141" t="n"/>
@@ -12654,8 +12653,7 @@
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
       <c r="F17" s="222" t="n"/>
-      <c r="G17" s="439" t="n"/>
-      <c r="H17" s="438" t="n"/>
+      <c r="H17" s="407" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
       <c r="L17" s="317" t="n"/>
@@ -13171,12 +13169,7 @@
         <f>B36+4</f>
         <v/>
       </c>
-      <c r="E36" s="440" t="inlineStr">
-        <is>
-          <t>Ing - APa
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="E36" s="440" t="n"/>
       <c r="F36" s="283" t="n"/>
       <c r="G36" s="436" t="inlineStr">
         <is>
@@ -13208,7 +13201,6 @@
       <c r="B37" s="313" t="n"/>
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
-      <c r="E37" s="437" t="n"/>
       <c r="F37" s="283" t="n"/>
       <c r="G37" s="437" t="n"/>
       <c r="H37" s="437" t="n"/>
@@ -13230,7 +13222,6 @@
       <c r="B38" s="313" t="n"/>
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
-      <c r="E38" s="439" t="n"/>
       <c r="F38" s="283" t="n"/>
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="439" t="n"/>
@@ -13332,7 +13323,12 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="H42" s="283" t="n"/>
+      <c r="H42" s="408" t="inlineStr">
+        <is>
+          <t>Ing - APa
+2º e 3º tempos</t>
+        </is>
+      </c>
       <c r="I42" s="283" t="n"/>
       <c r="J42" s="265" t="n"/>
       <c r="L42" s="259" t="inlineStr">
@@ -13350,7 +13346,7 @@
       <c r="E43" s="283" t="n"/>
       <c r="F43" s="437" t="n"/>
       <c r="G43" s="437" t="n"/>
-      <c r="H43" s="283" t="n"/>
+      <c r="H43" s="406" t="n"/>
       <c r="I43" s="283" t="n"/>
       <c r="J43" s="352" t="n"/>
       <c r="L43" s="331" t="n"/>
@@ -13363,7 +13359,7 @@
       <c r="E44" s="283" t="n"/>
       <c r="F44" s="439" t="n"/>
       <c r="G44" s="439" t="n"/>
-      <c r="H44" s="283" t="n"/>
+      <c r="H44" s="407" t="n"/>
       <c r="I44" s="283" t="n"/>
       <c r="J44" s="352" t="n"/>
       <c r="L44" s="331" t="n"/>
@@ -13732,7 +13728,6 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
-    <mergeCell ref="E36:E38"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="E45:E47"/>
     <mergeCell ref="L24:N24"/>
@@ -13746,6 +13741,7 @@
     <mergeCell ref="H33:H35"/>
     <mergeCell ref="E12:E14"/>
     <mergeCell ref="J33:J35"/>
+    <mergeCell ref="H42:H44"/>
     <mergeCell ref="J42:J44"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="J60:J62"/>
@@ -13784,6 +13780,7 @@
     <mergeCell ref="J48:J50"/>
     <mergeCell ref="D51:D53"/>
     <mergeCell ref="C3:C5"/>
+    <mergeCell ref="H15:H17"/>
     <mergeCell ref="D60:D62"/>
     <mergeCell ref="F60:F62"/>
     <mergeCell ref="M31:N31"/>
@@ -13810,7 +13807,6 @@
     <mergeCell ref="H36:H38"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
-    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>

</xml_diff>

<commit_message>
11C1/11C2: História reposicionada de quarta para terça (01/09, 03/11)
- 1ª prova: semana 5 quarta (02/09) -> semana 5 terça (01/09), 2º-3º
  tempos
- 2ª prova: semana 12 quarta (21/10) -> semana 14 terça (03/11), 2º-3º
  tempos

Terça 2º-3º tempos é a aula dupla real do prof. Ver em 11C1 (11C2
coberta por coordenação entre turmas irmãs) — elimina a cessão de
tempo que a posição anterior (quarta, 1º-2º tempos) exigia em ambas
as turmas.

Verificado com professor_presente_no_bloco() e aprovado pelo usuário
antes da execução.

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -12619,7 +12619,7 @@
       </c>
       <c r="F15" s="11" t="n"/>
       <c r="G15" s="453" t="n"/>
-      <c r="H15" s="408" t="inlineStr">
+      <c r="H15" s="440" t="inlineStr">
         <is>
           <t>Ing - APa
 2º e 3º tempos</t>
@@ -12638,7 +12638,7 @@
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
       <c r="F16" s="222" t="n"/>
-      <c r="H16" s="406" t="n"/>
+      <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
       <c r="L16" s="141" t="n"/>
@@ -12653,7 +12653,7 @@
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
       <c r="F17" s="222" t="n"/>
-      <c r="H17" s="407" t="n"/>
+      <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
       <c r="L17" s="317" t="n"/>
@@ -13323,7 +13323,7 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="H42" s="408" t="inlineStr">
+      <c r="H42" s="440" t="inlineStr">
         <is>
           <t>Ing - APa
 2º e 3º tempos</t>
@@ -13346,7 +13346,7 @@
       <c r="E43" s="283" t="n"/>
       <c r="F43" s="437" t="n"/>
       <c r="G43" s="437" t="n"/>
-      <c r="H43" s="406" t="n"/>
+      <c r="H43" s="437" t="n"/>
       <c r="I43" s="283" t="n"/>
       <c r="J43" s="352" t="n"/>
       <c r="L43" s="331" t="n"/>
@@ -13359,7 +13359,7 @@
       <c r="E44" s="283" t="n"/>
       <c r="F44" s="439" t="n"/>
       <c r="G44" s="439" t="n"/>
-      <c r="H44" s="407" t="n"/>
+      <c r="H44" s="439" t="n"/>
       <c r="I44" s="283" t="n"/>
       <c r="J44" s="352" t="n"/>
       <c r="L44" s="331" t="n"/>
@@ -16032,13 +16032,13 @@
         <v/>
       </c>
       <c r="E15" s="435" t="n"/>
-      <c r="F15" s="435" t="n"/>
-      <c r="G15" s="434" t="inlineStr">
+      <c r="F15" s="434" t="inlineStr">
         <is>
           <t>Hist - Ver
-1º e 2º tempos</t>
-        </is>
-      </c>
+2º e 3º tempos</t>
+        </is>
+      </c>
+      <c r="G15" s="434" t="n"/>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -16057,8 +16057,7 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="438" t="n"/>
-      <c r="F16" s="438" t="n"/>
-      <c r="G16" s="437" t="n"/>
+      <c r="F16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -16073,8 +16072,7 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="438" t="n"/>
-      <c r="F17" s="438" t="n"/>
-      <c r="G17" s="439" t="n"/>
+      <c r="F17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -16598,12 +16596,7 @@
       </c>
       <c r="E36" s="283" t="n"/>
       <c r="F36" s="435" t="n"/>
-      <c r="G36" s="434" t="inlineStr">
-        <is>
-          <t>Hist - Ver
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="G36" s="434" t="n"/>
       <c r="H36" s="283" t="n"/>
       <c r="I36" s="435" t="n"/>
       <c r="J36" s="265" t="n"/>
@@ -16625,7 +16618,6 @@
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="438" t="n"/>
-      <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="I37" s="438" t="n"/>
       <c r="J37" s="352" t="n"/>
@@ -16647,7 +16639,6 @@
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="438" t="n"/>
-      <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="438" t="n"/>
       <c r="J38" s="352" t="n"/>
@@ -16735,7 +16726,12 @@
         <v/>
       </c>
       <c r="E42" s="283" t="n"/>
-      <c r="F42" s="283" t="n"/>
+      <c r="F42" s="434" t="inlineStr">
+        <is>
+          <t>Hist - Ver
+2º e 3º tempos</t>
+        </is>
+      </c>
       <c r="G42" s="435" t="n"/>
       <c r="H42" s="458" t="inlineStr">
         <is>
@@ -16758,7 +16754,7 @@
       <c r="C43" s="313" t="n"/>
       <c r="D43" s="350" t="n"/>
       <c r="E43" s="283" t="n"/>
-      <c r="F43" s="283" t="n"/>
+      <c r="F43" s="437" t="n"/>
       <c r="G43" s="438" t="n"/>
       <c r="H43" s="437" t="n"/>
       <c r="I43" s="283" t="n"/>
@@ -16771,7 +16767,7 @@
       <c r="C44" s="313" t="n"/>
       <c r="D44" s="350" t="n"/>
       <c r="E44" s="283" t="n"/>
-      <c r="F44" s="283" t="n"/>
+      <c r="F44" s="439" t="n"/>
       <c r="G44" s="438" t="n"/>
       <c r="H44" s="439" t="n"/>
       <c r="I44" s="283" t="n"/>
@@ -17148,6 +17144,7 @@
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="D21:D23"/>
     <mergeCell ref="E60:E62"/>
+    <mergeCell ref="F15:F17"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
@@ -17243,8 +17240,8 @@
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
+    <mergeCell ref="F42:F44"/>
     <mergeCell ref="J36:J38"/>
-    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
@@ -17276,7 +17273,6 @@
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
@@ -17741,13 +17737,13 @@
         <v/>
       </c>
       <c r="E15" s="435" t="n"/>
-      <c r="F15" s="435" t="n"/>
-      <c r="G15" s="434" t="inlineStr">
+      <c r="F15" s="403" t="inlineStr">
         <is>
           <t>Hist - Ver
-1º e 2º tempos</t>
-        </is>
-      </c>
+2º e 3º tempos</t>
+        </is>
+      </c>
+      <c r="G15" s="434" t="n"/>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -17766,8 +17762,7 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="438" t="n"/>
-      <c r="F16" s="438" t="n"/>
-      <c r="G16" s="437" t="n"/>
+      <c r="F16" s="406" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -17782,8 +17777,7 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="438" t="n"/>
-      <c r="F17" s="438" t="n"/>
-      <c r="G17" s="439" t="n"/>
+      <c r="F17" s="407" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -18312,12 +18306,7 @@
         </is>
       </c>
       <c r="F36" s="435" t="n"/>
-      <c r="G36" s="434" t="inlineStr">
-        <is>
-          <t>Hist - Ver
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="G36" s="434" t="n"/>
       <c r="H36" s="283" t="n"/>
       <c r="I36" s="435" t="n"/>
       <c r="J36" s="265" t="n"/>
@@ -18339,7 +18328,6 @@
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="437" t="n"/>
       <c r="F37" s="438" t="n"/>
-      <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="I37" s="438" t="n"/>
       <c r="J37" s="352" t="n"/>
@@ -18361,7 +18349,6 @@
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="439" t="n"/>
       <c r="F38" s="438" t="n"/>
-      <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="438" t="n"/>
       <c r="J38" s="352" t="n"/>
@@ -18449,7 +18436,12 @@
         <v/>
       </c>
       <c r="E42" s="283" t="n"/>
-      <c r="F42" s="283" t="n"/>
+      <c r="F42" s="403" t="inlineStr">
+        <is>
+          <t>Hist - Ver
+2º e 3º tempos</t>
+        </is>
+      </c>
       <c r="G42" s="435" t="n"/>
       <c r="H42" s="458" t="inlineStr">
         <is>
@@ -18472,7 +18464,7 @@
       <c r="C43" s="313" t="n"/>
       <c r="D43" s="350" t="n"/>
       <c r="E43" s="283" t="n"/>
-      <c r="F43" s="283" t="n"/>
+      <c r="F43" s="406" t="n"/>
       <c r="G43" s="438" t="n"/>
       <c r="H43" s="437" t="n"/>
       <c r="I43" s="283" t="n"/>
@@ -18485,7 +18477,7 @@
       <c r="C44" s="313" t="n"/>
       <c r="D44" s="350" t="n"/>
       <c r="E44" s="283" t="n"/>
-      <c r="F44" s="283" t="n"/>
+      <c r="F44" s="407" t="n"/>
       <c r="G44" s="438" t="n"/>
       <c r="H44" s="439" t="n"/>
       <c r="I44" s="283" t="n"/>
@@ -18862,6 +18854,7 @@
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="D21:D23"/>
     <mergeCell ref="E60:E62"/>
+    <mergeCell ref="F15:F17"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
@@ -18956,8 +18949,8 @@
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
+    <mergeCell ref="F42:F44"/>
     <mergeCell ref="J36:J38"/>
-    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
@@ -18989,7 +18982,6 @@
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>

</xml_diff>

<commit_message>
12C1/12C2: Química e Biologia divididas entre semanas 12 e 15
- Filosofia: semana 12 quarta (21/10) -> semana 14 quarta (04/11),
  mantendo tempo próprio de cada turma (10º em 12C1, 4º em 12C2)
- Química (2ª prova): semana 14 sexta (06/11) -> semana 12 quarta
  (21/10), 1º tempo (mesmo tempo nas duas turmas, como exige a
  coordenação normal -- Química não tem a exceção de Fil/Soc)
- Biologia (2ª prova): semana 14 terça (03/11) -> semana 15 quinta
  (12/11), 5º-6º tempos

Duas tentativas iniciais corrigidas antes de fechar: Química com
tempos diferentes por turma violava a regra de coordenação (não está
na exceção); Biologia na quarta-feira semana 15 doaria a única aula
semanal de Sociologia (disciplina de aula única não pode doar) --
movida para quinta-feira.

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6611,10 +6611,10 @@
 10º e 11º tempos</t>
         </is>
       </c>
-      <c r="G36" s="457" t="inlineStr">
-        <is>
-          <t>Fil - LAn
-4º tempo</t>
+      <c r="G36" s="419" t="inlineStr">
+        <is>
+          <t>Qui - CAl/Fab
+1º tempo</t>
         </is>
       </c>
       <c r="H36" s="283" t="n"/>
@@ -6638,7 +6638,7 @@
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="437" t="n"/>
-      <c r="G37" s="437" t="n"/>
+      <c r="G37" s="406" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
@@ -6659,7 +6659,7 @@
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="439" t="n"/>
-      <c r="G38" s="439" t="n"/>
+      <c r="G38" s="407" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
@@ -6746,20 +6746,15 @@
         <v/>
       </c>
       <c r="E42" s="283" t="n"/>
-      <c r="F42" s="449" t="inlineStr">
-        <is>
-          <t>Bio - Ale
-1º e 2º tempos</t>
-        </is>
-      </c>
-      <c r="G42" s="283" t="n"/>
+      <c r="F42" s="449" t="n"/>
+      <c r="G42" s="457" t="inlineStr">
+        <is>
+          <t>Fil - LAn
+4º tempo</t>
+        </is>
+      </c>
       <c r="H42" s="283" t="n"/>
-      <c r="I42" s="451" t="inlineStr">
-        <is>
-          <t>Qui - CAl/Fab
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="I42" s="451" t="n"/>
       <c r="J42" s="265" t="n"/>
       <c r="L42" s="259" t="inlineStr">
         <is>
@@ -6774,10 +6769,8 @@
       <c r="C43" s="313" t="n"/>
       <c r="D43" s="350" t="n"/>
       <c r="E43" s="283" t="n"/>
-      <c r="F43" s="437" t="n"/>
-      <c r="G43" s="283" t="n"/>
+      <c r="G43" s="437" t="n"/>
       <c r="H43" s="283" t="n"/>
-      <c r="I43" s="437" t="n"/>
       <c r="J43" s="352" t="n"/>
       <c r="L43" s="331" t="n"/>
     </row>
@@ -6787,10 +6780,8 @@
       <c r="C44" s="313" t="n"/>
       <c r="D44" s="350" t="n"/>
       <c r="E44" s="283" t="n"/>
-      <c r="F44" s="439" t="n"/>
-      <c r="G44" s="283" t="n"/>
+      <c r="G44" s="439" t="n"/>
       <c r="H44" s="283" t="n"/>
-      <c r="I44" s="439" t="n"/>
       <c r="J44" s="352" t="n"/>
       <c r="L44" s="331" t="n"/>
     </row>
@@ -6824,8 +6815,13 @@
 1º e 2º tempos</t>
         </is>
       </c>
-      <c r="G45" s="435" t="n"/>
-      <c r="H45" s="283" t="n"/>
+      <c r="G45" s="449" t="n"/>
+      <c r="H45" s="417" t="inlineStr">
+        <is>
+          <t>Bio - Ale
+5º e 6º tempos</t>
+        </is>
+      </c>
       <c r="I45" s="386" t="inlineStr">
         <is>
           <t>2CH
@@ -6842,8 +6838,7 @@
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
-      <c r="G46" s="438" t="n"/>
-      <c r="H46" s="283" t="n"/>
+      <c r="H46" s="406" t="n"/>
       <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
@@ -6855,8 +6850,7 @@
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
-      <c r="G47" s="438" t="n"/>
-      <c r="H47" s="283" t="n"/>
+      <c r="H47" s="407" t="n"/>
       <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
@@ -7144,6 +7138,7 @@
     <mergeCell ref="D21:D23"/>
     <mergeCell ref="E60:E62"/>
     <mergeCell ref="F15:F17"/>
+    <mergeCell ref="G42:G44"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
@@ -7189,6 +7184,7 @@
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
     <mergeCell ref="B39:B41"/>
+    <mergeCell ref="H45:H47"/>
     <mergeCell ref="J30:J32"/>
     <mergeCell ref="B48:B50"/>
     <mergeCell ref="D48:D50"/>
@@ -7201,7 +7197,6 @@
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="E9:E11"/>
     <mergeCell ref="C27:C29"/>
-    <mergeCell ref="I42:I44"/>
     <mergeCell ref="B15:B17"/>
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="D24:D26"/>
@@ -7237,7 +7232,6 @@
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="H39:H41"/>
     <mergeCell ref="M29:N29"/>
-    <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="J45:J47"/>
@@ -20022,10 +20016,10 @@
 10º e 11º tempos</t>
         </is>
       </c>
-      <c r="G36" s="457" t="inlineStr">
-        <is>
-          <t>Fil - LAn
-10º tempo</t>
+      <c r="G36" s="451" t="inlineStr">
+        <is>
+          <t>Qui - CAl/Fab
+1º tempo</t>
         </is>
       </c>
       <c r="H36" s="283" t="n"/>
@@ -20157,20 +20151,15 @@
         <v/>
       </c>
       <c r="E42" s="283" t="n"/>
-      <c r="F42" s="449" t="inlineStr">
-        <is>
-          <t>Bio - Ale
-1º e 2º tempos</t>
-        </is>
-      </c>
-      <c r="G42" s="283" t="n"/>
+      <c r="F42" s="449" t="n"/>
+      <c r="G42" s="457" t="inlineStr">
+        <is>
+          <t>Fil - LAn
+10º tempo</t>
+        </is>
+      </c>
       <c r="H42" s="435" t="n"/>
-      <c r="I42" s="451" t="inlineStr">
-        <is>
-          <t>Qui - CAl/Fab
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="I42" s="451" t="n"/>
       <c r="J42" s="265" t="n"/>
       <c r="L42" s="259" t="inlineStr">
         <is>
@@ -20185,10 +20174,8 @@
       <c r="C43" s="313" t="n"/>
       <c r="D43" s="350" t="n"/>
       <c r="E43" s="283" t="n"/>
-      <c r="F43" s="437" t="n"/>
-      <c r="G43" s="283" t="n"/>
+      <c r="G43" s="437" t="n"/>
       <c r="H43" s="438" t="n"/>
-      <c r="I43" s="437" t="n"/>
       <c r="J43" s="352" t="n"/>
       <c r="L43" s="331" t="n"/>
     </row>
@@ -20198,10 +20185,8 @@
       <c r="C44" s="313" t="n"/>
       <c r="D44" s="350" t="n"/>
       <c r="E44" s="283" t="n"/>
-      <c r="F44" s="439" t="n"/>
-      <c r="G44" s="283" t="n"/>
+      <c r="G44" s="439" t="n"/>
       <c r="H44" s="438" t="n"/>
-      <c r="I44" s="439" t="n"/>
       <c r="J44" s="352" t="n"/>
       <c r="L44" s="331" t="n"/>
     </row>
@@ -20235,8 +20220,13 @@
 1º e 2º tempos</t>
         </is>
       </c>
-      <c r="G45" s="435" t="n"/>
-      <c r="H45" s="283" t="n"/>
+      <c r="G45" s="449" t="n"/>
+      <c r="H45" s="449" t="inlineStr">
+        <is>
+          <t>Bio - Ale
+5º e 6º tempos</t>
+        </is>
+      </c>
       <c r="I45" s="386" t="inlineStr">
         <is>
           <t>2CH
@@ -20253,8 +20243,7 @@
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
-      <c r="G46" s="438" t="n"/>
-      <c r="H46" s="283" t="n"/>
+      <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
@@ -20266,8 +20255,7 @@
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
-      <c r="G47" s="438" t="n"/>
-      <c r="H47" s="283" t="n"/>
+      <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
@@ -20555,6 +20543,7 @@
     <mergeCell ref="D21:D23"/>
     <mergeCell ref="E60:E62"/>
     <mergeCell ref="F15:F17"/>
+    <mergeCell ref="G42:G44"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
@@ -20600,6 +20589,7 @@
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
     <mergeCell ref="B39:B41"/>
+    <mergeCell ref="H45:H47"/>
     <mergeCell ref="J30:J32"/>
     <mergeCell ref="B48:B50"/>
     <mergeCell ref="D48:D50"/>
@@ -20612,7 +20602,6 @@
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="E9:E11"/>
     <mergeCell ref="C27:C29"/>
-    <mergeCell ref="I42:I44"/>
     <mergeCell ref="B15:B17"/>
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="D24:D26"/>
@@ -20648,7 +20637,6 @@
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="H39:H41"/>
     <mergeCell ref="M29:N29"/>
-    <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="J45:J47"/>

</xml_diff>

<commit_message>
12C1/12C2: Geografia e DaF reposicionadas + corrige feriado faltante
- DaF (2ª prova): semana 13 sexta (30/10) -> semana 12 sexta (23/10),
  mesmo bloco 6º-7º tempos
- Geografia (2ª prova): semana 15 segunda (09/11) -> semana 13 segunda
  (26/10), mesmo bloco 5º-6º tempos

Contexto: usuário pediu para avaliar mover Geografia para semana 13 ou
14. A opção de semana 14 (02/11) sugerida caía em cima do feriado de
Finados -- usuário corrigiu antes de eu aplicar.

Bug corrigido em verificar_calendario.py: FERIADOS só tinha 07/09 e
20/11, faltava 02/11 (Finados) -- gerar_calendario.py já bloqueava
esse dia via BLOQUEIOS, mas o checklist não cruzava contra isso, só
contra o próprio FERIADOS. Se a proposta de semana 14 tivesse sido
aplicada, o checklist não teria detectado o erro.

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6611,14 +6611,19 @@
 10º e 11º tempos</t>
         </is>
       </c>
-      <c r="G36" s="419" t="inlineStr">
+      <c r="G36" s="451" t="inlineStr">
         <is>
           <t>Qui - CAl/Fab
 1º tempo</t>
         </is>
       </c>
       <c r="H36" s="283" t="n"/>
-      <c r="I36" s="442" t="n"/>
+      <c r="I36" s="411" t="inlineStr">
+        <is>
+          <t>DaF - CBu-EFr-Eth
+6º e 7º tempos</t>
+        </is>
+      </c>
       <c r="J36" s="265" t="n"/>
       <c r="L36" s="81" t="inlineStr">
         <is>
@@ -6638,8 +6643,9 @@
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="437" t="n"/>
-      <c r="G37" s="406" t="n"/>
+      <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
+      <c r="I37" s="406" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
@@ -6659,8 +6665,9 @@
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="439" t="n"/>
-      <c r="G38" s="407" t="n"/>
+      <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
+      <c r="I38" s="407" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
@@ -6681,7 +6688,12 @@
         <f>B39+4</f>
         <v/>
       </c>
-      <c r="E39" s="283" t="n"/>
+      <c r="E39" s="410" t="inlineStr">
+        <is>
+          <t>Geo - Mar
+5º e 6º tempos</t>
+        </is>
+      </c>
       <c r="F39" s="283" t="n"/>
       <c r="G39" s="456" t="inlineStr">
         <is>
@@ -6695,12 +6707,7 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="I39" s="443" t="inlineStr">
-        <is>
-          <t>DaF - CBu-EFr-Eth
-6º e 7º tempos</t>
-        </is>
-      </c>
+      <c r="I39" s="443" t="n"/>
       <c r="J39" s="265" t="n"/>
     </row>
     <row r="40" ht="18" customFormat="1" customHeight="1" s="4">
@@ -6708,11 +6715,10 @@
       <c r="B40" s="313" t="n"/>
       <c r="C40" s="313" t="n"/>
       <c r="D40" s="350" t="n"/>
-      <c r="E40" s="283" t="n"/>
+      <c r="E40" s="406" t="n"/>
       <c r="F40" s="283" t="n"/>
       <c r="G40" s="437" t="n"/>
       <c r="H40" s="437" t="n"/>
-      <c r="I40" s="437" t="n"/>
       <c r="J40" s="352" t="n"/>
     </row>
     <row r="41" ht="18" customFormat="1" customHeight="1" s="4" thickBot="1">
@@ -6720,11 +6726,10 @@
       <c r="B41" s="313" t="n"/>
       <c r="C41" s="313" t="n"/>
       <c r="D41" s="350" t="n"/>
-      <c r="E41" s="283" t="n"/>
+      <c r="E41" s="407" t="n"/>
       <c r="F41" s="283" t="n"/>
       <c r="G41" s="439" t="n"/>
       <c r="H41" s="439" t="n"/>
-      <c r="I41" s="439" t="n"/>
       <c r="J41" s="352" t="n"/>
     </row>
     <row r="42" ht="18" customFormat="1" customHeight="1" s="4">
@@ -6803,12 +6808,7 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="442" t="inlineStr">
-        <is>
-          <t>Geo - Mar
-5º e 6º tempos</t>
-        </is>
-      </c>
+      <c r="E45" s="442" t="n"/>
       <c r="F45" s="441" t="inlineStr">
         <is>
           <t>Mat - Bre/JJ
@@ -6816,7 +6816,7 @@
         </is>
       </c>
       <c r="G45" s="449" t="n"/>
-      <c r="H45" s="417" t="inlineStr">
+      <c r="H45" s="449" t="inlineStr">
         <is>
           <t>Bio - Ale
 5º e 6º tempos</t>
@@ -6836,9 +6836,8 @@
       <c r="B46" s="313" t="n"/>
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
-      <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
-      <c r="H46" s="406" t="n"/>
+      <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
@@ -6848,9 +6847,8 @@
       <c r="B47" s="313" t="n"/>
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
-      <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
-      <c r="H47" s="407" t="n"/>
+      <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
@@ -7154,10 +7152,8 @@
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
     <mergeCell ref="A12:A14"/>
-    <mergeCell ref="E45:E47"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
-    <mergeCell ref="I39:I41"/>
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
@@ -7219,6 +7215,7 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
+    <mergeCell ref="E39:E41"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
     <mergeCell ref="B42:B44"/>
@@ -7267,6 +7264,7 @@
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
+    <mergeCell ref="I36:I38"/>
     <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
@@ -20023,7 +20021,12 @@
         </is>
       </c>
       <c r="H36" s="283" t="n"/>
-      <c r="I36" s="442" t="n"/>
+      <c r="I36" s="443" t="inlineStr">
+        <is>
+          <t>DaF - CBu-EFr-Eth
+6º e 7º tempos</t>
+        </is>
+      </c>
       <c r="J36" s="265" t="n"/>
       <c r="L36" s="81" t="inlineStr">
         <is>
@@ -20045,6 +20048,7 @@
       <c r="F37" s="437" t="n"/>
       <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
+      <c r="I37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
@@ -20066,6 +20070,7 @@
       <c r="F38" s="439" t="n"/>
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
+      <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
@@ -20086,7 +20091,12 @@
         <f>B39+4</f>
         <v/>
       </c>
-      <c r="E39" s="283" t="n"/>
+      <c r="E39" s="442" t="inlineStr">
+        <is>
+          <t>Geo - Mar
+5º e 6º tempos</t>
+        </is>
+      </c>
       <c r="F39" s="283" t="n"/>
       <c r="G39" s="456" t="inlineStr">
         <is>
@@ -20100,12 +20110,7 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="I39" s="443" t="inlineStr">
-        <is>
-          <t>DaF - CBu-EFr-Eth
-6º e 7º tempos</t>
-        </is>
-      </c>
+      <c r="I39" s="443" t="n"/>
       <c r="J39" s="265" t="n"/>
     </row>
     <row r="40" ht="18" customFormat="1" customHeight="1" s="4">
@@ -20113,11 +20118,10 @@
       <c r="B40" s="313" t="n"/>
       <c r="C40" s="313" t="n"/>
       <c r="D40" s="350" t="n"/>
-      <c r="E40" s="283" t="n"/>
+      <c r="E40" s="437" t="n"/>
       <c r="F40" s="283" t="n"/>
       <c r="G40" s="437" t="n"/>
       <c r="H40" s="437" t="n"/>
-      <c r="I40" s="437" t="n"/>
       <c r="J40" s="352" t="n"/>
     </row>
     <row r="41" ht="18" customFormat="1" customHeight="1" s="4" thickBot="1">
@@ -20125,11 +20129,10 @@
       <c r="B41" s="313" t="n"/>
       <c r="C41" s="313" t="n"/>
       <c r="D41" s="350" t="n"/>
-      <c r="E41" s="283" t="n"/>
+      <c r="E41" s="439" t="n"/>
       <c r="F41" s="283" t="n"/>
       <c r="G41" s="439" t="n"/>
       <c r="H41" s="439" t="n"/>
-      <c r="I41" s="439" t="n"/>
       <c r="J41" s="352" t="n"/>
     </row>
     <row r="42" ht="18" customFormat="1" customHeight="1" s="4">
@@ -20208,12 +20211,7 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="442" t="inlineStr">
-        <is>
-          <t>Geo - Mar
-5º e 6º tempos</t>
-        </is>
-      </c>
+      <c r="E45" s="442" t="n"/>
       <c r="F45" s="441" t="inlineStr">
         <is>
           <t>Mat - Bre/JJ
@@ -20241,7 +20239,6 @@
       <c r="B46" s="313" t="n"/>
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
-      <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
       <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
@@ -20253,7 +20250,6 @@
       <c r="B47" s="313" t="n"/>
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
-      <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
       <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
@@ -20559,10 +20555,8 @@
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
     <mergeCell ref="A12:A14"/>
-    <mergeCell ref="E45:E47"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
-    <mergeCell ref="I39:I41"/>
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
@@ -20624,6 +20618,7 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
+    <mergeCell ref="E39:E41"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
     <mergeCell ref="B42:B44"/>
@@ -20672,6 +20667,7 @@
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
+    <mergeCell ref="I36:I38"/>
     <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>

</xml_diff>

<commit_message>
12C1/12C2: Química corrigida para 2 tempos, movida para 09/11
2ª prova de Química estava com apenas 1 tempo (bug de rodada anterior)
-- corrigida para 2 tempos, seguindo o padrão normal de DOIS_TEMPOS
(igual à 1ª prova, já correta em 11/09).

Testadas todas as combinações de 2 tempos na quarta-feira (posição
antiga): 1º-2º doaria a única aula semanal de Sociologia em 12C1;
5º-6º cruza o recreio; 6º-7º é bloco inválido lá (7º tempo não existe
na grade de quarta). Nenhuma opção cabe na quarta-feira.

Movida para semana 15 segunda (09/11), 6º-7º tempos -- tempo próprio
da profa. Fab em 12C1 (12C2 coberta por coordenação entre turmas
irmãs); slot já estava livre (Geografia tinha saído de lá numa rodada
anterior).

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6611,12 +6611,7 @@
 10º e 11º tempos</t>
         </is>
       </c>
-      <c r="G36" s="451" t="inlineStr">
-        <is>
-          <t>Qui - CAl/Fab
-1º tempo</t>
-        </is>
-      </c>
+      <c r="G36" s="451" t="n"/>
       <c r="H36" s="283" t="n"/>
       <c r="I36" s="443" t="inlineStr">
         <is>
@@ -6643,7 +6638,6 @@
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="437" t="n"/>
-      <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="I37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
@@ -6665,7 +6659,6 @@
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="439" t="n"/>
-      <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
@@ -6808,7 +6801,12 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="442" t="n"/>
+      <c r="E45" s="419" t="inlineStr">
+        <is>
+          <t>Qui - CAl/Fab
+6º e 7º tempos</t>
+        </is>
+      </c>
       <c r="F45" s="441" t="inlineStr">
         <is>
           <t>Mat - Bre/JJ
@@ -6836,6 +6834,7 @@
       <c r="B46" s="313" t="n"/>
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
+      <c r="E46" s="406" t="n"/>
       <c r="F46" s="437" t="n"/>
       <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
@@ -6847,6 +6846,7 @@
       <c r="B47" s="313" t="n"/>
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
+      <c r="E47" s="407" t="n"/>
       <c r="F47" s="439" t="n"/>
       <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
@@ -7152,6 +7152,7 @@
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
     <mergeCell ref="A12:A14"/>
+    <mergeCell ref="E45:E47"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
     <mergeCell ref="B33:B35"/>
@@ -7262,7 +7263,6 @@
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
     <mergeCell ref="I30:I32"/>
@@ -11614,7 +11614,7 @@
       </c>
       <c r="E42" s="283" t="n"/>
       <c r="F42" s="283" t="n"/>
-      <c r="G42" s="419" t="inlineStr">
+      <c r="G42" s="451" t="inlineStr">
         <is>
           <t>Qui - Fab
 2º tempo</t>
@@ -11647,7 +11647,7 @@
       <c r="D43" s="350" t="n"/>
       <c r="E43" s="283" t="n"/>
       <c r="F43" s="283" t="n"/>
-      <c r="G43" s="406" t="n"/>
+      <c r="G43" s="437" t="n"/>
       <c r="H43" s="437" t="n"/>
       <c r="I43" s="437" t="n"/>
       <c r="J43" s="352" t="n"/>
@@ -11660,7 +11660,7 @@
       <c r="D44" s="350" t="n"/>
       <c r="E44" s="283" t="n"/>
       <c r="F44" s="283" t="n"/>
-      <c r="G44" s="407" t="n"/>
+      <c r="G44" s="439" t="n"/>
       <c r="H44" s="439" t="n"/>
       <c r="I44" s="439" t="n"/>
       <c r="J44" s="352" t="n"/>
@@ -20030,12 +20030,7 @@
 10º e 11º tempos</t>
         </is>
       </c>
-      <c r="G36" s="451" t="inlineStr">
-        <is>
-          <t>Qui - CAl/Fab
-1º tempo</t>
-        </is>
-      </c>
+      <c r="G36" s="451" t="n"/>
       <c r="H36" s="283" t="n"/>
       <c r="I36" s="443" t="inlineStr">
         <is>
@@ -20062,7 +20057,6 @@
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="437" t="n"/>
-      <c r="G37" s="437" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="I37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
@@ -20084,7 +20078,6 @@
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="439" t="n"/>
-      <c r="G38" s="439" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
@@ -20227,7 +20220,12 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="442" t="n"/>
+      <c r="E45" s="451" t="inlineStr">
+        <is>
+          <t>Qui - CAl/Fab
+6º e 7º tempos</t>
+        </is>
+      </c>
       <c r="F45" s="441" t="inlineStr">
         <is>
           <t>Mat - Bre/JJ
@@ -20255,6 +20253,7 @@
       <c r="B46" s="313" t="n"/>
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
+      <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
       <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
@@ -20266,6 +20265,7 @@
       <c r="B47" s="313" t="n"/>
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
+      <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
       <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
@@ -20571,6 +20571,7 @@
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
     <mergeCell ref="A12:A14"/>
+    <mergeCell ref="E45:E47"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
     <mergeCell ref="B33:B35"/>
@@ -20681,7 +20682,6 @@
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="G36:G38"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
     <mergeCell ref="I30:I32"/>

</xml_diff>

<commit_message>
10C2: Inglês (2ª prova) movida de 20/10 para 11/11
Bloco atual (terça, 4º-5º tempos) usava o 5º tempo próprio da profa.
Vir + o 4º emprestado de Artes. A aula dupla real dela nessa turma é
quarta-feira, 4º-5º tempos (zero cessão). 11/11 é a única
quarta-feira de novembro dentro do limite de 6 dias antes do CC final
(17/11) -- 18/11 e 25/11 já ficam depois do limite.

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6801,7 +6801,7 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="419" t="inlineStr">
+      <c r="E45" s="451" t="inlineStr">
         <is>
           <t>Qui - CAl/Fab
 6º e 7º tempos</t>
@@ -6834,7 +6834,7 @@
       <c r="B46" s="313" t="n"/>
       <c r="C46" s="313" t="n"/>
       <c r="D46" s="350" t="n"/>
-      <c r="E46" s="406" t="n"/>
+      <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
       <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
@@ -6846,7 +6846,7 @@
       <c r="B47" s="313" t="n"/>
       <c r="C47" s="313" t="n"/>
       <c r="D47" s="350" t="n"/>
-      <c r="E47" s="407" t="n"/>
+      <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
       <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
@@ -14864,12 +14864,7 @@
         <v/>
       </c>
       <c r="E36" s="283" t="n"/>
-      <c r="F36" s="440" t="inlineStr">
-        <is>
-          <t>Ing - Vir
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="F36" s="440" t="n"/>
       <c r="G36" s="436" t="inlineStr">
         <is>
           <t>GL - EFr-Car-Swa
@@ -14901,7 +14896,6 @@
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="283" t="n"/>
-      <c r="F37" s="437" t="n"/>
       <c r="G37" s="437" t="n"/>
       <c r="H37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
@@ -14922,7 +14916,6 @@
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="283" t="n"/>
-      <c r="F38" s="439" t="n"/>
       <c r="G38" s="439" t="n"/>
       <c r="H38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
@@ -15093,7 +15086,12 @@
 10º e 11º tempos</t>
         </is>
       </c>
-      <c r="G45" s="435" t="n"/>
+      <c r="G45" s="408" t="inlineStr">
+        <is>
+          <t>Ing - Vir
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="H45" s="435" t="n"/>
       <c r="I45" s="386" t="inlineStr">
         <is>
@@ -15111,7 +15109,7 @@
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
-      <c r="G46" s="438" t="n"/>
+      <c r="G46" s="406" t="n"/>
       <c r="H46" s="438" t="n"/>
       <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
@@ -15124,7 +15122,7 @@
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
-      <c r="G47" s="438" t="n"/>
+      <c r="G47" s="407" t="n"/>
       <c r="H47" s="438" t="n"/>
       <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
@@ -15442,6 +15440,7 @@
     <mergeCell ref="E45:E47"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
+    <mergeCell ref="G45:G47"/>
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
@@ -15506,7 +15505,6 @@
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="D36:D38"/>
     <mergeCell ref="M26:N26"/>
-    <mergeCell ref="F36:F38"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="J9:J11"/>

</xml_diff>

<commit_message>
12C1/12C2: Biologia (2ª prova) movida de 12/11 para 22/10
Semana 15 quinta (12/11) -> semana 12 quinta (22/10), mesmo bloco
5º-6º tempos -- mesmo dia da semana, só a semana mudou.

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6612,7 +6612,12 @@
         </is>
       </c>
       <c r="G36" s="451" t="n"/>
-      <c r="H36" s="283" t="n"/>
+      <c r="H36" s="417" t="inlineStr">
+        <is>
+          <t>Bio - Ale
+5º e 6º tempos</t>
+        </is>
+      </c>
       <c r="I36" s="443" t="inlineStr">
         <is>
           <t>DaF - CBu-EFr-Eth
@@ -6638,7 +6643,7 @@
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="437" t="n"/>
-      <c r="H37" s="283" t="n"/>
+      <c r="H37" s="406" t="n"/>
       <c r="I37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
@@ -6659,7 +6664,7 @@
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="439" t="n"/>
-      <c r="H38" s="283" t="n"/>
+      <c r="H38" s="407" t="n"/>
       <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
@@ -6814,12 +6819,7 @@
         </is>
       </c>
       <c r="G45" s="449" t="n"/>
-      <c r="H45" s="449" t="inlineStr">
-        <is>
-          <t>Bio - Ale
-5º e 6º tempos</t>
-        </is>
-      </c>
+      <c r="H45" s="449" t="n"/>
       <c r="I45" s="386" t="inlineStr">
         <is>
           <t>2CH
@@ -6836,7 +6836,6 @@
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
-      <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
@@ -6848,7 +6847,6 @@
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
-      <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
@@ -7181,7 +7179,6 @@
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="H45:H47"/>
     <mergeCell ref="J30:J32"/>
     <mergeCell ref="B48:B50"/>
     <mergeCell ref="D48:D50"/>
@@ -7231,6 +7228,7 @@
     <mergeCell ref="H39:H41"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="E15:E17"/>
+    <mergeCell ref="H36:H38"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
@@ -14683,7 +14681,7 @@
       </c>
       <c r="E30" s="283" t="n"/>
       <c r="F30" s="283" t="n"/>
-      <c r="G30" s="405" t="inlineStr">
+      <c r="G30" s="436" t="inlineStr">
         <is>
           <t>GL - EFr-Car-Swa
 2º e 3º tempos</t>
@@ -14721,7 +14719,7 @@
       <c r="D31" s="350" t="n"/>
       <c r="E31" s="283" t="n"/>
       <c r="F31" s="283" t="n"/>
-      <c r="G31" s="406" t="n"/>
+      <c r="G31" s="437" t="n"/>
       <c r="H31" s="437" t="n"/>
       <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
@@ -14740,7 +14738,7 @@
       <c r="D32" s="350" t="n"/>
       <c r="E32" s="283" t="n"/>
       <c r="F32" s="283" t="n"/>
-      <c r="G32" s="407" t="n"/>
+      <c r="G32" s="439" t="n"/>
       <c r="H32" s="439" t="n"/>
       <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
@@ -14866,7 +14864,7 @@
         <f>B36+4</f>
         <v/>
       </c>
-      <c r="E36" s="421" t="inlineStr">
+      <c r="E36" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - BPad/MFo/SMo
 1º ao 3º tempos</t>
@@ -14880,7 +14878,7 @@
 9º e 10º tempos</t>
         </is>
       </c>
-      <c r="I36" s="426" t="inlineStr">
+      <c r="I36" s="456" t="inlineStr">
         <is>
           <t>Soc - Kle
 5º tempo</t>
@@ -14903,9 +14901,9 @@
       <c r="B37" s="313" t="n"/>
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
-      <c r="E37" s="406" t="n"/>
+      <c r="E37" s="437" t="n"/>
       <c r="H37" s="437" t="n"/>
-      <c r="I37" s="406" t="n"/>
+      <c r="I37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
@@ -14923,9 +14921,9 @@
       <c r="B38" s="313" t="n"/>
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
-      <c r="E38" s="407" t="n"/>
+      <c r="E38" s="439" t="n"/>
       <c r="H38" s="439" t="n"/>
-      <c r="I38" s="407" t="n"/>
+      <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
     <row r="39" ht="18" customFormat="1" customHeight="1" s="4">
@@ -14946,7 +14944,7 @@
         <f>B39+4</f>
         <v/>
       </c>
-      <c r="E39" s="419" t="inlineStr">
+      <c r="E39" s="451" t="inlineStr">
         <is>
           <t>Qui - CAl
 4º e 5º tempos</t>
@@ -14973,7 +14971,7 @@
       <c r="B40" s="313" t="n"/>
       <c r="C40" s="313" t="n"/>
       <c r="D40" s="350" t="n"/>
-      <c r="E40" s="406" t="n"/>
+      <c r="E40" s="437" t="n"/>
       <c r="F40" s="283" t="n"/>
       <c r="G40" s="437" t="n"/>
       <c r="H40" s="437" t="n"/>
@@ -14985,7 +14983,7 @@
       <c r="B41" s="313" t="n"/>
       <c r="C41" s="313" t="n"/>
       <c r="D41" s="350" t="n"/>
-      <c r="E41" s="407" t="n"/>
+      <c r="E41" s="439" t="n"/>
       <c r="F41" s="283" t="n"/>
       <c r="G41" s="439" t="n"/>
       <c r="H41" s="439" t="n"/>
@@ -20023,7 +20021,12 @@
         </is>
       </c>
       <c r="G36" s="451" t="n"/>
-      <c r="H36" s="283" t="n"/>
+      <c r="H36" s="449" t="inlineStr">
+        <is>
+          <t>Bio - Ale
+5º e 6º tempos</t>
+        </is>
+      </c>
       <c r="I36" s="443" t="inlineStr">
         <is>
           <t>DaF - CBu-EFr-Eth
@@ -20049,7 +20052,7 @@
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="437" t="n"/>
-      <c r="H37" s="283" t="n"/>
+      <c r="H37" s="437" t="n"/>
       <c r="I37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
@@ -20070,7 +20073,7 @@
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="439" t="n"/>
-      <c r="H38" s="283" t="n"/>
+      <c r="H38" s="439" t="n"/>
       <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
@@ -20225,12 +20228,7 @@
         </is>
       </c>
       <c r="G45" s="449" t="n"/>
-      <c r="H45" s="449" t="inlineStr">
-        <is>
-          <t>Bio - Ale
-5º e 6º tempos</t>
-        </is>
-      </c>
+      <c r="H45" s="449" t="n"/>
       <c r="I45" s="386" t="inlineStr">
         <is>
           <t>2CH
@@ -20247,7 +20245,6 @@
       <c r="D46" s="350" t="n"/>
       <c r="E46" s="437" t="n"/>
       <c r="F46" s="437" t="n"/>
-      <c r="H46" s="437" t="n"/>
       <c r="I46" s="351" t="n"/>
       <c r="J46" s="352" t="n"/>
       <c r="L46" s="331" t="n"/>
@@ -20259,7 +20256,6 @@
       <c r="D47" s="350" t="n"/>
       <c r="E47" s="439" t="n"/>
       <c r="F47" s="439" t="n"/>
-      <c r="H47" s="439" t="n"/>
       <c r="I47" s="387" t="n"/>
       <c r="J47" s="352" t="n"/>
       <c r="L47" s="332" t="n"/>
@@ -20592,7 +20588,6 @@
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
     <mergeCell ref="B39:B41"/>
-    <mergeCell ref="H45:H47"/>
     <mergeCell ref="J30:J32"/>
     <mergeCell ref="B48:B50"/>
     <mergeCell ref="D48:D50"/>
@@ -20642,6 +20637,7 @@
     <mergeCell ref="H39:H41"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="E15:E17"/>
+    <mergeCell ref="H36:H38"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>

</xml_diff>

<commit_message>
10C1/10C2: Química (1ª prova) - mudança de dia, mesma semana
Pedido repassado do professor de Química: mudar de segunda (24/08)
para sexta (28/08), mesma semana.

Testados todos os blocos de 2 tempos na sexta-feira: só 3º-4º tempos
é válido para as duas turmas (4º-5º e 5º-6º ficam inválidos em 10C2
porque o 5º tempo é Sociologia, que não pode doar).

Movida: semana 4 segunda (24/08) -> semana 4 sexta (28/08), 3º-4º
tempos.

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6612,7 +6612,7 @@
         </is>
       </c>
       <c r="G36" s="451" t="n"/>
-      <c r="H36" s="417" t="inlineStr">
+      <c r="H36" s="449" t="inlineStr">
         <is>
           <t>Bio - Ale
 5º e 6º tempos</t>
@@ -6643,7 +6643,7 @@
       <c r="D37" s="350" t="n"/>
       <c r="E37" s="283" t="n"/>
       <c r="F37" s="437" t="n"/>
-      <c r="H37" s="406" t="n"/>
+      <c r="H37" s="437" t="n"/>
       <c r="I37" s="437" t="n"/>
       <c r="J37" s="352" t="n"/>
       <c r="L37" s="4" t="inlineStr">
@@ -6664,7 +6664,7 @@
       <c r="D38" s="350" t="n"/>
       <c r="E38" s="283" t="n"/>
       <c r="F38" s="439" t="n"/>
-      <c r="H38" s="407" t="n"/>
+      <c r="H38" s="439" t="n"/>
       <c r="I38" s="439" t="n"/>
       <c r="J38" s="352" t="n"/>
     </row>
@@ -12537,12 +12537,7 @@
         <f>B12+4</f>
         <v/>
       </c>
-      <c r="E12" s="451" t="inlineStr">
-        <is>
-          <t>Qui - CAl
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="E12" s="451" t="n"/>
       <c r="F12" s="449" t="inlineStr">
         <is>
           <t>Bio - Lza
@@ -12556,7 +12551,12 @@
         </is>
       </c>
       <c r="H12" s="11" t="n"/>
-      <c r="I12" s="11" t="n"/>
+      <c r="I12" s="451" t="inlineStr">
+        <is>
+          <t>Qui - CAl
+3º e 4º tempos</t>
+        </is>
+      </c>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
       <c r="M12" s="15" t="n"/>
@@ -12568,11 +12568,10 @@
       <c r="B13" s="313" t="n"/>
       <c r="C13" s="313" t="n"/>
       <c r="D13" s="314" t="n"/>
-      <c r="E13" s="437" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="437" t="n"/>
       <c r="H13" s="222" t="n"/>
-      <c r="I13" s="222" t="n"/>
+      <c r="I13" s="437" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
@@ -12584,11 +12583,10 @@
       <c r="B14" s="313" t="n"/>
       <c r="C14" s="313" t="n"/>
       <c r="D14" s="314" t="n"/>
-      <c r="E14" s="439" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="439" t="n"/>
       <c r="H14" s="222" t="n"/>
-      <c r="I14" s="222" t="n"/>
+      <c r="I14" s="439" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
@@ -13736,7 +13734,6 @@
     <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
-    <mergeCell ref="E12:E14"/>
     <mergeCell ref="J33:J35"/>
     <mergeCell ref="H42:H44"/>
     <mergeCell ref="J42:J44"/>
@@ -13845,6 +13842,7 @@
     <mergeCell ref="M28:N28"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B18:B20"/>
+    <mergeCell ref="I12:I14"/>
     <mergeCell ref="B60:B62"/>
     <mergeCell ref="B9:B11"/>
     <mergeCell ref="F33:F35"/>
@@ -14230,12 +14228,7 @@
         <f>B12+4</f>
         <v/>
       </c>
-      <c r="E12" s="451" t="inlineStr">
-        <is>
-          <t>Qui - CAl
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="E12" s="451" t="n"/>
       <c r="F12" s="449" t="inlineStr">
         <is>
           <t>Bio - Lza
@@ -14249,7 +14242,12 @@
         </is>
       </c>
       <c r="H12" s="11" t="n"/>
-      <c r="I12" s="11" t="n"/>
+      <c r="I12" s="419" t="inlineStr">
+        <is>
+          <t>Qui - CAl
+3º e 4º tempos</t>
+        </is>
+      </c>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
       <c r="M12" s="15" t="n"/>
@@ -14261,11 +14259,10 @@
       <c r="B13" s="313" t="n"/>
       <c r="C13" s="313" t="n"/>
       <c r="D13" s="314" t="n"/>
-      <c r="E13" s="437" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="437" t="n"/>
       <c r="H13" s="222" t="n"/>
-      <c r="I13" s="222" t="n"/>
+      <c r="I13" s="406" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
@@ -14277,11 +14274,10 @@
       <c r="B14" s="313" t="n"/>
       <c r="C14" s="313" t="n"/>
       <c r="D14" s="314" t="n"/>
-      <c r="E14" s="439" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="439" t="n"/>
       <c r="H14" s="222" t="n"/>
-      <c r="I14" s="222" t="n"/>
+      <c r="I14" s="407" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
@@ -15441,7 +15437,6 @@
     <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
-    <mergeCell ref="E12:E14"/>
     <mergeCell ref="J33:J35"/>
     <mergeCell ref="J42:J44"/>
     <mergeCell ref="B3:B5"/>
@@ -15548,6 +15543,7 @@
     <mergeCell ref="M28:N28"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B18:B20"/>
+    <mergeCell ref="I12:I14"/>
     <mergeCell ref="B60:B62"/>
     <mergeCell ref="B9:B11"/>
     <mergeCell ref="F33:F35"/>

</xml_diff>

<commit_message>
12C1/12C2: LP/LIT/RED movida de 09/10 para 06/10
Testadas todas as combinações de 3 tempos na semana 10 (vazia):
- 07/10 (quarta) rejeitado: 2º tempo é Sociologia, não pode doar.
- Quinta 1º-3º (Artes+Física, manhã) e terça 9º-11º (Apoio+História,
  tarde) são as duas opções válidas encontradas.

Aplicado, a pedido do usuário: LP/LIT/RED semana 10 sexta (09/10) ->
semana 10 terça (06/10), tempos 9º-11º.

verificar_calendario.py: 0 PROBLEMA (com o AVISO esperado de
'tempos 7-11', escolha consciente do usuário). 5 relatórios
regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6430,15 +6430,15 @@
         <v/>
       </c>
       <c r="E30" s="435" t="n"/>
-      <c r="F30" s="435" t="n"/>
+      <c r="F30" s="421" t="inlineStr">
+        <is>
+          <t>LP/LIT/RED - AMu/Deb
+9º ao 11º tempos</t>
+        </is>
+      </c>
       <c r="G30" s="435" t="n"/>
       <c r="H30" s="435" t="n"/>
-      <c r="I30" s="458" t="inlineStr">
-        <is>
-          <t>LP/LIT/RED - AMu/Deb
-1º ao 3º tempos</t>
-        </is>
-      </c>
+      <c r="I30" s="458" t="n"/>
       <c r="J30" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -6458,10 +6458,9 @@
       <c r="C31" s="313" t="n"/>
       <c r="D31" s="350" t="n"/>
       <c r="E31" s="438" t="n"/>
-      <c r="F31" s="438" t="n"/>
+      <c r="F31" s="406" t="n"/>
       <c r="G31" s="438" t="n"/>
       <c r="H31" s="438" t="n"/>
-      <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -6477,10 +6476,9 @@
       <c r="C32" s="313" t="n"/>
       <c r="D32" s="350" t="n"/>
       <c r="E32" s="438" t="n"/>
-      <c r="F32" s="438" t="n"/>
+      <c r="F32" s="407" t="n"/>
       <c r="G32" s="438" t="n"/>
       <c r="H32" s="438" t="n"/>
-      <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -7175,6 +7173,7 @@
     <mergeCell ref="G57:G59"/>
     <mergeCell ref="A60:A62"/>
     <mergeCell ref="I57:I59"/>
+    <mergeCell ref="F30:F32"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
@@ -7263,7 +7262,6 @@
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
-    <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>
@@ -11748,7 +11746,7 @@
         </is>
       </c>
       <c r="G48" s="441" t="n"/>
-      <c r="H48" s="409" t="inlineStr">
+      <c r="H48" s="441" t="inlineStr">
         <is>
           <t>Mat - BrSa
 4º e 5º tempos</t>
@@ -11767,7 +11765,7 @@
       <c r="C49" s="313" t="n"/>
       <c r="D49" s="350" t="n"/>
       <c r="F49" s="437" t="n"/>
-      <c r="H49" s="406" t="n"/>
+      <c r="H49" s="437" t="n"/>
       <c r="I49" s="315" t="n"/>
       <c r="J49" s="352" t="n"/>
     </row>
@@ -11777,7 +11775,7 @@
       <c r="C50" s="313" t="n"/>
       <c r="D50" s="350" t="n"/>
       <c r="F50" s="439" t="n"/>
-      <c r="H50" s="407" t="n"/>
+      <c r="H50" s="439" t="n"/>
       <c r="I50" s="315" t="n"/>
       <c r="J50" s="352" t="n"/>
     </row>
@@ -19831,15 +19829,15 @@
         <v/>
       </c>
       <c r="E30" s="283" t="n"/>
-      <c r="F30" s="435" t="n"/>
+      <c r="F30" s="458" t="inlineStr">
+        <is>
+          <t>LP/LIT/RED - AMu/Deb
+9º ao 11º tempos</t>
+        </is>
+      </c>
       <c r="G30" s="435" t="n"/>
       <c r="H30" s="435" t="n"/>
-      <c r="I30" s="458" t="inlineStr">
-        <is>
-          <t>LP/LIT/RED - AMu/Deb
-1º ao 3º tempos</t>
-        </is>
-      </c>
+      <c r="I30" s="458" t="n"/>
       <c r="J30" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -19859,10 +19857,9 @@
       <c r="C31" s="313" t="n"/>
       <c r="D31" s="350" t="n"/>
       <c r="E31" s="283" t="n"/>
-      <c r="F31" s="438" t="n"/>
+      <c r="F31" s="437" t="n"/>
       <c r="G31" s="438" t="n"/>
       <c r="H31" s="438" t="n"/>
-      <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -19878,10 +19875,9 @@
       <c r="C32" s="313" t="n"/>
       <c r="D32" s="350" t="n"/>
       <c r="E32" s="283" t="n"/>
-      <c r="F32" s="438" t="n"/>
+      <c r="F32" s="439" t="n"/>
       <c r="G32" s="438" t="n"/>
       <c r="H32" s="438" t="n"/>
-      <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -20576,6 +20572,7 @@
     <mergeCell ref="G57:G59"/>
     <mergeCell ref="A60:A62"/>
     <mergeCell ref="I57:I59"/>
+    <mergeCell ref="F30:F32"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
@@ -20664,7 +20661,6 @@
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
-    <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>

</xml_diff>

<commit_message>
12C1/12C2: LP/LIT/RED revertida de volta para 09/10
Usuário pediu para reverter a mudança anterior (terça 06/10): mantida
na posição original, semana 10 sexta (09/10), tempos 1º-3º.

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6430,15 +6430,15 @@
         <v/>
       </c>
       <c r="E30" s="435" t="n"/>
-      <c r="F30" s="421" t="inlineStr">
-        <is>
-          <t>LP/LIT/RED - AMu/Deb
-9º ao 11º tempos</t>
-        </is>
-      </c>
+      <c r="F30" s="458" t="n"/>
       <c r="G30" s="435" t="n"/>
       <c r="H30" s="435" t="n"/>
-      <c r="I30" s="458" t="n"/>
+      <c r="I30" s="421" t="inlineStr">
+        <is>
+          <t>LP/LIT/RED - AMu/Deb
+1º ao 3º tempos</t>
+        </is>
+      </c>
       <c r="J30" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -6458,9 +6458,9 @@
       <c r="C31" s="313" t="n"/>
       <c r="D31" s="350" t="n"/>
       <c r="E31" s="438" t="n"/>
-      <c r="F31" s="406" t="n"/>
       <c r="G31" s="438" t="n"/>
       <c r="H31" s="438" t="n"/>
+      <c r="I31" s="406" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -6476,9 +6476,9 @@
       <c r="C32" s="313" t="n"/>
       <c r="D32" s="350" t="n"/>
       <c r="E32" s="438" t="n"/>
-      <c r="F32" s="407" t="n"/>
       <c r="G32" s="438" t="n"/>
       <c r="H32" s="438" t="n"/>
+      <c r="I32" s="407" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -7173,7 +7173,6 @@
     <mergeCell ref="G57:G59"/>
     <mergeCell ref="A60:A62"/>
     <mergeCell ref="I57:I59"/>
-    <mergeCell ref="F30:F32"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
@@ -7262,6 +7261,7 @@
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
+    <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>
@@ -19829,15 +19829,15 @@
         <v/>
       </c>
       <c r="E30" s="283" t="n"/>
-      <c r="F30" s="458" t="inlineStr">
-        <is>
-          <t>LP/LIT/RED - AMu/Deb
-9º ao 11º tempos</t>
-        </is>
-      </c>
+      <c r="F30" s="458" t="n"/>
       <c r="G30" s="435" t="n"/>
       <c r="H30" s="435" t="n"/>
-      <c r="I30" s="458" t="n"/>
+      <c r="I30" s="458" t="inlineStr">
+        <is>
+          <t>LP/LIT/RED - AMu/Deb
+1º ao 3º tempos</t>
+        </is>
+      </c>
       <c r="J30" s="183" t="inlineStr">
         <is>
           <t>unterrichtsfrei sem aula</t>
@@ -19857,9 +19857,9 @@
       <c r="C31" s="313" t="n"/>
       <c r="D31" s="350" t="n"/>
       <c r="E31" s="283" t="n"/>
-      <c r="F31" s="437" t="n"/>
       <c r="G31" s="438" t="n"/>
       <c r="H31" s="438" t="n"/>
+      <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -19875,9 +19875,9 @@
       <c r="C32" s="313" t="n"/>
       <c r="D32" s="350" t="n"/>
       <c r="E32" s="283" t="n"/>
-      <c r="F32" s="439" t="n"/>
       <c r="G32" s="438" t="n"/>
       <c r="H32" s="438" t="n"/>
+      <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -20572,7 +20572,6 @@
     <mergeCell ref="G57:G59"/>
     <mergeCell ref="A60:A62"/>
     <mergeCell ref="I57:I59"/>
-    <mergeCell ref="F30:F32"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
@@ -20661,6 +20660,7 @@
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="I36:I38"/>
+    <mergeCell ref="I30:I32"/>
     <mergeCell ref="A48:A50"/>
     <mergeCell ref="I45:I47"/>
     <mergeCell ref="F54:F56"/>

</xml_diff>

<commit_message>
11C1/11C2: 3 reposicionamentos (Inglês, Geografia, Matemática)
Análise apresentada ao usuário antes de aplicar, conforme pedido.

1. Inglês (11C1 apenas): semana 9 segunda (28/09) -> semana 12
   segunda (19/10), mesmo bloco 6º-7º tempos.
2. Geografia (11C1+11C2): semana 10 quarta (07/10) -> semana 5
   segunda (31/08), tempos 2º-3º.
3. Matemática (11C1+11C2): semana 8 segunda (21/09) -> semana 4
   quinta (27/08), tempos 1º-2º (bloco antigo não cabia em nenhuma
   das duas semanas pedidas na segunda-feira; quinta foi a
   alternativa encontrada, livre nas duas semanas -- usei semana 4
   por padrão, sem diferença técnica frente à semana 6).

verificar_calendario.py: 0 PROBLEMA. 5 relatórios regenerados.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6433,7 +6433,7 @@
       <c r="F30" s="458" t="n"/>
       <c r="G30" s="435" t="n"/>
       <c r="H30" s="435" t="n"/>
-      <c r="I30" s="421" t="inlineStr">
+      <c r="I30" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - AMu/Deb
 1º ao 3º tempos</t>
@@ -6460,7 +6460,7 @@
       <c r="E31" s="438" t="n"/>
       <c r="G31" s="438" t="n"/>
       <c r="H31" s="438" t="n"/>
-      <c r="I31" s="406" t="n"/>
+      <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
       <c r="M31" s="328" t="inlineStr">
@@ -6478,7 +6478,7 @@
       <c r="E32" s="438" t="n"/>
       <c r="G32" s="438" t="n"/>
       <c r="H32" s="438" t="n"/>
-      <c r="I32" s="407" t="n"/>
+      <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
       <c r="M32" s="15" t="n"/>
@@ -15949,7 +15949,12 @@
 2º ao 7º tempos</t>
         </is>
       </c>
-      <c r="H12" s="435" t="n"/>
+      <c r="H12" s="441" t="inlineStr">
+        <is>
+          <t>Mat - ClaMe/JJ
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="I12" s="11" t="n"/>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
@@ -15965,7 +15970,7 @@
       <c r="E13" s="437" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="437" t="n"/>
-      <c r="H13" s="438" t="n"/>
+      <c r="H13" s="437" t="n"/>
       <c r="I13" s="222" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
@@ -15981,7 +15986,7 @@
       <c r="E14" s="439" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="439" t="n"/>
-      <c r="H14" s="438" t="n"/>
+      <c r="H14" s="439" t="n"/>
       <c r="I14" s="222" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
@@ -16007,7 +16012,12 @@
         <f>B15+4</f>
         <v/>
       </c>
-      <c r="E15" s="435" t="n"/>
+      <c r="E15" s="442" t="inlineStr">
+        <is>
+          <t>Geo - Mar
+2º e 3º tempos</t>
+        </is>
+      </c>
       <c r="F15" s="434" t="inlineStr">
         <is>
           <t>Hist - Ver
@@ -16032,7 +16042,7 @@
       <c r="B16" s="313" t="n"/>
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
-      <c r="E16" s="438" t="n"/>
+      <c r="E16" s="437" t="n"/>
       <c r="F16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
@@ -16047,7 +16057,7 @@
       <c r="B17" s="313" t="n"/>
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
-      <c r="E17" s="438" t="n"/>
+      <c r="E17" s="439" t="n"/>
       <c r="F17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
@@ -16240,12 +16250,7 @@
         <f>B24+4</f>
         <v/>
       </c>
-      <c r="E24" s="441" t="inlineStr">
-        <is>
-          <t>Mat - ClaMe/JJ
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="E24" s="441" t="n"/>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="459" t="inlineStr">
         <is>
@@ -16269,7 +16274,6 @@
       <c r="B25" s="313" t="n"/>
       <c r="C25" s="313" t="n"/>
       <c r="D25" s="350" t="n"/>
-      <c r="E25" s="437" t="n"/>
       <c r="F25" s="283" t="n"/>
       <c r="G25" s="447" t="n"/>
       <c r="H25" s="283" t="n"/>
@@ -16288,7 +16292,6 @@
       <c r="B26" s="313" t="n"/>
       <c r="C26" s="313" t="n"/>
       <c r="D26" s="350" t="n"/>
-      <c r="E26" s="439" t="n"/>
       <c r="F26" s="283" t="n"/>
       <c r="G26" s="448" t="n"/>
       <c r="H26" s="283" t="n"/>
@@ -16320,12 +16323,7 @@
         <f>B27+4</f>
         <v/>
       </c>
-      <c r="E27" s="460" t="inlineStr">
-        <is>
-          <t>Ing - Bea
-6º e 7º tempos</t>
-        </is>
-      </c>
+      <c r="E27" s="460" t="n"/>
       <c r="F27" s="435" t="n"/>
       <c r="G27" s="435" t="n"/>
       <c r="H27" s="283" t="n"/>
@@ -16344,7 +16342,6 @@
       <c r="B28" s="313" t="n"/>
       <c r="C28" s="313" t="n"/>
       <c r="D28" s="350" t="n"/>
-      <c r="E28" s="437" t="n"/>
       <c r="F28" s="438" t="n"/>
       <c r="G28" s="438" t="n"/>
       <c r="H28" s="283" t="n"/>
@@ -16363,7 +16360,6 @@
       <c r="B29" s="313" t="n"/>
       <c r="C29" s="313" t="n"/>
       <c r="D29" s="350" t="n"/>
-      <c r="E29" s="439" t="n"/>
       <c r="F29" s="438" t="n"/>
       <c r="G29" s="438" t="n"/>
       <c r="H29" s="283" t="n"/>
@@ -16397,12 +16393,7 @@
       </c>
       <c r="E30" s="435" t="n"/>
       <c r="F30" s="283" t="n"/>
-      <c r="G30" s="442" t="inlineStr">
-        <is>
-          <t>Geo - Mar
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="G30" s="442" t="n"/>
       <c r="H30" s="283" t="n"/>
       <c r="I30" s="283" t="n"/>
       <c r="J30" s="183" t="inlineStr">
@@ -16425,7 +16416,6 @@
       <c r="D31" s="350" t="n"/>
       <c r="E31" s="438" t="n"/>
       <c r="F31" s="283" t="n"/>
-      <c r="G31" s="437" t="n"/>
       <c r="H31" s="283" t="n"/>
       <c r="I31" s="283" t="n"/>
       <c r="J31" s="315" t="n"/>
@@ -16444,7 +16434,6 @@
       <c r="D32" s="350" t="n"/>
       <c r="E32" s="438" t="n"/>
       <c r="F32" s="283" t="n"/>
-      <c r="G32" s="439" t="n"/>
       <c r="H32" s="283" t="n"/>
       <c r="I32" s="283" t="n"/>
       <c r="J32" s="315" t="n"/>
@@ -16570,7 +16559,12 @@
         <f>B36+4</f>
         <v/>
       </c>
-      <c r="E36" s="283" t="n"/>
+      <c r="E36" s="440" t="inlineStr">
+        <is>
+          <t>Ing - Bea
+6º e 7º tempos</t>
+        </is>
+      </c>
       <c r="F36" s="435" t="n"/>
       <c r="G36" s="434" t="n"/>
       <c r="H36" s="283" t="n"/>
@@ -16592,7 +16586,7 @@
       <c r="B37" s="313" t="n"/>
       <c r="C37" s="313" t="n"/>
       <c r="D37" s="350" t="n"/>
-      <c r="E37" s="283" t="n"/>
+      <c r="E37" s="437" t="n"/>
       <c r="F37" s="438" t="n"/>
       <c r="H37" s="283" t="n"/>
       <c r="I37" s="438" t="n"/>
@@ -16613,7 +16607,7 @@
       <c r="B38" s="313" t="n"/>
       <c r="C38" s="313" t="n"/>
       <c r="D38" s="350" t="n"/>
-      <c r="E38" s="283" t="n"/>
+      <c r="E38" s="439" t="n"/>
       <c r="F38" s="438" t="n"/>
       <c r="H38" s="283" t="n"/>
       <c r="I38" s="438" t="n"/>
@@ -17135,11 +17129,11 @@
     <mergeCell ref="A42:A44"/>
     <mergeCell ref="C36:C38"/>
     <mergeCell ref="H57:H59"/>
+    <mergeCell ref="E36:E38"/>
     <mergeCell ref="A12:A14"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
     <mergeCell ref="G45:G47"/>
-    <mergeCell ref="G30:G32"/>
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
@@ -17163,7 +17157,6 @@
     <mergeCell ref="G57:G59"/>
     <mergeCell ref="A60:A62"/>
     <mergeCell ref="I57:I59"/>
-    <mergeCell ref="E24:E26"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
@@ -17180,7 +17173,6 @@
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="E9:E11"/>
     <mergeCell ref="C27:C29"/>
-    <mergeCell ref="E27:E29"/>
     <mergeCell ref="B15:B17"/>
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="D24:D26"/>
@@ -17217,6 +17209,7 @@
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="F42:F44"/>
+    <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
@@ -17236,6 +17229,7 @@
     <mergeCell ref="E54:E56"/>
     <mergeCell ref="I60:I62"/>
     <mergeCell ref="B54:B56"/>
+    <mergeCell ref="H12:H14"/>
     <mergeCell ref="D54:D56"/>
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="H48:H50"/>
@@ -17654,7 +17648,12 @@
 2º ao 7º tempos</t>
         </is>
       </c>
-      <c r="H12" s="435" t="n"/>
+      <c r="H12" s="409" t="inlineStr">
+        <is>
+          <t>Mat - ClaMe/JJ
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="I12" s="11" t="n"/>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
@@ -17670,7 +17669,7 @@
       <c r="E13" s="222" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="437" t="n"/>
-      <c r="H13" s="438" t="n"/>
+      <c r="H13" s="406" t="n"/>
       <c r="I13" s="222" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
@@ -17686,7 +17685,7 @@
       <c r="E14" s="222" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="439" t="n"/>
-      <c r="H14" s="438" t="n"/>
+      <c r="H14" s="407" t="n"/>
       <c r="I14" s="222" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
@@ -17712,7 +17711,12 @@
         <f>B15+4</f>
         <v/>
       </c>
-      <c r="E15" s="435" t="n"/>
+      <c r="E15" s="410" t="inlineStr">
+        <is>
+          <t>Geo - Mar
+2º e 3º tempos</t>
+        </is>
+      </c>
       <c r="F15" s="434" t="inlineStr">
         <is>
           <t>Hist - Ver
@@ -17737,7 +17741,7 @@
       <c r="B16" s="313" t="n"/>
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
-      <c r="E16" s="438" t="n"/>
+      <c r="E16" s="406" t="n"/>
       <c r="F16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
@@ -17752,7 +17756,7 @@
       <c r="B17" s="313" t="n"/>
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
-      <c r="E17" s="438" t="n"/>
+      <c r="E17" s="407" t="n"/>
       <c r="F17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
@@ -17950,12 +17954,7 @@
         <f>B24+4</f>
         <v/>
       </c>
-      <c r="E24" s="441" t="inlineStr">
-        <is>
-          <t>Mat - ClaMe/JJ
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="E24" s="441" t="n"/>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="459" t="inlineStr">
         <is>
@@ -17979,7 +17978,6 @@
       <c r="B25" s="313" t="n"/>
       <c r="C25" s="313" t="n"/>
       <c r="D25" s="350" t="n"/>
-      <c r="E25" s="437" t="n"/>
       <c r="F25" s="283" t="n"/>
       <c r="G25" s="447" t="n"/>
       <c r="H25" s="283" t="n"/>
@@ -17998,7 +17996,6 @@
       <c r="B26" s="313" t="n"/>
       <c r="C26" s="313" t="n"/>
       <c r="D26" s="350" t="n"/>
-      <c r="E26" s="439" t="n"/>
       <c r="F26" s="283" t="n"/>
       <c r="G26" s="448" t="n"/>
       <c r="H26" s="283" t="n"/>
@@ -18102,12 +18099,7 @@
       </c>
       <c r="E30" s="435" t="n"/>
       <c r="F30" s="283" t="n"/>
-      <c r="G30" s="442" t="inlineStr">
-        <is>
-          <t>Geo - Mar
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="G30" s="442" t="n"/>
       <c r="H30" s="283" t="n"/>
       <c r="I30" s="283" t="n"/>
       <c r="J30" s="183" t="inlineStr">
@@ -18130,7 +18122,6 @@
       <c r="D31" s="350" t="n"/>
       <c r="E31" s="438" t="n"/>
       <c r="F31" s="283" t="n"/>
-      <c r="G31" s="437" t="n"/>
       <c r="H31" s="283" t="n"/>
       <c r="I31" s="283" t="n"/>
       <c r="J31" s="315" t="n"/>
@@ -18149,7 +18140,6 @@
       <c r="D32" s="350" t="n"/>
       <c r="E32" s="438" t="n"/>
       <c r="F32" s="283" t="n"/>
-      <c r="G32" s="439" t="n"/>
       <c r="H32" s="283" t="n"/>
       <c r="I32" s="283" t="n"/>
       <c r="J32" s="315" t="n"/>
@@ -18850,7 +18840,6 @@
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="C12:C14"/>
     <mergeCell ref="G45:G47"/>
-    <mergeCell ref="G30:G32"/>
     <mergeCell ref="B33:B35"/>
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
@@ -18873,7 +18862,6 @@
     <mergeCell ref="G57:G59"/>
     <mergeCell ref="A60:A62"/>
     <mergeCell ref="I57:I59"/>
-    <mergeCell ref="E24:E26"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
@@ -18926,6 +18914,7 @@
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="F42:F44"/>
+    <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
@@ -18945,6 +18934,7 @@
     <mergeCell ref="E54:E56"/>
     <mergeCell ref="I60:I62"/>
     <mergeCell ref="B54:B56"/>
+    <mergeCell ref="H12:H14"/>
     <mergeCell ref="D54:D56"/>
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="H48:H50"/>

</xml_diff>

<commit_message>
10C: move Matematica (1a prova) para semana 7, antes da 1a segunda chamada
10C1/10C2: Mat semana 10 quarta (08/10) -> semana 7 segunda (14/09),
1o-2o tempos. A 1a ocorrencia de Matematica estava dentro da janela de
P2, deixando P1 sem nenhuma prova de Matematica antes da 1a segunda
chamada (19/09/2026, nao marcada no modelo). Testadas semanas 5 e 6
(invalidas: grupo 1 sem excecao de Ingles / teto semanal) antes de
confirmar semana 7. 2a ocorrencia (semana 15, 10/11) inalterada.

11C1/11C2: confirmada a permanencia de Matematica na semana 4 (27/08)
apos testar e reverter a alternativa de semana 6, que gerava 3
PROBLEMAS (grupo 1 repetido em ambas as turmas, alem do teto semanal
ja identificado no 11C2).

verificar_calendario.py: 0 PROBLEMA. 5 relatorios regenerados.
estado_2sem_2026.md atualizado com o racional das duas mudancas.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -12757,7 +12757,12 @@
         <f>B21+4</f>
         <v/>
       </c>
-      <c r="E21" s="435" t="n"/>
+      <c r="E21" s="441" t="inlineStr">
+        <is>
+          <t>Mat - BrSa/FBri
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="F21" s="62" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="452" t="inlineStr">
@@ -12789,7 +12794,7 @@
       <c r="B22" s="313" t="n"/>
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
-      <c r="E22" s="438" t="n"/>
+      <c r="E22" s="437" t="n"/>
       <c r="F22" s="63" t="n"/>
       <c r="G22" s="222" t="n"/>
       <c r="H22" s="437" t="n"/>
@@ -12804,7 +12809,7 @@
       <c r="B23" s="313" t="n"/>
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
-      <c r="E23" s="438" t="n"/>
+      <c r="E23" s="439" t="n"/>
       <c r="F23" s="63" t="n"/>
       <c r="G23" s="222" t="n"/>
       <c r="H23" s="439" t="n"/>
@@ -12984,12 +12989,7 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="H30" s="441" t="inlineStr">
-        <is>
-          <t>Mat - BrSa/FBri
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H30" s="441" t="n"/>
       <c r="I30" s="442" t="inlineStr">
         <is>
           <t>Geo - Mlo
@@ -13017,7 +13017,6 @@
       <c r="E31" s="283" t="n"/>
       <c r="F31" s="283" t="n"/>
       <c r="G31" s="437" t="n"/>
-      <c r="H31" s="437" t="n"/>
       <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
@@ -13036,7 +13035,6 @@
       <c r="E32" s="283" t="n"/>
       <c r="F32" s="283" t="n"/>
       <c r="G32" s="439" t="n"/>
-      <c r="H32" s="439" t="n"/>
       <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -13730,6 +13728,7 @@
     <mergeCell ref="H33:H35"/>
     <mergeCell ref="J33:J35"/>
     <mergeCell ref="H42:H44"/>
+    <mergeCell ref="E21:E23"/>
     <mergeCell ref="J42:J44"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="J60:J62"/>
@@ -13818,7 +13817,6 @@
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="F57:F59"/>
     <mergeCell ref="J21:J23"/>
-    <mergeCell ref="H30:H32"/>
     <mergeCell ref="J39:J41"/>
     <mergeCell ref="J51:J53"/>
     <mergeCell ref="C33:C35"/>
@@ -14450,7 +14448,12 @@
         <f>B21+4</f>
         <v/>
       </c>
-      <c r="E21" s="435" t="n"/>
+      <c r="E21" s="409" t="inlineStr">
+        <is>
+          <t>Mat - BrSa/FBri
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="F21" s="62" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="452" t="inlineStr">
@@ -14482,7 +14485,7 @@
       <c r="B22" s="313" t="n"/>
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
-      <c r="E22" s="438" t="n"/>
+      <c r="E22" s="406" t="n"/>
       <c r="F22" s="63" t="n"/>
       <c r="G22" s="222" t="n"/>
       <c r="H22" s="437" t="n"/>
@@ -14497,7 +14500,7 @@
       <c r="B23" s="313" t="n"/>
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
-      <c r="E23" s="438" t="n"/>
+      <c r="E23" s="407" t="n"/>
       <c r="F23" s="63" t="n"/>
       <c r="G23" s="222" t="n"/>
       <c r="H23" s="439" t="n"/>
@@ -14677,12 +14680,7 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="H30" s="441" t="inlineStr">
-        <is>
-          <t>Mat - BrSa/FBri
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H30" s="441" t="n"/>
       <c r="I30" s="442" t="inlineStr">
         <is>
           <t>Geo - Mlo
@@ -14710,7 +14708,6 @@
       <c r="E31" s="283" t="n"/>
       <c r="F31" s="283" t="n"/>
       <c r="G31" s="437" t="n"/>
-      <c r="H31" s="437" t="n"/>
       <c r="I31" s="437" t="n"/>
       <c r="J31" s="315" t="n"/>
       <c r="L31" s="27" t="n"/>
@@ -14729,7 +14726,6 @@
       <c r="E32" s="283" t="n"/>
       <c r="F32" s="283" t="n"/>
       <c r="G32" s="439" t="n"/>
-      <c r="H32" s="439" t="n"/>
       <c r="I32" s="439" t="n"/>
       <c r="J32" s="315" t="n"/>
       <c r="L32" s="28" t="n"/>
@@ -15432,6 +15428,7 @@
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
     <mergeCell ref="J33:J35"/>
+    <mergeCell ref="E21:E23"/>
     <mergeCell ref="J42:J44"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="J60:J62"/>
@@ -15519,7 +15516,6 @@
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="F57:F59"/>
     <mergeCell ref="J21:J23"/>
-    <mergeCell ref="H30:H32"/>
     <mergeCell ref="J39:J41"/>
     <mergeCell ref="J51:J53"/>
     <mergeCell ref="C33:C35"/>
@@ -17648,7 +17644,7 @@
 2º ao 7º tempos</t>
         </is>
       </c>
-      <c r="H12" s="409" t="inlineStr">
+      <c r="H12" s="441" t="inlineStr">
         <is>
           <t>Mat - ClaMe/JJ
 1º e 2º tempos</t>
@@ -17669,7 +17665,7 @@
       <c r="E13" s="222" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="437" t="n"/>
-      <c r="H13" s="406" t="n"/>
+      <c r="H13" s="437" t="n"/>
       <c r="I13" s="222" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
@@ -17685,7 +17681,7 @@
       <c r="E14" s="222" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="439" t="n"/>
-      <c r="H14" s="407" t="n"/>
+      <c r="H14" s="439" t="n"/>
       <c r="I14" s="222" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
@@ -17711,7 +17707,7 @@
         <f>B15+4</f>
         <v/>
       </c>
-      <c r="E15" s="410" t="inlineStr">
+      <c r="E15" s="442" t="inlineStr">
         <is>
           <t>Geo - Mar
 2º e 3º tempos</t>
@@ -17741,7 +17737,7 @@
       <c r="B16" s="313" t="n"/>
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
-      <c r="E16" s="406" t="n"/>
+      <c r="E16" s="437" t="n"/>
       <c r="F16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
@@ -17756,7 +17752,7 @@
       <c r="B17" s="313" t="n"/>
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
-      <c r="E17" s="407" t="n"/>
+      <c r="E17" s="439" t="n"/>
       <c r="F17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>

</xml_diff>

<commit_message>
11C1/11C2: Matematica para semana 6 (10/09), excecao explicita ao grupo 1
Matematica (11C1+11C2): semana 4 quinta (27/08) -> semana 6 quinta
(10/09), mesmo bloco 1o-2o tempos, a pedido explicito do usuario mesmo
sabendo que viola a regra do grupo 1 (Mat+DaF sem Ingles na mesma
semana).

Ingles (11C2 apenas): semana 6 sexta (11/09) -> semana 4 sexta
(28/08), mesmo bloco 6o-7o tempos, para resolver o teto de 3
avaliacoes/semana do 11C2 (sem essa troca a semana 6 teria 4
avaliacoes no 11C2).

verificar_calendario.py fecha com 2 PROBLEMA(S) esperados e
autorizados pelo usuario (grupo 1 repetido ['DaF','Mat'] em 11C1 e
11C2) -- documentado em estado_2sem_2026.md como excecao explicita,
nao um erro de geracao. 5 relatorios regenerados.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -14448,7 +14448,7 @@
         <f>B21+4</f>
         <v/>
       </c>
-      <c r="E21" s="409" t="inlineStr">
+      <c r="E21" s="441" t="inlineStr">
         <is>
           <t>Mat - BrSa/FBri
 1º e 2º tempos</t>
@@ -14485,7 +14485,7 @@
       <c r="B22" s="313" t="n"/>
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
-      <c r="E22" s="406" t="n"/>
+      <c r="E22" s="437" t="n"/>
       <c r="F22" s="63" t="n"/>
       <c r="G22" s="222" t="n"/>
       <c r="H22" s="437" t="n"/>
@@ -14500,7 +14500,7 @@
       <c r="B23" s="313" t="n"/>
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
-      <c r="E23" s="407" t="n"/>
+      <c r="E23" s="439" t="n"/>
       <c r="F23" s="63" t="n"/>
       <c r="G23" s="222" t="n"/>
       <c r="H23" s="439" t="n"/>
@@ -15945,12 +15945,7 @@
 2º ao 7º tempos</t>
         </is>
       </c>
-      <c r="H12" s="441" t="inlineStr">
-        <is>
-          <t>Mat - ClaMe/JJ
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="H12" s="441" t="n"/>
       <c r="I12" s="11" t="n"/>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
@@ -15966,7 +15961,6 @@
       <c r="E13" s="437" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="437" t="n"/>
-      <c r="H13" s="437" t="n"/>
       <c r="I13" s="222" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
@@ -15982,7 +15976,6 @@
       <c r="E14" s="439" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="439" t="n"/>
-      <c r="H14" s="439" t="n"/>
       <c r="I14" s="222" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
@@ -16097,7 +16090,12 @@
 6º e 7º tempos</t>
         </is>
       </c>
-      <c r="H18" s="11" t="n"/>
+      <c r="H18" s="441" t="inlineStr">
+        <is>
+          <t>Mat - ClaMe/JJ
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="I18" s="382" t="n"/>
       <c r="J18" s="183" t="n"/>
       <c r="L18" s="17" t="n"/>
@@ -16112,7 +16110,7 @@
       <c r="E19" s="315" t="n"/>
       <c r="F19" s="437" t="n"/>
       <c r="G19" s="437" t="n"/>
-      <c r="H19" s="222" t="n"/>
+      <c r="H19" s="437" t="n"/>
       <c r="I19" s="383" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
@@ -16135,7 +16133,7 @@
       <c r="E20" s="315" t="n"/>
       <c r="F20" s="439" t="n"/>
       <c r="G20" s="439" t="n"/>
-      <c r="H20" s="222" t="n"/>
+      <c r="H20" s="439" t="n"/>
       <c r="I20" s="384" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
@@ -17134,6 +17132,7 @@
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
+    <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
     <mergeCell ref="E12:E14"/>
@@ -17225,7 +17224,6 @@
     <mergeCell ref="E54:E56"/>
     <mergeCell ref="I60:I62"/>
     <mergeCell ref="B54:B56"/>
-    <mergeCell ref="H12:H14"/>
     <mergeCell ref="D54:D56"/>
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="H48:H50"/>
@@ -17644,13 +17642,13 @@
 2º ao 7º tempos</t>
         </is>
       </c>
-      <c r="H12" s="441" t="inlineStr">
-        <is>
-          <t>Mat - ClaMe/JJ
-1º e 2º tempos</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="n"/>
+      <c r="H12" s="441" t="n"/>
+      <c r="I12" s="408" t="inlineStr">
+        <is>
+          <t>Ing - PaH
+6º e 7º tempos</t>
+        </is>
+      </c>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
       <c r="M12" s="15" t="n"/>
@@ -17665,8 +17663,7 @@
       <c r="E13" s="222" t="n"/>
       <c r="F13" s="437" t="n"/>
       <c r="G13" s="437" t="n"/>
-      <c r="H13" s="437" t="n"/>
-      <c r="I13" s="222" t="n"/>
+      <c r="I13" s="406" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
@@ -17681,8 +17678,7 @@
       <c r="E14" s="222" t="n"/>
       <c r="F14" s="439" t="n"/>
       <c r="G14" s="439" t="n"/>
-      <c r="H14" s="439" t="n"/>
-      <c r="I14" s="222" t="n"/>
+      <c r="I14" s="407" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
@@ -17796,13 +17792,13 @@
 6º e 7º tempos</t>
         </is>
       </c>
-      <c r="H18" s="11" t="n"/>
-      <c r="I18" s="431" t="inlineStr">
-        <is>
-          <t>Ing - PaH
-6º e 7º tempos</t>
-        </is>
-      </c>
+      <c r="H18" s="441" t="inlineStr">
+        <is>
+          <t>Mat - ClaMe/JJ
+1º e 2º tempos</t>
+        </is>
+      </c>
+      <c r="I18" s="431" t="n"/>
       <c r="J18" s="183" t="n"/>
       <c r="L18" s="17" t="n"/>
       <c r="M18" s="15" t="n"/>
@@ -17816,8 +17812,7 @@
       <c r="E19" s="315" t="n"/>
       <c r="F19" s="437" t="n"/>
       <c r="G19" s="437" t="n"/>
-      <c r="H19" s="222" t="n"/>
-      <c r="I19" s="383" t="n"/>
+      <c r="H19" s="437" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
         <is>
@@ -17839,8 +17834,7 @@
       <c r="E20" s="315" t="n"/>
       <c r="F20" s="439" t="n"/>
       <c r="G20" s="439" t="n"/>
-      <c r="H20" s="222" t="n"/>
-      <c r="I20" s="384" t="n"/>
+      <c r="H20" s="439" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
       <c r="M20" s="29" t="n"/>
@@ -18840,6 +18834,7 @@
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
+    <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
     <mergeCell ref="J33:J35"/>
@@ -18918,7 +18913,6 @@
     <mergeCell ref="A27:A29"/>
     <mergeCell ref="G18:G20"/>
     <mergeCell ref="G24:G26"/>
-    <mergeCell ref="I18:I20"/>
     <mergeCell ref="D15:D17"/>
     <mergeCell ref="C57:C59"/>
     <mergeCell ref="D12:D14"/>
@@ -18930,7 +18924,6 @@
     <mergeCell ref="E54:E56"/>
     <mergeCell ref="I60:I62"/>
     <mergeCell ref="B54:B56"/>
-    <mergeCell ref="H12:H14"/>
     <mergeCell ref="D54:D56"/>
     <mergeCell ref="J12:J14"/>
     <mergeCell ref="H48:H50"/>
@@ -18951,6 +18944,7 @@
     <mergeCell ref="M28:N28"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B18:B20"/>
+    <mergeCell ref="I12:I14"/>
     <mergeCell ref="B60:B62"/>
     <mergeCell ref="B9:B11"/>
     <mergeCell ref="F33:F35"/>

</xml_diff>

<commit_message>
11C: Historia (1a prova) para quarta (02/09); skill: evitar Qui/Fis como doadoras
Historia (11C1+11C2): semana5 terca (01/09) -> semana5 quarta (02/09),
mesmo bloco 1-2 tempos. Troca os doadores de Mat/JJ+Qui/CAl (11C2) por
Mat/ClaMe (11C1) + Geo/Mar (11C2) -- a pedido do usuario, para evitar
usar Quimica como doadora, mesmo isso nao sendo uma melhora estrita no
numero de avisos (troca lateral, ver estado_2sem_2026.md).

verificar_calendario.py fecha so com os 2 PROBLEMA ja autorizados do
11C (grupo 1). 5 relatorios regenerados.

Skill (calendario-provas/SKILL.md): novo criterio de preferencia
documentado -- evitar usar tempos de Quimica e Fisica como doadores
quando houver alternativa igualmente valida nas demais regras. Nao e
regra absoluta; se a unica opcao viavel exigir esse doador, aceitar
normalmente.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -14299,7 +14299,7 @@
       </c>
       <c r="G15" s="11" t="n"/>
       <c r="H15" s="435" t="n"/>
-      <c r="I15" s="419" t="inlineStr">
+      <c r="I15" s="451" t="inlineStr">
         <is>
           <t>Qui - CAl
 3º e 4º tempos</t>
@@ -14319,7 +14319,7 @@
       <c r="F16" s="437" t="n"/>
       <c r="G16" s="222" t="n"/>
       <c r="H16" s="438" t="n"/>
-      <c r="I16" s="406" t="n"/>
+      <c r="I16" s="437" t="n"/>
       <c r="J16" s="315" t="n"/>
       <c r="L16" s="141" t="n"/>
       <c r="M16" s="317" t="n"/>
@@ -14335,7 +14335,7 @@
       <c r="F17" s="439" t="n"/>
       <c r="G17" s="222" t="n"/>
       <c r="H17" s="438" t="n"/>
-      <c r="I17" s="407" t="n"/>
+      <c r="I17" s="439" t="n"/>
       <c r="J17" s="315" t="n"/>
       <c r="L17" s="317" t="n"/>
       <c r="M17" s="317" t="n"/>
@@ -16003,13 +16003,13 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="F15" s="434" t="inlineStr">
+      <c r="F15" s="434" t="n"/>
+      <c r="G15" s="470" t="inlineStr">
         <is>
           <t>Hist - Ver
-2º e 3º tempos</t>
-        </is>
-      </c>
-      <c r="G15" s="434" t="n"/>
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -16028,7 +16028,7 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="F16" s="437" t="n"/>
+      <c r="G16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -16043,7 +16043,7 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="F17" s="439" t="n"/>
+      <c r="G17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -17104,7 +17104,6 @@
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="D21:D23"/>
     <mergeCell ref="E60:E62"/>
-    <mergeCell ref="F15:F17"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
@@ -17202,6 +17201,7 @@
     <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
+    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
@@ -17705,13 +17705,13 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="F15" s="434" t="inlineStr">
+      <c r="F15" s="434" t="n"/>
+      <c r="G15" s="468" t="inlineStr">
         <is>
           <t>Hist - Ver
-2º e 3º tempos</t>
-        </is>
-      </c>
-      <c r="G15" s="434" t="n"/>
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -17730,7 +17730,7 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="F16" s="437" t="n"/>
+      <c r="G16" s="406" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -17745,7 +17745,7 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="F17" s="439" t="n"/>
+      <c r="G17" s="407" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -18806,7 +18806,6 @@
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="D21:D23"/>
     <mergeCell ref="E60:E62"/>
-    <mergeCell ref="F15:F17"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
@@ -18903,6 +18902,7 @@
     <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
+    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>

</xml_diff>

<commit_message>
11C: Historia (1a prova) para quarta (02/09); skill: evitar Qui/Fis como doadoras (#52)
Historia (11C1+11C2): semana5 terca (01/09) -> semana5 quarta (02/09),
mesmo bloco 1-2 tempos. Troca os doadores de Mat/JJ+Qui/CAl (11C2) por
Mat/ClaMe (11C1) + Geo/Mar (11C2) -- a pedido do usuario, para evitar
usar Quimica como doadora, mesmo isso nao sendo uma melhora estrita no
numero de avisos (troca lateral, ver estado_2sem_2026.md).

verificar_calendario.py fecha so com os 2 PROBLEMA ja autorizados do
11C (grupo 1). 5 relatorios regenerados.

Skill (calendario-provas/SKILL.md): novo criterio de preferencia
documentado -- evitar usar tempos de Quimica e Fisica como doadores
quando houver alternativa igualmente valida nas demais regras. Nao e
regra absoluta; se a unica opcao viavel exigir esse doador, aceitar
normalmente.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -14299,7 +14299,7 @@
       </c>
       <c r="G15" s="11" t="n"/>
       <c r="H15" s="435" t="n"/>
-      <c r="I15" s="419" t="inlineStr">
+      <c r="I15" s="451" t="inlineStr">
         <is>
           <t>Qui - CAl
 3º e 4º tempos</t>
@@ -14319,7 +14319,7 @@
       <c r="F16" s="437" t="n"/>
       <c r="G16" s="222" t="n"/>
       <c r="H16" s="438" t="n"/>
-      <c r="I16" s="406" t="n"/>
+      <c r="I16" s="437" t="n"/>
       <c r="J16" s="315" t="n"/>
       <c r="L16" s="141" t="n"/>
       <c r="M16" s="317" t="n"/>
@@ -14335,7 +14335,7 @@
       <c r="F17" s="439" t="n"/>
       <c r="G17" s="222" t="n"/>
       <c r="H17" s="438" t="n"/>
-      <c r="I17" s="407" t="n"/>
+      <c r="I17" s="439" t="n"/>
       <c r="J17" s="315" t="n"/>
       <c r="L17" s="317" t="n"/>
       <c r="M17" s="317" t="n"/>
@@ -16003,13 +16003,13 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="F15" s="434" t="inlineStr">
+      <c r="F15" s="434" t="n"/>
+      <c r="G15" s="470" t="inlineStr">
         <is>
           <t>Hist - Ver
-2º e 3º tempos</t>
-        </is>
-      </c>
-      <c r="G15" s="434" t="n"/>
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -16028,7 +16028,7 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="F16" s="437" t="n"/>
+      <c r="G16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -16043,7 +16043,7 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="F17" s="439" t="n"/>
+      <c r="G17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -17104,7 +17104,6 @@
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="D21:D23"/>
     <mergeCell ref="E60:E62"/>
-    <mergeCell ref="F15:F17"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
@@ -17202,6 +17201,7 @@
     <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
+    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
@@ -17705,13 +17705,13 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="F15" s="434" t="inlineStr">
+      <c r="F15" s="434" t="n"/>
+      <c r="G15" s="468" t="inlineStr">
         <is>
           <t>Hist - Ver
-2º e 3º tempos</t>
-        </is>
-      </c>
-      <c r="G15" s="434" t="n"/>
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -17730,7 +17730,7 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="F16" s="437" t="n"/>
+      <c r="G16" s="406" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -17745,7 +17745,7 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="F17" s="439" t="n"/>
+      <c r="G17" s="407" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -18806,7 +18806,6 @@
     <mergeCell ref="B21:B23"/>
     <mergeCell ref="D21:D23"/>
     <mergeCell ref="E60:E62"/>
-    <mergeCell ref="F15:F17"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
@@ -18903,6 +18902,7 @@
     <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
+    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>

</xml_diff>

<commit_message>
10C: remove 1a prova de GL (26/08), sem substituicao -- excecao pontual
GL (10C1+10C2): celula de semana4 quarta (26/08) esvaziada, nada
recolocado. GL passa a ter so 1 prova no semestre (07/10, mantida).
Confirmado com o usuario antes de aplicar (AskUserQuestion).

verificar_calendario.py acusa 2 PROBLEMA novos, esperados e
autorizados: "GL tem 1 provas (esperado 2)" em 10C1 e 10C2.

Pedido explicito do usuario: NAO registrar como regra geral na skill
-- e mudanca excepcional deste semestre, documentada so em
estado_2sem_2026.md. calendario-provas/SKILL.md nao foi alterado.

5 relatorios regenerados.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -12538,12 +12538,7 @@
 6º e 7º tempos</t>
         </is>
       </c>
-      <c r="G12" s="436" t="inlineStr">
-        <is>
-          <t>GL - EFr-Car-Swa
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="G12" s="436" t="n"/>
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="451" t="n"/>
       <c r="J12" s="183" t="n"/>
@@ -12558,7 +12553,6 @@
       <c r="C13" s="313" t="n"/>
       <c r="D13" s="314" t="n"/>
       <c r="F13" s="437" t="n"/>
-      <c r="G13" s="437" t="n"/>
       <c r="H13" s="222" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
@@ -12572,7 +12566,6 @@
       <c r="C14" s="313" t="n"/>
       <c r="D14" s="314" t="n"/>
       <c r="F14" s="439" t="n"/>
-      <c r="G14" s="439" t="n"/>
       <c r="H14" s="222" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
@@ -13670,7 +13663,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="168">
+  <mergeCells count="167">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -13776,7 +13769,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G12:G14"/>
     <mergeCell ref="E39:E41"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
@@ -14225,12 +14217,7 @@
 6º e 7º tempos</t>
         </is>
       </c>
-      <c r="G12" s="436" t="inlineStr">
-        <is>
-          <t>GL - EFr-Car-Swa
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="G12" s="436" t="n"/>
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="451" t="n"/>
       <c r="J12" s="183" t="n"/>
@@ -14245,7 +14232,6 @@
       <c r="C13" s="313" t="n"/>
       <c r="D13" s="314" t="n"/>
       <c r="F13" s="437" t="n"/>
-      <c r="G13" s="437" t="n"/>
       <c r="H13" s="222" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
@@ -14259,7 +14245,6 @@
       <c r="C14" s="313" t="n"/>
       <c r="D14" s="314" t="n"/>
       <c r="F14" s="439" t="n"/>
-      <c r="G14" s="439" t="n"/>
       <c r="H14" s="222" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
@@ -15367,7 +15352,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="168">
+  <mergeCells count="167">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -15473,7 +15458,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G12:G14"/>
     <mergeCell ref="E39:E41"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
@@ -17706,7 +17690,7 @@
         </is>
       </c>
       <c r="F15" s="434" t="n"/>
-      <c r="G15" s="468" t="inlineStr">
+      <c r="G15" s="470" t="inlineStr">
         <is>
           <t>Hist - Ver
 1º e 2º tempos</t>
@@ -17730,7 +17714,7 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="G16" s="406" t="n"/>
+      <c r="G16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -17745,7 +17729,7 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="G17" s="407" t="n"/>
+      <c r="G17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>

</xml_diff>

<commit_message>
10C: remove 1a prova de GL (26/08), sem substituicao -- excecao pontual (#53)
GL (10C1+10C2): celula de semana4 quarta (26/08) esvaziada, nada
recolocado. GL passa a ter so 1 prova no semestre (07/10, mantida).
Confirmado com o usuario antes de aplicar (AskUserQuestion).

verificar_calendario.py acusa 2 PROBLEMA novos, esperados e
autorizados: "GL tem 1 provas (esperado 2)" em 10C1 e 10C2.

Pedido explicito do usuario: NAO registrar como regra geral na skill
-- e mudanca excepcional deste semestre, documentada so em
estado_2sem_2026.md. calendario-provas/SKILL.md nao foi alterado.

5 relatorios regenerados.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -12538,12 +12538,7 @@
 6º e 7º tempos</t>
         </is>
       </c>
-      <c r="G12" s="436" t="inlineStr">
-        <is>
-          <t>GL - EFr-Car-Swa
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="G12" s="436" t="n"/>
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="451" t="n"/>
       <c r="J12" s="183" t="n"/>
@@ -12558,7 +12553,6 @@
       <c r="C13" s="313" t="n"/>
       <c r="D13" s="314" t="n"/>
       <c r="F13" s="437" t="n"/>
-      <c r="G13" s="437" t="n"/>
       <c r="H13" s="222" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
@@ -12572,7 +12566,6 @@
       <c r="C14" s="313" t="n"/>
       <c r="D14" s="314" t="n"/>
       <c r="F14" s="439" t="n"/>
-      <c r="G14" s="439" t="n"/>
       <c r="H14" s="222" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
@@ -13670,7 +13663,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="168">
+  <mergeCells count="167">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -13776,7 +13769,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G12:G14"/>
     <mergeCell ref="E39:E41"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
@@ -14225,12 +14217,7 @@
 6º e 7º tempos</t>
         </is>
       </c>
-      <c r="G12" s="436" t="inlineStr">
-        <is>
-          <t>GL - EFr-Car-Swa
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="G12" s="436" t="n"/>
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="451" t="n"/>
       <c r="J12" s="183" t="n"/>
@@ -14245,7 +14232,6 @@
       <c r="C13" s="313" t="n"/>
       <c r="D13" s="314" t="n"/>
       <c r="F13" s="437" t="n"/>
-      <c r="G13" s="437" t="n"/>
       <c r="H13" s="222" t="n"/>
       <c r="J13" s="315" t="n"/>
       <c r="L13" s="15" t="n"/>
@@ -14259,7 +14245,6 @@
       <c r="C14" s="313" t="n"/>
       <c r="D14" s="314" t="n"/>
       <c r="F14" s="439" t="n"/>
-      <c r="G14" s="439" t="n"/>
       <c r="H14" s="222" t="n"/>
       <c r="J14" s="315" t="n"/>
       <c r="L14" s="15" t="n"/>
@@ -15367,7 +15352,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="168">
+  <mergeCells count="167">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -15473,7 +15458,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G12:G14"/>
     <mergeCell ref="E39:E41"/>
     <mergeCell ref="G39:G41"/>
     <mergeCell ref="D27:D29"/>
@@ -17706,7 +17690,7 @@
         </is>
       </c>
       <c r="F15" s="434" t="n"/>
-      <c r="G15" s="468" t="inlineStr">
+      <c r="G15" s="470" t="inlineStr">
         <is>
           <t>Hist - Ver
 1º e 2º tempos</t>
@@ -17730,7 +17714,7 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="G16" s="406" t="n"/>
+      <c r="G16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -17745,7 +17729,7 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="G17" s="407" t="n"/>
+      <c r="G17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>

</xml_diff>

<commit_message>
11C: Quimica para 15/09 e GL para semana 8, em cadeia
Quimica (11C1+11C2): semana6 terca (08/09) -> semana7 terca (15/09),
mesmo bloco 2o-3o tempos.

GL (11C1+11C2): semana7 quarta (16/09) -> semana8 segunda (21/09),
tempos 4o-5o (doadores Redacao/ACo no 11C1, Ingles/PaH no 11C2 --
nenhum Quimica/Fisica). Necessario porque a Quimica ocuparia a 4a
avaliacao da semana 7, que ja tinha 3 (Bio, GL, Fis).

Analise apresentada e aprovada antes de aplicar. Distancia entre as 2
ocorrencias de GL: 7 semanas (piso desejavel). verificar_calendario.py
fecha so com os 4 PROBLEMA ja conhecidos e autorizados -- nenhum novo,
nem aviso novo. 5 relatorios regenerados.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -16058,12 +16058,7 @@
           <t>unterrichtsfrei sem aula</t>
         </is>
       </c>
-      <c r="F18" s="451" t="inlineStr">
-        <is>
-          <t>Qui - CAl
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="F18" s="451" t="n"/>
       <c r="G18" s="443" t="inlineStr">
         <is>
           <t>DaF - CBu-SGa-Swa
@@ -16088,7 +16083,6 @@
       <c r="C19" s="313" t="n"/>
       <c r="D19" s="314" t="n"/>
       <c r="E19" s="315" t="n"/>
-      <c r="F19" s="437" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="437" t="n"/>
       <c r="I19" s="383" t="n"/>
@@ -16111,7 +16105,6 @@
       <c r="C20" s="313" t="n"/>
       <c r="D20" s="314" t="n"/>
       <c r="E20" s="315" t="n"/>
-      <c r="F20" s="439" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="439" t="n"/>
       <c r="I20" s="384" t="n"/>
@@ -16144,13 +16137,13 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="F21" s="62" t="n"/>
-      <c r="G21" s="436" t="inlineStr">
-        <is>
-          <t>GL - CBu-Swa-SGa
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="F21" s="451" t="inlineStr">
+        <is>
+          <t>Qui - CAl
+2º e 3º tempos</t>
+        </is>
+      </c>
+      <c r="G21" s="436" t="n"/>
       <c r="H21" s="452" t="inlineStr">
         <is>
           <t>Fis - Cadu
@@ -16181,8 +16174,7 @@
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="437" t="n"/>
-      <c r="F22" s="63" t="n"/>
-      <c r="G22" s="437" t="n"/>
+      <c r="F22" s="437" t="n"/>
       <c r="H22" s="437" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
@@ -16196,8 +16188,7 @@
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="439" t="n"/>
-      <c r="F23" s="63" t="n"/>
-      <c r="G23" s="439" t="n"/>
+      <c r="F23" s="439" t="n"/>
       <c r="H23" s="439" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
@@ -16224,7 +16215,12 @@
         <f>B24+4</f>
         <v/>
       </c>
-      <c r="E24" s="441" t="n"/>
+      <c r="E24" s="436" t="inlineStr">
+        <is>
+          <t>GL - CBu-Swa-SGa
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="459" t="inlineStr">
         <is>
@@ -16248,6 +16244,7 @@
       <c r="B25" s="313" t="n"/>
       <c r="C25" s="313" t="n"/>
       <c r="D25" s="350" t="n"/>
+      <c r="E25" s="437" t="n"/>
       <c r="F25" s="283" t="n"/>
       <c r="G25" s="447" t="n"/>
       <c r="H25" s="283" t="n"/>
@@ -16266,6 +16263,7 @@
       <c r="B26" s="313" t="n"/>
       <c r="C26" s="313" t="n"/>
       <c r="D26" s="350" t="n"/>
+      <c r="E26" s="439" t="n"/>
       <c r="F26" s="283" t="n"/>
       <c r="G26" s="448" t="n"/>
       <c r="H26" s="283" t="n"/>
@@ -17091,6 +17089,7 @@
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
+    <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
     <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
@@ -17131,6 +17130,7 @@
     <mergeCell ref="G57:G59"/>
     <mergeCell ref="A60:A62"/>
     <mergeCell ref="I57:I59"/>
+    <mergeCell ref="E24:E26"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
@@ -17168,7 +17168,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G21:G23"/>
     <mergeCell ref="G12:G14"/>
     <mergeCell ref="E39:E41"/>
     <mergeCell ref="G39:G41"/>
@@ -17178,7 +17177,6 @@
     <mergeCell ref="M26:N26"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
-    <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
@@ -17760,12 +17758,7 @@
           <t>unterrichtsfrei sem aula</t>
         </is>
       </c>
-      <c r="F18" s="451" t="inlineStr">
-        <is>
-          <t>Qui - CAl
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="F18" s="451" t="n"/>
       <c r="G18" s="443" t="inlineStr">
         <is>
           <t>DaF - CBu-SGa-Swa
@@ -17790,7 +17783,6 @@
       <c r="C19" s="313" t="n"/>
       <c r="D19" s="314" t="n"/>
       <c r="E19" s="315" t="n"/>
-      <c r="F19" s="437" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="437" t="n"/>
       <c r="J19" s="315" t="n"/>
@@ -17812,7 +17804,6 @@
       <c r="C20" s="313" t="n"/>
       <c r="D20" s="314" t="n"/>
       <c r="E20" s="315" t="n"/>
-      <c r="F20" s="439" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="439" t="n"/>
       <c r="J20" s="315" t="n"/>
@@ -17844,13 +17835,13 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="F21" s="62" t="n"/>
-      <c r="G21" s="436" t="inlineStr">
-        <is>
-          <t>GL - CBu-Swa-SGa
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="F21" s="419" t="inlineStr">
+        <is>
+          <t>Qui - CAl
+2º e 3º tempos</t>
+        </is>
+      </c>
+      <c r="G21" s="436" t="n"/>
       <c r="H21" s="452" t="inlineStr">
         <is>
           <t>Fis - Cadu
@@ -17881,8 +17872,7 @@
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="437" t="n"/>
-      <c r="F22" s="63" t="n"/>
-      <c r="G22" s="437" t="n"/>
+      <c r="F22" s="406" t="n"/>
       <c r="H22" s="437" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
@@ -17896,8 +17886,7 @@
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="439" t="n"/>
-      <c r="F23" s="63" t="n"/>
-      <c r="G23" s="439" t="n"/>
+      <c r="F23" s="407" t="n"/>
       <c r="H23" s="439" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
@@ -17924,7 +17913,12 @@
         <f>B24+4</f>
         <v/>
       </c>
-      <c r="E24" s="441" t="n"/>
+      <c r="E24" s="405" t="inlineStr">
+        <is>
+          <t>GL - CBu-Swa-SGa
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="459" t="inlineStr">
         <is>
@@ -17948,6 +17942,7 @@
       <c r="B25" s="313" t="n"/>
       <c r="C25" s="313" t="n"/>
       <c r="D25" s="350" t="n"/>
+      <c r="E25" s="406" t="n"/>
       <c r="F25" s="283" t="n"/>
       <c r="G25" s="447" t="n"/>
       <c r="H25" s="283" t="n"/>
@@ -17966,6 +17961,7 @@
       <c r="B26" s="313" t="n"/>
       <c r="C26" s="313" t="n"/>
       <c r="D26" s="350" t="n"/>
+      <c r="E26" s="407" t="n"/>
       <c r="F26" s="283" t="n"/>
       <c r="G26" s="448" t="n"/>
       <c r="H26" s="283" t="n"/>
@@ -18793,6 +18789,7 @@
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="B57:B59"/>
+    <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
     <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
@@ -18832,6 +18829,7 @@
     <mergeCell ref="G57:G59"/>
     <mergeCell ref="A60:A62"/>
     <mergeCell ref="I57:I59"/>
+    <mergeCell ref="E24:E26"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="A54:A56"/>
@@ -18869,7 +18867,6 @@
     <mergeCell ref="I54:I56"/>
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="C45:C47"/>
-    <mergeCell ref="G21:G23"/>
     <mergeCell ref="G12:G14"/>
     <mergeCell ref="E39:E41"/>
     <mergeCell ref="G39:G41"/>
@@ -18879,7 +18876,6 @@
     <mergeCell ref="M26:N26"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
-    <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>

</xml_diff>

<commit_message>
9C: DaF volta a ter 1a prova, 24/09 (aula dupla real, zero doador)
Reverte parcialmente a excecao "1 prova so" de 13/08 (commit
c85173f): DaF removida de UMA_PROVA_POR_TURMA (9C1/9C2) em
gerar_calendario.py -- GL continua com 1 prova so, DaF volta ao padrao
normal de 2 ocorrencias.

DaF (9C1+9C2): nova 1a prova em semana8 quinta (24/09), tempos 1o-2o
-- aula dupla real nas duas turmas, sem nenhum doador. Preferida sobre
a data inicialmente sugerida pelo usuario (22/09, terca), que exigiria
tomar tempo de Portugues/Jana no 9C1 (ja acima do teto de cessao).
2a prova (semana13, 27/10) inalterada.

verificar_calendario.py fecha so com os 4 PROBLEMA ja conhecidos e
autorizados -- nenhum novo. 1 AVISO leve novo (DaF cede na semana 7,
vespera da propria prova na semana 8 -- cessao pre-existente que virou
vespera com a prova nova). Distancia entre as 2 provas de DaF: 5
semanas (acima do piso minimo de 4).

5 relatorios regenerados.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -9494,7 +9494,12 @@
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="438" t="n"/>
-      <c r="H24" s="283" t="n"/>
+      <c r="H24" s="443" t="inlineStr">
+        <is>
+          <t>DaF - Caro-SGa-EFr
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="I24" s="446" t="n"/>
       <c r="J24" s="265" t="n"/>
       <c r="L24" s="318" t="inlineStr">
@@ -9513,7 +9518,7 @@
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
       <c r="G25" s="438" t="n"/>
-      <c r="H25" s="283" t="n"/>
+      <c r="H25" s="437" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
       <c r="M25" s="321" t="inlineStr">
@@ -9531,7 +9536,7 @@
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
       <c r="G26" s="438" t="n"/>
-      <c r="H26" s="283" t="n"/>
+      <c r="H26" s="439" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
       <c r="M26" s="323" t="inlineStr">
@@ -10314,7 +10319,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="165">
+  <mergeCells count="166">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -10411,6 +10416,7 @@
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="H15:H17"/>
     <mergeCell ref="D60:D62"/>
+    <mergeCell ref="H24:H26"/>
     <mergeCell ref="F60:F62"/>
     <mergeCell ref="M31:N31"/>
     <mergeCell ref="A36:A38"/>
@@ -11166,7 +11172,12 @@
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="438" t="n"/>
-      <c r="H24" s="283" t="n"/>
+      <c r="H24" s="411" t="inlineStr">
+        <is>
+          <t>DaF - Caro-SGa-EFr
+1º e 2º tempos</t>
+        </is>
+      </c>
       <c r="I24" s="446" t="n"/>
       <c r="J24" s="265" t="n"/>
       <c r="L24" s="318" t="inlineStr">
@@ -11185,7 +11196,7 @@
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
       <c r="G25" s="438" t="n"/>
-      <c r="H25" s="283" t="n"/>
+      <c r="H25" s="406" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
       <c r="M25" s="321" t="inlineStr">
@@ -11203,7 +11214,7 @@
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
       <c r="G26" s="438" t="n"/>
-      <c r="H26" s="283" t="n"/>
+      <c r="H26" s="407" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
       <c r="M26" s="323" t="inlineStr">
@@ -11986,7 +11997,7 @@
       <c r="J62" s="353" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="165">
+  <mergeCells count="166">
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="G54:G56"/>
     <mergeCell ref="C21:C23"/>
@@ -12083,6 +12094,7 @@
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="H15:H17"/>
     <mergeCell ref="D60:D62"/>
+    <mergeCell ref="H24:H26"/>
     <mergeCell ref="F60:F62"/>
     <mergeCell ref="M31:N31"/>
     <mergeCell ref="A36:A38"/>
@@ -17835,7 +17847,7 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="F21" s="419" t="inlineStr">
+      <c r="F21" s="451" t="inlineStr">
         <is>
           <t>Qui - CAl
 2º e 3º tempos</t>
@@ -17872,7 +17884,7 @@
       <c r="C22" s="313" t="n"/>
       <c r="D22" s="314" t="n"/>
       <c r="E22" s="437" t="n"/>
-      <c r="F22" s="406" t="n"/>
+      <c r="F22" s="437" t="n"/>
       <c r="H22" s="437" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
@@ -17886,7 +17898,7 @@
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="314" t="n"/>
       <c r="E23" s="439" t="n"/>
-      <c r="F23" s="407" t="n"/>
+      <c r="F23" s="439" t="n"/>
       <c r="H23" s="439" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
@@ -17913,7 +17925,7 @@
         <f>B24+4</f>
         <v/>
       </c>
-      <c r="E24" s="405" t="inlineStr">
+      <c r="E24" s="436" t="inlineStr">
         <is>
           <t>GL - CBu-Swa-SGa
 4º e 5º tempos</t>
@@ -17942,7 +17954,7 @@
       <c r="B25" s="313" t="n"/>
       <c r="C25" s="313" t="n"/>
       <c r="D25" s="350" t="n"/>
-      <c r="E25" s="406" t="n"/>
+      <c r="E25" s="437" t="n"/>
       <c r="F25" s="283" t="n"/>
       <c r="G25" s="447" t="n"/>
       <c r="H25" s="283" t="n"/>
@@ -17961,7 +17973,7 @@
       <c r="B26" s="313" t="n"/>
       <c r="C26" s="313" t="n"/>
       <c r="D26" s="350" t="n"/>
-      <c r="E26" s="407" t="n"/>
+      <c r="E26" s="439" t="n"/>
       <c r="F26" s="283" t="n"/>
       <c r="G26" s="448" t="n"/>
       <c r="H26" s="283" t="n"/>

</xml_diff>

<commit_message>
12C: Matematica (1a prova) para 17/09, excecao autorizada ao grupo 1
Matematica (12C1+12C2): semana6 quinta (10/09) -> semana7 quinta
(17/09), mesmo bloco 4o-5o tempos.

Analise apresentada e aprovada antes de aplicar: semana7 ja tem DaF
(14/09), tambem do grupo 1 -- par Mat+DaF sem Ingles viola a regra do
grupo 1. Usuario confirmou aplicar mesmo assim, como excecao pontual
(mesmo tratamento da Matematica do 11C na semana 6).

verificar_calendario.py acusa 2 PROBLEMA novos, esperados e
autorizados: "semana 7 com grupo 1 repetido ['DaF','Mat']" em 12C1 e
12C2. 2a prova (semana15, 10/11) inalterada. 5 relatorios
regenerados.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6120,12 +6120,7 @@
         </is>
       </c>
       <c r="G18" s="11" t="n"/>
-      <c r="H18" s="441" t="inlineStr">
-        <is>
-          <t>Mat - Bre/JJ
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H18" s="441" t="n"/>
       <c r="I18" s="432" t="inlineStr">
         <is>
           <t>Qui - CAl/Fab
@@ -6145,7 +6140,6 @@
       <c r="E19" s="315" t="n"/>
       <c r="F19" s="437" t="n"/>
       <c r="G19" s="222" t="n"/>
-      <c r="H19" s="437" t="n"/>
       <c r="I19" s="383" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
@@ -6168,7 +6162,6 @@
       <c r="E20" s="315" t="n"/>
       <c r="F20" s="439" t="n"/>
       <c r="G20" s="222" t="n"/>
-      <c r="H20" s="439" t="n"/>
       <c r="I20" s="384" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
@@ -6206,7 +6199,12 @@
         </is>
       </c>
       <c r="G21" s="435" t="n"/>
-      <c r="H21" s="435" t="n"/>
+      <c r="H21" s="409" t="inlineStr">
+        <is>
+          <t>Mat - Bre/JJ
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -6233,7 +6231,7 @@
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
       <c r="G22" s="438" t="n"/>
-      <c r="H22" s="438" t="n"/>
+      <c r="H22" s="406" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -6248,7 +6246,7 @@
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
       <c r="G23" s="438" t="n"/>
-      <c r="H23" s="438" t="n"/>
+      <c r="H23" s="407" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -7138,6 +7136,7 @@
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
+    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -7156,7 +7155,6 @@
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
     <mergeCell ref="H27:H29"/>
-    <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
     <mergeCell ref="E12:E14"/>
@@ -11172,7 +11170,7 @@
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="438" t="n"/>
-      <c r="H24" s="411" t="inlineStr">
+      <c r="H24" s="443" t="inlineStr">
         <is>
           <t>DaF - Caro-SGa-EFr
 1º e 2º tempos</t>
@@ -11196,7 +11194,7 @@
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
       <c r="G25" s="438" t="n"/>
-      <c r="H25" s="406" t="n"/>
+      <c r="H25" s="437" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
       <c r="M25" s="321" t="inlineStr">
@@ -11214,7 +11212,7 @@
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
       <c r="G26" s="438" t="n"/>
-      <c r="H26" s="407" t="n"/>
+      <c r="H26" s="439" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
       <c r="M26" s="323" t="inlineStr">
@@ -19487,12 +19485,7 @@
         </is>
       </c>
       <c r="G18" s="11" t="n"/>
-      <c r="H18" s="441" t="inlineStr">
-        <is>
-          <t>Mat - Bre/JJ
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H18" s="441" t="n"/>
       <c r="I18" s="432" t="inlineStr">
         <is>
           <t>Qui - CAl/Fab
@@ -19512,7 +19505,6 @@
       <c r="E19" s="315" t="n"/>
       <c r="F19" s="437" t="n"/>
       <c r="G19" s="222" t="n"/>
-      <c r="H19" s="437" t="n"/>
       <c r="I19" s="383" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
@@ -19535,7 +19527,6 @@
       <c r="E20" s="315" t="n"/>
       <c r="F20" s="439" t="n"/>
       <c r="G20" s="222" t="n"/>
-      <c r="H20" s="439" t="n"/>
       <c r="I20" s="384" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
@@ -19573,7 +19564,12 @@
         </is>
       </c>
       <c r="G21" s="435" t="n"/>
-      <c r="H21" s="435" t="n"/>
+      <c r="H21" s="441" t="inlineStr">
+        <is>
+          <t>Mat - Bre/JJ
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -19600,7 +19596,7 @@
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
       <c r="G22" s="438" t="n"/>
-      <c r="H22" s="438" t="n"/>
+      <c r="H22" s="437" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -19615,7 +19611,7 @@
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
       <c r="G23" s="438" t="n"/>
-      <c r="H23" s="438" t="n"/>
+      <c r="H23" s="439" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -20505,6 +20501,7 @@
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
+    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -20523,7 +20520,6 @@
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
     <mergeCell ref="H27:H29"/>
-    <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
     <mergeCell ref="E12:E14"/>

</xml_diff>

<commit_message>
12C: Matematica (1a prova) para 17/09, excecao autorizada ao grupo 1 (#55)
Matematica (12C1+12C2): semana6 quinta (10/09) -> semana7 quinta
(17/09), mesmo bloco 4o-5o tempos.

Analise apresentada e aprovada antes de aplicar: semana7 ja tem DaF
(14/09), tambem do grupo 1 -- par Mat+DaF sem Ingles viola a regra do
grupo 1. Usuario confirmou aplicar mesmo assim, como excecao pontual
(mesmo tratamento da Matematica do 11C na semana 6).

verificar_calendario.py acusa 2 PROBLEMA novos, esperados e
autorizados: "semana 7 com grupo 1 repetido ['DaF','Mat']" em 12C1 e
12C2. 2a prova (semana15, 10/11) inalterada. 5 relatorios
regenerados.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6120,12 +6120,7 @@
         </is>
       </c>
       <c r="G18" s="11" t="n"/>
-      <c r="H18" s="441" t="inlineStr">
-        <is>
-          <t>Mat - Bre/JJ
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H18" s="441" t="n"/>
       <c r="I18" s="432" t="inlineStr">
         <is>
           <t>Qui - CAl/Fab
@@ -6145,7 +6140,6 @@
       <c r="E19" s="315" t="n"/>
       <c r="F19" s="437" t="n"/>
       <c r="G19" s="222" t="n"/>
-      <c r="H19" s="437" t="n"/>
       <c r="I19" s="383" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
@@ -6168,7 +6162,6 @@
       <c r="E20" s="315" t="n"/>
       <c r="F20" s="439" t="n"/>
       <c r="G20" s="222" t="n"/>
-      <c r="H20" s="439" t="n"/>
       <c r="I20" s="384" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
@@ -6206,7 +6199,12 @@
         </is>
       </c>
       <c r="G21" s="435" t="n"/>
-      <c r="H21" s="435" t="n"/>
+      <c r="H21" s="409" t="inlineStr">
+        <is>
+          <t>Mat - Bre/JJ
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -6233,7 +6231,7 @@
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
       <c r="G22" s="438" t="n"/>
-      <c r="H22" s="438" t="n"/>
+      <c r="H22" s="406" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -6248,7 +6246,7 @@
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
       <c r="G23" s="438" t="n"/>
-      <c r="H23" s="438" t="n"/>
+      <c r="H23" s="407" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -7138,6 +7136,7 @@
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
+    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -7156,7 +7155,6 @@
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
     <mergeCell ref="H27:H29"/>
-    <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
     <mergeCell ref="E12:E14"/>
@@ -11172,7 +11170,7 @@
       <c r="E24" s="283" t="n"/>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="438" t="n"/>
-      <c r="H24" s="411" t="inlineStr">
+      <c r="H24" s="443" t="inlineStr">
         <is>
           <t>DaF - Caro-SGa-EFr
 1º e 2º tempos</t>
@@ -11196,7 +11194,7 @@
       <c r="E25" s="283" t="n"/>
       <c r="F25" s="283" t="n"/>
       <c r="G25" s="438" t="n"/>
-      <c r="H25" s="406" t="n"/>
+      <c r="H25" s="437" t="n"/>
       <c r="J25" s="352" t="n"/>
       <c r="L25" s="44" t="n"/>
       <c r="M25" s="321" t="inlineStr">
@@ -11214,7 +11212,7 @@
       <c r="E26" s="283" t="n"/>
       <c r="F26" s="283" t="n"/>
       <c r="G26" s="438" t="n"/>
-      <c r="H26" s="407" t="n"/>
+      <c r="H26" s="439" t="n"/>
       <c r="J26" s="352" t="n"/>
       <c r="L26" s="43" t="n"/>
       <c r="M26" s="323" t="inlineStr">
@@ -19487,12 +19485,7 @@
         </is>
       </c>
       <c r="G18" s="11" t="n"/>
-      <c r="H18" s="441" t="inlineStr">
-        <is>
-          <t>Mat - Bre/JJ
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="H18" s="441" t="n"/>
       <c r="I18" s="432" t="inlineStr">
         <is>
           <t>Qui - CAl/Fab
@@ -19512,7 +19505,6 @@
       <c r="E19" s="315" t="n"/>
       <c r="F19" s="437" t="n"/>
       <c r="G19" s="222" t="n"/>
-      <c r="H19" s="437" t="n"/>
       <c r="I19" s="383" t="n"/>
       <c r="J19" s="315" t="n"/>
       <c r="L19" s="29" t="inlineStr">
@@ -19535,7 +19527,6 @@
       <c r="E20" s="315" t="n"/>
       <c r="F20" s="439" t="n"/>
       <c r="G20" s="222" t="n"/>
-      <c r="H20" s="439" t="n"/>
       <c r="I20" s="384" t="n"/>
       <c r="J20" s="315" t="n"/>
       <c r="L20" s="29" t="n"/>
@@ -19573,7 +19564,12 @@
         </is>
       </c>
       <c r="G21" s="435" t="n"/>
-      <c r="H21" s="435" t="n"/>
+      <c r="H21" s="441" t="inlineStr">
+        <is>
+          <t>Mat - Bre/JJ
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="262" t="inlineStr">
         <is>
@@ -19600,7 +19596,7 @@
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
       <c r="G22" s="438" t="n"/>
-      <c r="H22" s="438" t="n"/>
+      <c r="H22" s="437" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -19615,7 +19611,7 @@
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
       <c r="G23" s="438" t="n"/>
-      <c r="H23" s="438" t="n"/>
+      <c r="H23" s="439" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -20505,6 +20501,7 @@
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="F21:F23"/>
     <mergeCell ref="D57:D59"/>
+    <mergeCell ref="H21:H23"/>
     <mergeCell ref="F51:F53"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="H51:H53"/>
@@ -20523,7 +20520,6 @@
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="D42:D44"/>
     <mergeCell ref="H27:H29"/>
-    <mergeCell ref="H18:H20"/>
     <mergeCell ref="J18:J20"/>
     <mergeCell ref="H33:H35"/>
     <mergeCell ref="E12:E14"/>

</xml_diff>

<commit_message>
11C: Historia (1a prova) para 08/09 a tarde, excecao autorizada
Historia (11C1+11C2): semana5 quarta (02/09) -> semana6 terca (08/09),
tempos 10o-11o (aula dupla real do 11C2, a tarde). Doadores no 11C1:
Redacao/ACo (10o tempo) e Fisica/Cadu (11o tempo).

3 alternativas analisadas e apresentadas antes de aplicar: 08/09 manha
(forcaria Quimica como doadora, recusado); 16/09 com Fisica realocada
(mais limpa, nao escolhida); 08/09 tarde (escolhida pelo usuario,
mesmo custando 2 estouros de teto novos).

verificar_calendario.py fecha so com os 6 PROBLEMA ja conhecidos e
autorizados -- nenhum novo. Novos AVISOs esperados e autorizados como
excecao pontual (nao vira regra na skill): Historia nos tempos 7-11
(flexibilizacao consciente da regra de tarde), Redacao/ACo e
Fisica/Cadu (11C1) acima do teto de cessao, mais vespera leve da
Fisica.

5 relatorios regenerados.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6199,7 +6199,7 @@
         </is>
       </c>
       <c r="G21" s="435" t="n"/>
-      <c r="H21" s="409" t="inlineStr">
+      <c r="H21" s="441" t="inlineStr">
         <is>
           <t>Mat - Bre/JJ
 4º e 5º tempos</t>
@@ -6231,7 +6231,7 @@
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
       <c r="G22" s="438" t="n"/>
-      <c r="H22" s="406" t="n"/>
+      <c r="H22" s="437" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -6246,7 +6246,7 @@
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
       <c r="G23" s="438" t="n"/>
-      <c r="H23" s="407" t="n"/>
+      <c r="H23" s="439" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -15998,12 +15998,7 @@
         </is>
       </c>
       <c r="F15" s="434" t="n"/>
-      <c r="G15" s="470" t="inlineStr">
-        <is>
-          <t>Hist - Ver
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="G15" s="470" t="n"/>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -16022,7 +16017,6 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="G16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -16037,7 +16031,6 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="G17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -16068,7 +16061,12 @@
           <t>unterrichtsfrei sem aula</t>
         </is>
       </c>
-      <c r="F18" s="451" t="n"/>
+      <c r="F18" s="470" t="inlineStr">
+        <is>
+          <t>Hist - Ver
+10º e 11º tempos</t>
+        </is>
+      </c>
       <c r="G18" s="443" t="inlineStr">
         <is>
           <t>DaF - CBu-SGa-Swa
@@ -16093,6 +16091,7 @@
       <c r="C19" s="313" t="n"/>
       <c r="D19" s="314" t="n"/>
       <c r="E19" s="315" t="n"/>
+      <c r="F19" s="437" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="437" t="n"/>
       <c r="I19" s="383" t="n"/>
@@ -16115,6 +16114,7 @@
       <c r="C20" s="313" t="n"/>
       <c r="D20" s="314" t="n"/>
       <c r="E20" s="315" t="n"/>
+      <c r="F20" s="439" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="439" t="n"/>
       <c r="I20" s="384" t="n"/>
@@ -17187,13 +17187,13 @@
     <mergeCell ref="M26:N26"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
+    <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
-    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
@@ -17698,12 +17698,7 @@
         </is>
       </c>
       <c r="F15" s="434" t="n"/>
-      <c r="G15" s="470" t="inlineStr">
-        <is>
-          <t>Hist - Ver
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="G15" s="470" t="n"/>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -17722,7 +17717,6 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="G16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -17737,7 +17731,6 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="G17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -17768,7 +17761,12 @@
           <t>unterrichtsfrei sem aula</t>
         </is>
       </c>
-      <c r="F18" s="451" t="n"/>
+      <c r="F18" s="468" t="inlineStr">
+        <is>
+          <t>Hist - Ver
+10º e 11º tempos</t>
+        </is>
+      </c>
       <c r="G18" s="443" t="inlineStr">
         <is>
           <t>DaF - CBu-SGa-Swa
@@ -17793,6 +17791,7 @@
       <c r="C19" s="313" t="n"/>
       <c r="D19" s="314" t="n"/>
       <c r="E19" s="315" t="n"/>
+      <c r="F19" s="406" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="437" t="n"/>
       <c r="J19" s="315" t="n"/>
@@ -17814,6 +17813,7 @@
       <c r="C20" s="313" t="n"/>
       <c r="D20" s="314" t="n"/>
       <c r="E20" s="315" t="n"/>
+      <c r="F20" s="407" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="439" t="n"/>
       <c r="J20" s="315" t="n"/>
@@ -18886,13 +18886,13 @@
     <mergeCell ref="M26:N26"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
+    <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
-    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>

</xml_diff>

<commit_message>
11C: Historia (1a prova) para 08/09 a tarde, excecao autorizada (#56)
Historia (11C1+11C2): semana5 quarta (02/09) -> semana6 terca (08/09),
tempos 10o-11o (aula dupla real do 11C2, a tarde). Doadores no 11C1:
Redacao/ACo (10o tempo) e Fisica/Cadu (11o tempo).

3 alternativas analisadas e apresentadas antes de aplicar: 08/09 manha
(forcaria Quimica como doadora, recusado); 16/09 com Fisica realocada
(mais limpa, nao escolhida); 08/09 tarde (escolhida pelo usuario,
mesmo custando 2 estouros de teto novos).

verificar_calendario.py fecha so com os 6 PROBLEMA ja conhecidos e
autorizados -- nenhum novo. Novos AVISOs esperados e autorizados como
excecao pontual (nao vira regra na skill): Historia nos tempos 7-11
(flexibilizacao consciente da regra de tarde), Redacao/ACo e
Fisica/Cadu (11C1) acima do teto de cessao, mais vespera leve da
Fisica.

5 relatorios regenerados.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_3_Calendario_Provas_2026_2SEM.xlsx
@@ -6199,7 +6199,7 @@
         </is>
       </c>
       <c r="G21" s="435" t="n"/>
-      <c r="H21" s="409" t="inlineStr">
+      <c r="H21" s="441" t="inlineStr">
         <is>
           <t>Mat - Bre/JJ
 4º e 5º tempos</t>
@@ -6231,7 +6231,7 @@
       <c r="E22" s="437" t="n"/>
       <c r="F22" s="437" t="n"/>
       <c r="G22" s="438" t="n"/>
-      <c r="H22" s="406" t="n"/>
+      <c r="H22" s="437" t="n"/>
       <c r="I22" s="222" t="n"/>
       <c r="J22" s="315" t="n"/>
       <c r="L22" s="18" t="n"/>
@@ -6246,7 +6246,7 @@
       <c r="E23" s="439" t="n"/>
       <c r="F23" s="439" t="n"/>
       <c r="G23" s="438" t="n"/>
-      <c r="H23" s="407" t="n"/>
+      <c r="H23" s="439" t="n"/>
       <c r="I23" s="222" t="n"/>
       <c r="J23" s="315" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -15998,12 +15998,7 @@
         </is>
       </c>
       <c r="F15" s="434" t="n"/>
-      <c r="G15" s="470" t="inlineStr">
-        <is>
-          <t>Hist - Ver
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="G15" s="470" t="n"/>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -16022,7 +16017,6 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="G16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -16037,7 +16031,6 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="G17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -16068,7 +16061,12 @@
           <t>unterrichtsfrei sem aula</t>
         </is>
       </c>
-      <c r="F18" s="451" t="n"/>
+      <c r="F18" s="470" t="inlineStr">
+        <is>
+          <t>Hist - Ver
+10º e 11º tempos</t>
+        </is>
+      </c>
       <c r="G18" s="443" t="inlineStr">
         <is>
           <t>DaF - CBu-SGa-Swa
@@ -16093,6 +16091,7 @@
       <c r="C19" s="313" t="n"/>
       <c r="D19" s="314" t="n"/>
       <c r="E19" s="315" t="n"/>
+      <c r="F19" s="437" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="437" t="n"/>
       <c r="I19" s="383" t="n"/>
@@ -16115,6 +16114,7 @@
       <c r="C20" s="313" t="n"/>
       <c r="D20" s="314" t="n"/>
       <c r="E20" s="315" t="n"/>
+      <c r="F20" s="439" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="439" t="n"/>
       <c r="I20" s="384" t="n"/>
@@ -17187,13 +17187,13 @@
     <mergeCell ref="M26:N26"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
+    <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
-    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>
@@ -17698,12 +17698,7 @@
         </is>
       </c>
       <c r="F15" s="434" t="n"/>
-      <c r="G15" s="470" t="inlineStr">
-        <is>
-          <t>Hist - Ver
-1º e 2º tempos</t>
-        </is>
-      </c>
+      <c r="G15" s="470" t="n"/>
       <c r="H15" s="458" t="inlineStr">
         <is>
           <t>LP/LIT/RED - ACo/AMu/Raf
@@ -17722,7 +17717,6 @@
       <c r="C16" s="313" t="n"/>
       <c r="D16" s="314" t="n"/>
       <c r="E16" s="437" t="n"/>
-      <c r="G16" s="437" t="n"/>
       <c r="H16" s="437" t="n"/>
       <c r="I16" s="222" t="n"/>
       <c r="J16" s="315" t="n"/>
@@ -17737,7 +17731,6 @@
       <c r="C17" s="313" t="n"/>
       <c r="D17" s="314" t="n"/>
       <c r="E17" s="439" t="n"/>
-      <c r="G17" s="439" t="n"/>
       <c r="H17" s="439" t="n"/>
       <c r="I17" s="222" t="n"/>
       <c r="J17" s="315" t="n"/>
@@ -17768,7 +17761,12 @@
           <t>unterrichtsfrei sem aula</t>
         </is>
       </c>
-      <c r="F18" s="451" t="n"/>
+      <c r="F18" s="468" t="inlineStr">
+        <is>
+          <t>Hist - Ver
+10º e 11º tempos</t>
+        </is>
+      </c>
       <c r="G18" s="443" t="inlineStr">
         <is>
           <t>DaF - CBu-SGa-Swa
@@ -17793,6 +17791,7 @@
       <c r="C19" s="313" t="n"/>
       <c r="D19" s="314" t="n"/>
       <c r="E19" s="315" t="n"/>
+      <c r="F19" s="406" t="n"/>
       <c r="G19" s="437" t="n"/>
       <c r="H19" s="437" t="n"/>
       <c r="J19" s="315" t="n"/>
@@ -17814,6 +17813,7 @@
       <c r="C20" s="313" t="n"/>
       <c r="D20" s="314" t="n"/>
       <c r="E20" s="315" t="n"/>
+      <c r="F20" s="407" t="n"/>
       <c r="G20" s="439" t="n"/>
       <c r="H20" s="439" t="n"/>
       <c r="J20" s="315" t="n"/>
@@ -18886,13 +18886,13 @@
     <mergeCell ref="M26:N26"/>
     <mergeCell ref="D45:D47"/>
     <mergeCell ref="H9:H11"/>
+    <mergeCell ref="F18:F20"/>
     <mergeCell ref="J9:J11"/>
     <mergeCell ref="F45:F47"/>
     <mergeCell ref="M29:N29"/>
     <mergeCell ref="F42:F44"/>
     <mergeCell ref="E15:E17"/>
     <mergeCell ref="J36:J38"/>
-    <mergeCell ref="G15:G17"/>
     <mergeCell ref="J45:J47"/>
     <mergeCell ref="C60:C62"/>
     <mergeCell ref="B6:B8"/>

</xml_diff>